<commit_message>
added gauss for abel
</commit_message>
<xml_diff>
--- a/results/aligned_results.xlsx
+++ b/results/aligned_results.xlsx
@@ -17,16 +17,13 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -37,7 +34,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -45,21 +42,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -425,56 +413,46 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J101"/>
+  <dimension ref="A1:H101"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>Radius_mm_Left</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>Cu I 465.1_Left</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>Cu I 510.5_Left</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>Cu I 515.3_Left</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>Cu I 521.8_Left</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>Radius_mm_Right</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
-        <is>
-          <t>Cu I 465.1_Right</t>
-        </is>
-      </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>Cu I 510.5_Right</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>Cu I 515.3_Right</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>Cu I 521.8_Right</t>
         </is>
@@ -485,3199 +463,2599 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>865.6824070287303</v>
+        <v>17888.64366085385</v>
       </c>
       <c r="C2" t="n">
-        <v>2083.193004277779</v>
+        <v>5135.76495171912</v>
       </c>
       <c r="D2" t="n">
-        <v>4923.728818947581</v>
+        <v>8685.470403811776</v>
       </c>
       <c r="E2" t="n">
-        <v>6051.947326830919</v>
+        <v>0</v>
       </c>
       <c r="F2" t="n">
-        <v>0</v>
+        <v>16386.65016889948</v>
       </c>
       <c r="G2" t="n">
-        <v>889.866794891168</v>
+        <v>5254.246639211582</v>
       </c>
       <c r="H2" t="n">
-        <v>1204.203361230557</v>
-      </c>
-      <c r="I2" t="n">
-        <v>3763.578190100568</v>
-      </c>
-      <c r="J2" t="n">
-        <v>10010.30469287295</v>
+        <v>8426.799372843785</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>0.02364141414141414</v>
+        <v>0.03616666666666667</v>
       </c>
       <c r="B3" t="n">
-        <v>784.4186851102008</v>
+        <v>17832.75660390735</v>
       </c>
       <c r="C3" t="n">
-        <v>2460.789953362717</v>
+        <v>5123.051644782186</v>
       </c>
       <c r="D3" t="n">
-        <v>4681.743015622311</v>
+        <v>8681.625423709229</v>
       </c>
       <c r="E3" t="n">
-        <v>5948.254853459384</v>
+        <v>0.03507070707070707</v>
       </c>
       <c r="F3" t="n">
-        <v>0.02004040404040404</v>
+        <v>16378.55442631159</v>
       </c>
       <c r="G3" t="n">
-        <v>823.0547129044185</v>
+        <v>5257.461187315059</v>
       </c>
       <c r="H3" t="n">
-        <v>2149.128102361662</v>
-      </c>
-      <c r="I3" t="n">
-        <v>3679.658466597645</v>
-      </c>
-      <c r="J3" t="n">
-        <v>9522.006622575544</v>
+        <v>8412.755837120521</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>0.04728282828282828</v>
+        <v>0.07233333333333333</v>
       </c>
       <c r="B4" t="n">
-        <v>718.2595839911933</v>
+        <v>17773.7015421398</v>
       </c>
       <c r="C4" t="n">
-        <v>2826.749782569463</v>
+        <v>5108.009642331043</v>
       </c>
       <c r="D4" t="n">
-        <v>4455.407939538371</v>
+        <v>8673.603555006081</v>
       </c>
       <c r="E4" t="n">
-        <v>5849.132174465274</v>
+        <v>0.07014141414141414</v>
       </c>
       <c r="F4" t="n">
-        <v>0.04008080808080808</v>
+        <v>16367.63178189033</v>
       </c>
       <c r="G4" t="n">
-        <v>770.3347191308683</v>
+        <v>5257.060152077372</v>
       </c>
       <c r="H4" t="n">
-        <v>3031.251084045102</v>
-      </c>
-      <c r="I4" t="n">
-        <v>3601.680276543333</v>
-      </c>
-      <c r="J4" t="n">
-        <v>9080.667688480919</v>
+        <v>8393.64232361695</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>0.07092424242424242</v>
+        <v>0.1085</v>
       </c>
       <c r="B5" t="n">
-        <v>673.6956043671628</v>
+        <v>17710.90273945525</v>
       </c>
       <c r="C5" t="n">
-        <v>3178.068412132941</v>
+        <v>5090.381540920207</v>
       </c>
       <c r="D5" t="n">
-        <v>4250.577839698563</v>
+        <v>8660.247223302698</v>
       </c>
       <c r="E5" t="n">
-        <v>5756.527439456071</v>
+        <v>0.1052121212121212</v>
       </c>
       <c r="F5" t="n">
-        <v>0.06012121212121212</v>
+        <v>16352.99377994298</v>
       </c>
       <c r="G5" t="n">
-        <v>732.8596844586247</v>
+        <v>5252.606938598494</v>
       </c>
       <c r="H5" t="n">
-        <v>3827.659804423981</v>
-      </c>
-      <c r="I5" t="n">
-        <v>3532.209675543438</v>
-      </c>
-      <c r="J5" t="n">
-        <v>8706.493965451607</v>
+        <v>8369.366349510328</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>0.09456565656565656</v>
+        <v>0.1446666666666667</v>
       </c>
       <c r="B6" t="n">
-        <v>639.4918411699599</v>
+        <v>17643.78445975776</v>
       </c>
       <c r="C6" t="n">
-        <v>3511.74176228808</v>
+        <v>5069.909937104188</v>
       </c>
       <c r="D6" t="n">
-        <v>4073.106965105702</v>
+        <v>8640.398854199459</v>
       </c>
       <c r="E6" t="n">
-        <v>5672.388798039263</v>
+        <v>0.1402828282828283</v>
       </c>
       <c r="F6" t="n">
-        <v>0.08016161616161616</v>
+        <v>16333.75196477681</v>
       </c>
       <c r="G6" t="n">
-        <v>706.3128641581368</v>
+        <v>5243.664951978401</v>
       </c>
       <c r="H6" t="n">
-        <v>4515.441761641402</v>
-      </c>
-      <c r="I6" t="n">
-        <v>3473.812719203768</v>
-      </c>
-      <c r="J6" t="n">
-        <v>8418.92189398805</v>
+        <v>8339.835431977912</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
-        <v>0.1182070707070707</v>
+        <v>0.1808333333333333</v>
       </c>
       <c r="B7" t="n">
-        <v>612.9321639877876</v>
+        <v>17571.77096695139</v>
       </c>
       <c r="C7" t="n">
-        <v>3824.765753269806</v>
+        <v>5046.337427437502</v>
       </c>
       <c r="D7" t="n">
-        <v>3928.84956476259</v>
+        <v>8612.900873296723</v>
       </c>
       <c r="E7" t="n">
-        <v>5598.664399822335</v>
+        <v>0.1753535353535354</v>
       </c>
       <c r="F7" t="n">
-        <v>0.1002020202020202</v>
+        <v>16309.01788069911</v>
       </c>
       <c r="G7" t="n">
-        <v>692.5291510299987</v>
+        <v>5229.797597317065</v>
       </c>
       <c r="H7" t="n">
-        <v>5071.684453840469</v>
-      </c>
-      <c r="I7" t="n">
-        <v>3428.23049775692</v>
-      </c>
-      <c r="J7" t="n">
-        <v>8180.68990968829</v>
+        <v>8304.957088196958</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
-        <v>0.1418484848484848</v>
+        <v>0.217</v>
       </c>
       <c r="B8" t="n">
-        <v>592.5388918628342</v>
+        <v>17494.28652494021</v>
       </c>
       <c r="C8" t="n">
-        <v>4114.136305313046</v>
+        <v>5019.406608474663</v>
       </c>
       <c r="D8" t="n">
-        <v>3814.06851611082</v>
+        <v>8576.595706194865</v>
       </c>
       <c r="E8" t="n">
-        <v>5537.242772150468</v>
+        <v>0.2104242424242424</v>
       </c>
       <c r="F8" t="n">
-        <v>0.1202424242424242</v>
+        <v>16277.90307201715</v>
       </c>
       <c r="G8" t="n">
-        <v>689.6493474431543</v>
+        <v>5210.568279714459</v>
       </c>
       <c r="H8" t="n">
-        <v>5496.074495763962</v>
-      </c>
-      <c r="I8" t="n">
-        <v>3388.030756257088</v>
-      </c>
-      <c r="J8" t="n">
-        <v>7963.713208247505</v>
+        <v>8264.638835344722</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
-        <v>0.165489898989899</v>
+        <v>0.2531666666666667</v>
       </c>
       <c r="B9" t="n">
-        <v>573.2388615769848</v>
+        <v>17410.75539762826</v>
       </c>
       <c r="C9" t="n">
-        <v>4376.849338652729</v>
+        <v>4988.860076770186</v>
       </c>
       <c r="D9" t="n">
-        <v>3709.065661195702</v>
+        <v>8530.325778494249</v>
       </c>
       <c r="E9" t="n">
-        <v>5482.611112943129</v>
+        <v>0.2454949494949495</v>
       </c>
       <c r="F9" t="n">
-        <v>0.1402828282828283</v>
+        <v>16239.51908303822</v>
       </c>
       <c r="G9" t="n">
-        <v>681.6492503267685</v>
+        <v>5185.540404270557</v>
       </c>
       <c r="H9" t="n">
-        <v>5872.25520987022</v>
-      </c>
-      <c r="I9" t="n">
-        <v>3351.132945742486</v>
-      </c>
-      <c r="J9" t="n">
-        <v>7770.500915521243</v>
+        <v>8218.788190598463</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="n">
-        <v>0.1891313131313131</v>
+        <v>0.2893333333333333</v>
       </c>
       <c r="B10" t="n">
-        <v>556.9266187419701</v>
+        <v>17320.60184891961</v>
       </c>
       <c r="C10" t="n">
-        <v>4609.900773523777</v>
+        <v>4954.440428878583</v>
       </c>
       <c r="D10" t="n">
-        <v>3613.865817380909</v>
+        <v>8472.933515795252</v>
       </c>
       <c r="E10" t="n">
-        <v>5430.36597413321</v>
+        <v>0.2805656565656566</v>
       </c>
       <c r="F10" t="n">
-        <v>0.1603232323232323</v>
+        <v>16192.97745806958</v>
       </c>
       <c r="G10" t="n">
-        <v>662.2050262159645</v>
+        <v>5154.277376085332</v>
       </c>
       <c r="H10" t="n">
-        <v>6208.971366707489</v>
-      </c>
-      <c r="I10" t="n">
-        <v>3317.929316120174</v>
-      </c>
-      <c r="J10" t="n">
-        <v>7603.562157365049</v>
+        <v>8167.312671135434</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="n">
-        <v>0.2127727272727273</v>
+        <v>0.3255</v>
       </c>
       <c r="B11" t="n">
-        <v>542.3613621577981</v>
+        <v>17223.25014271832</v>
       </c>
       <c r="C11" t="n">
-        <v>4810.286530161124</v>
+        <v>4915.890261354367</v>
       </c>
       <c r="D11" t="n">
-        <v>3529.455446798599</v>
+        <v>8403.261343698239</v>
       </c>
       <c r="E11" t="n">
-        <v>5380.778376943994</v>
+        <v>0.3156363636363637</v>
       </c>
       <c r="F11" t="n">
-        <v>0.1803636363636363</v>
+        <v>16137.38974141853</v>
       </c>
       <c r="G11" t="n">
-        <v>640.3566753426252</v>
+        <v>5116.342600258759</v>
       </c>
       <c r="H11" t="n">
-        <v>6504.281479090492</v>
-      </c>
-      <c r="I11" t="n">
-        <v>3288.812117297214</v>
-      </c>
-      <c r="J11" t="n">
-        <v>7461.470815817882</v>
+        <v>8110.119794132899</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="n">
-        <v>0.2364141414141414</v>
+        <v>0.3616666666666667</v>
       </c>
       <c r="B12" t="n">
-        <v>528.6229493095777</v>
+        <v>17118.12454292845</v>
       </c>
       <c r="C12" t="n">
-        <v>4975.420561920268</v>
+        <v>4872.952170752055</v>
       </c>
       <c r="D12" t="n">
-        <v>3456.821011580934</v>
+        <v>8320.151687803578</v>
       </c>
       <c r="E12" t="n">
-        <v>5334.119342598766</v>
+        <v>0.3507070707070707</v>
       </c>
       <c r="F12" t="n">
-        <v>0.2004040404040404</v>
+        <v>16071.86747739233</v>
       </c>
       <c r="G12" t="n">
-        <v>622.6717600100702</v>
+        <v>5071.299481890811</v>
       </c>
       <c r="H12" t="n">
-        <v>6756.24405983395</v>
-      </c>
-      <c r="I12" t="n">
-        <v>3262.853717053957</v>
-      </c>
-      <c r="J12" t="n">
-        <v>7322.970660003706</v>
+        <v>8047.11707676811</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="n">
-        <v>0.2600555555555555</v>
+        <v>0.3978333333333333</v>
       </c>
       <c r="B13" t="n">
-        <v>516.3440096466652</v>
+        <v>17004.64931345405</v>
       </c>
       <c r="C13" t="n">
-        <v>5122.387644888244</v>
+        <v>4825.36875362616</v>
       </c>
       <c r="D13" t="n">
-        <v>3395.070695802939</v>
+        <v>8222.446973711645</v>
       </c>
       <c r="E13" t="n">
-        <v>5290.659892320808</v>
+        <v>0.3857777777777778</v>
       </c>
       <c r="F13" t="n">
-        <v>0.2204444444444444</v>
+        <v>15995.52221029826</v>
       </c>
       <c r="G13" t="n">
-        <v>610.33554977482</v>
+        <v>5019.196819224666</v>
       </c>
       <c r="H13" t="n">
-        <v>6963.75812323656</v>
-      </c>
-      <c r="I13" t="n">
-        <v>3236.97688276238</v>
-      </c>
-      <c r="J13" t="n">
-        <v>7187.928136590104</v>
+        <v>7978.212036218324</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="n">
-        <v>0.2836969696969697</v>
+        <v>0.434</v>
       </c>
       <c r="B14" t="n">
-        <v>504.7354394514246</v>
+        <v>16882.24871819918</v>
       </c>
       <c r="C14" t="n">
-        <v>5261.240704675292</v>
+        <v>4772.882606531195</v>
       </c>
       <c r="D14" t="n">
-        <v>3334.579516891185</v>
+        <v>8114.033591711061</v>
       </c>
       <c r="E14" t="n">
-        <v>5250.592862137552</v>
+        <v>0.4208484848484849</v>
       </c>
       <c r="F14" t="n">
-        <v>0.2404848484848485</v>
+        <v>15907.46548444361</v>
       </c>
       <c r="G14" t="n">
-        <v>599.0532081194068</v>
+        <v>4964.250279682486</v>
       </c>
       <c r="H14" t="n">
-        <v>7159.340544929423</v>
-      </c>
-      <c r="I14" t="n">
-        <v>3211.609076416421</v>
-      </c>
-      <c r="J14" t="n">
-        <v>7060.468205603302</v>
+        <v>7905.384402759887</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="n">
-        <v>0.3073383838383838</v>
+        <v>0.4701666666666667</v>
       </c>
       <c r="B15" t="n">
-        <v>493.603041351157</v>
+        <v>16750.3470210679</v>
       </c>
       <c r="C15" t="n">
-        <v>5391.734062420092</v>
+        <v>4717.230580940112</v>
       </c>
       <c r="D15" t="n">
-        <v>3275.16000967023</v>
+        <v>8002.882034525599</v>
       </c>
       <c r="E15" t="n">
-        <v>5211.562162758041</v>
+        <v>0.4559191919191919</v>
       </c>
       <c r="F15" t="n">
-        <v>0.2605252525252525</v>
+        <v>15806.80884413566</v>
       </c>
       <c r="G15" t="n">
-        <v>588.7666969236585</v>
+        <v>4907.202710297628</v>
       </c>
       <c r="H15" t="n">
-        <v>7352.462591661018</v>
-      </c>
-      <c r="I15" t="n">
-        <v>3187.383029576048</v>
-      </c>
-      <c r="J15" t="n">
-        <v>6944.715827069534</v>
+        <v>7830.440490489347</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="n">
-        <v>0.330979797979798</v>
+        <v>0.5063333333333333</v>
       </c>
       <c r="B16" t="n">
-        <v>483.3881690524303</v>
+        <v>16608.36848596428</v>
       </c>
       <c r="C16" t="n">
-        <v>5513.622039261325</v>
+        <v>4660.152642162172</v>
       </c>
       <c r="D16" t="n">
-        <v>3218.382864015139</v>
+        <v>7888.982739125892</v>
       </c>
       <c r="E16" t="n">
-        <v>5172.508601904848</v>
+        <v>0.490989898989899</v>
       </c>
       <c r="F16" t="n">
-        <v>0.2805656565656566</v>
+        <v>15692.66383368167</v>
       </c>
       <c r="G16" t="n">
-        <v>579.6645638666905</v>
+        <v>4847.638947347634</v>
       </c>
       <c r="H16" t="n">
-        <v>7532.03817860666</v>
-      </c>
-      <c r="I16" t="n">
-        <v>3164.924624755445</v>
-      </c>
-      <c r="J16" t="n">
-        <v>6838.777428078112</v>
+        <v>7752.336804543338</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="n">
-        <v>0.3546212121212121</v>
+        <v>0.5425</v>
       </c>
       <c r="B17" t="n">
-        <v>473.9764497825018</v>
+        <v>16455.73737679236</v>
       </c>
       <c r="C17" t="n">
-        <v>5626.658956337669</v>
+        <v>4601.396057506347</v>
       </c>
       <c r="D17" t="n">
-        <v>3165.818769800976</v>
+        <v>7772.189472288319</v>
       </c>
       <c r="E17" t="n">
-        <v>5133.637897973065</v>
+        <v>0.5260606060606061</v>
       </c>
       <c r="F17" t="n">
-        <v>0.3006060606060606</v>
+        <v>15564.14199738893</v>
       </c>
       <c r="G17" t="n">
-        <v>572.6344761808111</v>
+        <v>4785.14382711004</v>
       </c>
       <c r="H17" t="n">
-        <v>7686.98122094166</v>
-      </c>
-      <c r="I17" t="n">
-        <v>3143.456096871338</v>
-      </c>
-      <c r="J17" t="n">
-        <v>6734.612325670932</v>
+        <v>7670.023938820856</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="n">
-        <v>0.3782626262626262</v>
+        <v>0.5786666666666667</v>
       </c>
       <c r="B18" t="n">
-        <v>463.7470625401458</v>
+        <v>16291.87795745622</v>
       </c>
       <c r="C18" t="n">
-        <v>5730.599134787805</v>
+        <v>4540.708094281616</v>
       </c>
       <c r="D18" t="n">
-        <v>3118.781219049842</v>
+        <v>7652.356000789257</v>
       </c>
       <c r="E18" t="n">
-        <v>5095.15576935779</v>
+        <v>0.5611313131313131</v>
       </c>
       <c r="F18" t="n">
-        <v>0.3206464646464646</v>
+        <v>15420.35487956472</v>
       </c>
       <c r="G18" t="n">
-        <v>575.9970081861096</v>
+        <v>4719.302185862387</v>
       </c>
       <c r="H18" t="n">
-        <v>7806.205633841335</v>
-      </c>
-      <c r="I18" t="n">
-        <v>3122.095084061247</v>
-      </c>
-      <c r="J18" t="n">
-        <v>6633.080007295061</v>
+        <v>7582.452487220898</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="n">
-        <v>0.4019040404040404</v>
+        <v>0.6148333333333333</v>
       </c>
       <c r="B19" t="n">
-        <v>448.5446330378237</v>
+        <v>16116.2144918599</v>
       </c>
       <c r="C19" t="n">
-        <v>5825.196895750412</v>
+        <v>4477.83601979695</v>
       </c>
       <c r="D19" t="n">
-        <v>3073.504464298197</v>
+        <v>7529.336091405085</v>
       </c>
       <c r="E19" t="n">
-        <v>5057.267934454116</v>
+        <v>0.5962020202020202</v>
       </c>
       <c r="F19" t="n">
-        <v>0.3406868686868686</v>
+        <v>15260.41402451631</v>
       </c>
       <c r="G19" t="n">
-        <v>575.8682632369224</v>
+        <v>4649.698859882211</v>
       </c>
       <c r="H19" t="n">
-        <v>7892.657635861482</v>
-      </c>
-      <c r="I19" t="n">
-        <v>3100.820240620682</v>
-      </c>
-      <c r="J19" t="n">
-        <v>6535.211469494767</v>
+        <v>7488.573043642458</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="n">
-        <v>0.4255454545454545</v>
+        <v>0.651</v>
       </c>
       <c r="B20" t="n">
-        <v>433.6730633125138</v>
+        <v>15928.17124390747</v>
       </c>
       <c r="C20" t="n">
-        <v>5910.206560364172</v>
+        <v>4412.527101361327</v>
       </c>
       <c r="D20" t="n">
-        <v>3028.746826118712</v>
+        <v>7402.98351091218</v>
       </c>
       <c r="E20" t="n">
-        <v>5020.13805191938</v>
+        <v>0.6312727272727273</v>
       </c>
       <c r="F20" t="n">
-        <v>0.3607272727272727</v>
+        <v>15083.43097655099</v>
       </c>
       <c r="G20" t="n">
-        <v>562.8110432830608</v>
+        <v>4575.918685447054</v>
       </c>
       <c r="H20" t="n">
-        <v>7973.844062608211</v>
-      </c>
-      <c r="I20" t="n">
-        <v>3079.610220845152</v>
-      </c>
-      <c r="J20" t="n">
-        <v>6442.077231956048</v>
+        <v>7387.336201984535</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="n">
-        <v>0.4491868686868687</v>
+        <v>0.6871666666666667</v>
       </c>
       <c r="B21" t="n">
-        <v>428.3439535760392</v>
+        <v>15727.17247750298</v>
       </c>
       <c r="C21" t="n">
-        <v>5985.382449767763</v>
+        <v>4344.528606283721</v>
       </c>
       <c r="D21" t="n">
-        <v>2985.164882722694</v>
+        <v>7273.152026086922</v>
       </c>
       <c r="E21" t="n">
-        <v>4983.241672585024</v>
+        <v>0.6663434343434343</v>
       </c>
       <c r="F21" t="n">
-        <v>0.3807676767676768</v>
+        <v>14894.78223835455</v>
       </c>
       <c r="G21" t="n">
-        <v>545.4911130608871</v>
+        <v>4497.546498834456</v>
       </c>
       <c r="H21" t="n">
-        <v>8050.089973234722</v>
-      </c>
-      <c r="I21" t="n">
-        <v>3058.472372575648</v>
-      </c>
-      <c r="J21" t="n">
-        <v>6354.913394019221</v>
+        <v>7277.692556146124</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="n">
-        <v>0.4728282828282828</v>
+        <v>0.7233333333333334</v>
       </c>
       <c r="B22" t="n">
-        <v>430.6567907517198</v>
+        <v>15512.6424565505</v>
       </c>
       <c r="C22" t="n">
-        <v>6051.09450389373</v>
+        <v>4273.587801873107</v>
       </c>
       <c r="D22" t="n">
-        <v>2943.415212321445</v>
+        <v>7139.695403705689</v>
       </c>
       <c r="E22" t="n">
-        <v>4946.360127308643</v>
+        <v>0.7014141414141415</v>
       </c>
       <c r="F22" t="n">
-        <v>0.4008080808080808</v>
+        <v>14703.94023103996</v>
       </c>
       <c r="G22" t="n">
-        <v>530.1250262547433</v>
+        <v>4414.167136321952</v>
       </c>
       <c r="H22" t="n">
-        <v>8120.38572527291</v>
-      </c>
-      <c r="I22" t="n">
-        <v>3037.596043911325</v>
-      </c>
-      <c r="J22" t="n">
-        <v>6271.714402665562</v>
+        <v>7158.592700026222</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="n">
-        <v>0.4964696969696969</v>
+        <v>0.7595</v>
       </c>
       <c r="B23" t="n">
-        <v>425.4534892153519</v>
+        <v>15284.00544495409</v>
       </c>
       <c r="C23" t="n">
-        <v>6114.979559225862</v>
+        <v>4199.451955438461</v>
       </c>
       <c r="D23" t="n">
-        <v>2904.153793871633</v>
+        <v>7002.467410544858</v>
       </c>
       <c r="E23" t="n">
-        <v>4909.491029526505</v>
+        <v>0.7364848484848485</v>
       </c>
       <c r="F23" t="n">
-        <v>0.4208484848484848</v>
+        <v>14511.05535405958</v>
       </c>
       <c r="G23" t="n">
-        <v>519.4103331397937</v>
+        <v>4325.365434187084</v>
       </c>
       <c r="H23" t="n">
-        <v>8183.721676254672</v>
-      </c>
-      <c r="I23" t="n">
-        <v>3016.971568671855</v>
-      </c>
-      <c r="J23" t="n">
-        <v>6189.506030086553</v>
+        <v>7028.987227523824</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="n">
-        <v>0.5201111111111111</v>
+        <v>0.7956666666666666</v>
       </c>
       <c r="B24" t="n">
-        <v>419.1937199567632</v>
+        <v>15042.00498262525</v>
       </c>
       <c r="C24" t="n">
-        <v>6178.616766079259</v>
+        <v>4121.868334288755</v>
       </c>
       <c r="D24" t="n">
-        <v>2866.396113941826</v>
+        <v>6861.321813380808</v>
       </c>
       <c r="E24" t="n">
-        <v>4872.631992674882</v>
+        <v>0.7715555555555556</v>
       </c>
       <c r="F24" t="n">
-        <v>0.4408888888888889</v>
+        <v>14316.1625600031</v>
       </c>
       <c r="G24" t="n">
-        <v>510.8657591289827</v>
+        <v>4231.089084409849</v>
       </c>
       <c r="H24" t="n">
-        <v>8239.088183711905</v>
-      </c>
-      <c r="I24" t="n">
-        <v>2996.539858135026</v>
-      </c>
-      <c r="J24" t="n">
-        <v>6105.314048473678</v>
+        <v>6887.826732537927</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="n">
-        <v>0.5437525252525253</v>
+        <v>0.8318333333333333</v>
       </c>
       <c r="B25" t="n">
-        <v>412.6257748311829</v>
+        <v>14792.5799576008</v>
       </c>
       <c r="C25" t="n">
-        <v>6241.017938469985</v>
+        <v>4040.584205732968</v>
       </c>
       <c r="D25" t="n">
-        <v>2829.031256296425</v>
+        <v>6717.164071823307</v>
       </c>
       <c r="E25" t="n">
-        <v>4835.780630190042</v>
+        <v>0.8066262626262627</v>
       </c>
       <c r="F25" t="n">
-        <v>0.4609292929292929</v>
+        <v>14119.2968014602</v>
       </c>
       <c r="G25" t="n">
-        <v>507.2876708528731</v>
+        <v>4135.503822411232</v>
       </c>
       <c r="H25" t="n">
-        <v>8287.458910734253</v>
-      </c>
-      <c r="I25" t="n">
-        <v>2976.241823578631</v>
-      </c>
-      <c r="J25" t="n">
-        <v>6012.919205532704</v>
+        <v>6738.827986163923</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="n">
-        <v>0.5673939393939393</v>
+        <v>0.868</v>
       </c>
       <c r="B26" t="n">
-        <v>405.8005996200005</v>
+        <v>14537.0636421949</v>
       </c>
       <c r="C26" t="n">
-        <v>6301.194890414103</v>
+        <v>3955.697878128658</v>
       </c>
       <c r="D26" t="n">
-        <v>2792.347844065059</v>
+        <v>6572.787961890905</v>
       </c>
       <c r="E26" t="n">
-        <v>4798.948186441286</v>
+        <v>0.8416969696969697</v>
       </c>
       <c r="F26" t="n">
-        <v>0.4809696969696969</v>
+        <v>13920.49303102057</v>
       </c>
       <c r="G26" t="n">
-        <v>511.8783448596097</v>
+        <v>4039.90149084446</v>
       </c>
       <c r="H26" t="n">
-        <v>8336.060747008743</v>
-      </c>
-      <c r="I26" t="n">
-        <v>2960.8514804897</v>
-      </c>
-      <c r="J26" t="n">
-        <v>5901.460208364874</v>
+        <v>6588.611152781132</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="n">
-        <v>0.5910353535353535</v>
+        <v>0.9041666666666667</v>
       </c>
       <c r="B27" t="n">
-        <v>398.9939615755933</v>
+        <v>14276.08406593561</v>
       </c>
       <c r="C27" t="n">
-        <v>6358.159435927678</v>
+        <v>3869.909054639823</v>
       </c>
       <c r="D27" t="n">
-        <v>2756.634500377355</v>
+        <v>6428.290713827078</v>
       </c>
       <c r="E27" t="n">
-        <v>4762.242270687074</v>
+        <v>0.8767676767676768</v>
       </c>
       <c r="F27" t="n">
-        <v>0.501010101010101</v>
+        <v>13719.7862012739</v>
       </c>
       <c r="G27" t="n">
-        <v>508.1043037260272</v>
+        <v>3944.281193279488</v>
       </c>
       <c r="H27" t="n">
-        <v>8383.006043966288</v>
-      </c>
-      <c r="I27" t="n">
-        <v>2956.298580880249</v>
-      </c>
-      <c r="J27" t="n">
-        <v>5782.580823694039</v>
+        <v>6437.459518785306</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="n">
-        <v>0.6146767676767676</v>
+        <v>0.9403333333333334</v>
       </c>
       <c r="B28" t="n">
-        <v>392.3619656535236</v>
+        <v>14010.269258351</v>
       </c>
       <c r="C28" t="n">
-        <v>6410.923389026772</v>
+        <v>3783.881261627669</v>
       </c>
       <c r="D28" t="n">
-        <v>2722.179848362943</v>
+        <v>6283.602324161471</v>
       </c>
       <c r="E28" t="n">
-        <v>4725.640799350064</v>
+        <v>0.9118383838383839</v>
       </c>
       <c r="F28" t="n">
-        <v>0.521050505050505</v>
+        <v>13517.21126480988</v>
       </c>
       <c r="G28" t="n">
-        <v>493.3372200838896</v>
+        <v>3848.642033286267</v>
       </c>
       <c r="H28" t="n">
-        <v>8425.217712958232</v>
-      </c>
-      <c r="I28" t="n">
-        <v>2955.296967621645</v>
-      </c>
-      <c r="J28" t="n">
-        <v>5670.289439426502</v>
+        <v>6285.601891119897</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="n">
-        <v>0.6383181818181818</v>
+        <v>0.9765</v>
       </c>
       <c r="B29" t="n">
-        <v>385.8130651904148</v>
+        <v>13740.24724896912</v>
       </c>
       <c r="C29" t="n">
-        <v>6458.498563727453</v>
+        <v>3697.670768942999</v>
       </c>
       <c r="D29" t="n">
-        <v>2688.825316156264</v>
+        <v>6138.65278942372</v>
       </c>
       <c r="E29" t="n">
-        <v>4689.087044590377</v>
+        <v>0.9469090909090909</v>
       </c>
       <c r="F29" t="n">
-        <v>0.5410909090909091</v>
+        <v>13312.80317421819</v>
       </c>
       <c r="G29" t="n">
-        <v>476.3129461646791</v>
+        <v>3752.983114434755</v>
       </c>
       <c r="H29" t="n">
-        <v>8459.618665335922</v>
-      </c>
-      <c r="I29" t="n">
-        <v>2950.19423618774</v>
-      </c>
-      <c r="J29" t="n">
-        <v>5578.594443468568</v>
+        <v>6133.267076728361</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="n">
-        <v>0.661959595959596</v>
+        <v>1.012666666666667</v>
       </c>
       <c r="B30" t="n">
-        <v>379.3555266845918</v>
+        <v>13466.64606731802</v>
       </c>
       <c r="C30" t="n">
-        <v>6499.896774045781</v>
+        <v>3611.333846436616</v>
       </c>
       <c r="D30" t="n">
-        <v>2655.781950071684</v>
+        <v>5993.372106143467</v>
       </c>
       <c r="E30" t="n">
-        <v>4652.524278568134</v>
+        <v>0.981979797979798</v>
       </c>
       <c r="F30" t="n">
-        <v>0.5611313131313131</v>
+        <v>13106.59688208853</v>
       </c>
       <c r="G30" t="n">
-        <v>464.2322878488595</v>
+        <v>3657.303540294904</v>
       </c>
       <c r="H30" t="n">
-        <v>8483.237525474706</v>
-      </c>
-      <c r="I30" t="n">
-        <v>2933.430992158958</v>
-      </c>
-      <c r="J30" t="n">
-        <v>5526.109811751687</v>
+        <v>5980.683882554144</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="n">
-        <v>0.68560101010101</v>
+        <v>1.048833333333333</v>
       </c>
       <c r="B31" t="n">
-        <v>372.9999717565862</v>
+        <v>13190.09374292579</v>
       </c>
       <c r="C31" t="n">
-        <v>6534.234387059149</v>
+        <v>3524.926763959322</v>
       </c>
       <c r="D31" t="n">
-        <v>2623.163113639309</v>
+        <v>5847.690270850348</v>
       </c>
       <c r="E31" t="n">
-        <v>4615.895773443448</v>
+        <v>1.017050505050505</v>
       </c>
       <c r="F31" t="n">
-        <v>0.5811717171717171</v>
+        <v>12898.62734101058</v>
       </c>
       <c r="G31" t="n">
-        <v>455.6822684318745</v>
+        <v>3561.602414436667</v>
       </c>
       <c r="H31" t="n">
-        <v>8499.516289749963</v>
-      </c>
-      <c r="I31" t="n">
-        <v>2904.767449588554</v>
-      </c>
-      <c r="J31" t="n">
-        <v>5506.319622405206</v>
+        <v>5828.081115540705</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="n">
-        <v>0.7092424242424242</v>
+        <v>1.085</v>
       </c>
       <c r="B32" t="n">
-        <v>366.6836521180621</v>
+        <v>12911.21830532046</v>
       </c>
       <c r="C32" t="n">
-        <v>6566.174730913884</v>
+        <v>3438.505791361922</v>
       </c>
       <c r="D32" t="n">
-        <v>2591.118763104572</v>
+        <v>5701.537280074006</v>
       </c>
       <c r="E32" t="n">
-        <v>4577.542421409027</v>
+        <v>1.052121212121212</v>
       </c>
       <c r="F32" t="n">
-        <v>0.6012121212121212</v>
+        <v>12688.92950357404</v>
       </c>
       <c r="G32" t="n">
-        <v>447.6097173271286</v>
+        <v>3465.878840430001</v>
       </c>
       <c r="H32" t="n">
-        <v>8512.603307716234</v>
-      </c>
-      <c r="I32" t="n">
-        <v>2869.541260128647</v>
-      </c>
-      <c r="J32" t="n">
-        <v>5490.514514362858</v>
+        <v>5675.68758263149</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="n">
-        <v>0.7328838383838383</v>
+        <v>1.121166666666667</v>
       </c>
       <c r="B33" t="n">
-        <v>360.3973758716846</v>
+        <v>12630.64778403011</v>
       </c>
       <c r="C33" t="n">
-        <v>6597.893575248001</v>
+        <v>3352.127198495219</v>
       </c>
       <c r="D33" t="n">
-        <v>2559.798854712912</v>
+        <v>5554.843130344079</v>
       </c>
       <c r="E33" t="n">
-        <v>4529.451993365768</v>
+        <v>1.087191919191919</v>
       </c>
       <c r="F33" t="n">
-        <v>0.6212525252525252</v>
+        <v>12477.53832236858</v>
       </c>
       <c r="G33" t="n">
-        <v>440.1525614807746</v>
+        <v>3370.131921844858</v>
       </c>
       <c r="H33" t="n">
-        <v>8524.122072151524</v>
-      </c>
-      <c r="I33" t="n">
-        <v>2831.761571193147</v>
-      </c>
-      <c r="J33" t="n">
-        <v>5450.02616431052</v>
+        <v>5523.732090769958</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="n">
-        <v>0.7565252525252525</v>
+        <v>1.157333333333333</v>
       </c>
       <c r="B34" t="n">
-        <v>354.1605796100892</v>
+        <v>12349.01020858279</v>
       </c>
       <c r="C34" t="n">
-        <v>6628.318410817437</v>
+        <v>3265.847255210015</v>
       </c>
       <c r="D34" t="n">
-        <v>2529.240064015699</v>
+        <v>5407.537818190205</v>
       </c>
       <c r="E34" t="n">
-        <v>4474.507374470011</v>
+        <v>1.122262626262626</v>
       </c>
       <c r="F34" t="n">
-        <v>0.6412929292929292</v>
+        <v>12264.4887499839</v>
       </c>
       <c r="G34" t="n">
-        <v>433.3526401266465</v>
+        <v>3274.360762251192</v>
       </c>
       <c r="H34" t="n">
-        <v>8535.696075833845</v>
-      </c>
-      <c r="I34" t="n">
-        <v>2795.437530195965</v>
-      </c>
-      <c r="J34" t="n">
-        <v>5390.780766785788</v>
+        <v>5372.44344689956</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="n">
-        <v>0.7801666666666667</v>
+        <v>1.1935</v>
       </c>
       <c r="B35" t="n">
-        <v>347.9525490750225</v>
+        <v>12066.93360850656</v>
       </c>
       <c r="C35" t="n">
-        <v>6656.376728378122</v>
+        <v>3179.722231357116</v>
       </c>
       <c r="D35" t="n">
-        <v>2498.962817209406</v>
+        <v>5259.551340142026</v>
       </c>
       <c r="E35" t="n">
-        <v>4417.438958910997</v>
+        <v>1.157333333333333</v>
       </c>
       <c r="F35" t="n">
-        <v>0.6613333333333333</v>
+        <v>12049.81573900969</v>
       </c>
       <c r="G35" t="n">
-        <v>429.2998719119789</v>
+        <v>3178.563109817148</v>
       </c>
       <c r="H35" t="n">
-        <v>8548.9488115412</v>
-      </c>
-      <c r="I35" t="n">
-        <v>2764.578284551013</v>
-      </c>
-      <c r="J35" t="n">
-        <v>5331.345125347491</v>
+        <v>5222.050457963746</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="n">
-        <v>0.8038080808080807</v>
+        <v>1.229666666666667</v>
       </c>
       <c r="B36" t="n">
-        <v>341.802944081653</v>
+        <v>11785.04601332947</v>
       </c>
       <c r="C36" t="n">
-        <v>6680.996018685989</v>
+        <v>3093.808396787322</v>
       </c>
       <c r="D36" t="n">
-        <v>2468.966416076752</v>
+        <v>5110.495407741039</v>
       </c>
       <c r="E36" t="n">
-        <v>4362.977140877961</v>
+        <v>1.19240404040404</v>
       </c>
       <c r="F36" t="n">
-        <v>0.6813737373737373</v>
+        <v>11833.55424203564</v>
       </c>
       <c r="G36" t="n">
-        <v>433.4626940562725</v>
+        <v>3082.719459081293</v>
       </c>
       <c r="H36" t="n">
-        <v>8568.307621727694</v>
-      </c>
-      <c r="I36" t="n">
-        <v>2739.98457347341</v>
-      </c>
-      <c r="J36" t="n">
-        <v>5271.355373764671</v>
+        <v>5072.668441850999</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="n">
-        <v>0.8274494949494949</v>
+        <v>1.265833333333333</v>
       </c>
       <c r="B37" t="n">
-        <v>335.8994561833159</v>
+        <v>11503.97545257961</v>
       </c>
       <c r="C37" t="n">
-        <v>6701.103772496969</v>
+        <v>3008.162021351439</v>
       </c>
       <c r="D37" t="n">
-        <v>2439.337038556927</v>
+        <v>4960.206008567165</v>
       </c>
       <c r="E37" t="n">
-        <v>4315.85231456014</v>
+        <v>1.227474747474748</v>
       </c>
       <c r="F37" t="n">
-        <v>0.7014141414141414</v>
+        <v>11615.73921165143</v>
       </c>
       <c r="G37" t="n">
-        <v>430.9788534842766</v>
+        <v>2986.832613394722</v>
       </c>
       <c r="H37" t="n">
-        <v>8597.652098493323</v>
-      </c>
-      <c r="I37" t="n">
-        <v>2715.74274649979</v>
-      </c>
-      <c r="J37" t="n">
-        <v>5210.447645806368</v>
+        <v>4923.477508557384</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="n">
-        <v>0.851090909090909</v>
+        <v>1.302</v>
       </c>
       <c r="B38" t="n">
-        <v>329.9802514690314</v>
+        <v>11224.34995578501</v>
       </c>
       <c r="C38" t="n">
-        <v>6715.627480566999</v>
+        <v>2922.729177964994</v>
       </c>
       <c r="D38" t="n">
-        <v>2410.160862589119</v>
+        <v>4808.949553207667</v>
       </c>
       <c r="E38" t="n">
-        <v>4280.717103619624</v>
+        <v>1.262545454545455</v>
       </c>
       <c r="F38" t="n">
-        <v>0.7214545454545453</v>
+        <v>11396.40560044675</v>
       </c>
       <c r="G38" t="n">
-        <v>418.1498768456062</v>
+        <v>2890.914180725715</v>
       </c>
       <c r="H38" t="n">
-        <v>8629.595844592013</v>
-      </c>
-      <c r="I38" t="n">
-        <v>2691.82062268032</v>
-      </c>
-      <c r="J38" t="n">
-        <v>5148.34814309725</v>
+        <v>4774.330103712502</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="n">
-        <v>0.8747323232323232</v>
+        <v>1.338166666666667</v>
       </c>
       <c r="B39" t="n">
-        <v>320.7812946227391</v>
+        <v>10946.79755247374</v>
       </c>
       <c r="C39" t="n">
-        <v>6723.494633652009</v>
+        <v>2837.354814357551</v>
       </c>
       <c r="D39" t="n">
-        <v>2381.504760934612</v>
+        <v>4656.992452249816</v>
       </c>
       <c r="E39" t="n">
-        <v>4257.480579007199</v>
+        <v>1.297616161616162</v>
       </c>
       <c r="F39" t="n">
-        <v>0.7414949494949494</v>
+        <v>11175.56209863386</v>
       </c>
       <c r="G39" t="n">
-        <v>402.4491903859934</v>
+        <v>2794.97576904255</v>
       </c>
       <c r="H39" t="n">
-        <v>8656.309418278954</v>
-      </c>
-      <c r="I39" t="n">
-        <v>2668.532228958447</v>
-      </c>
-      <c r="J39" t="n">
-        <v>5085.684331061922</v>
+        <v>4625.303533333908</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="n">
-        <v>0.8983737373737374</v>
+        <v>1.374333333333333</v>
       </c>
       <c r="B40" t="n">
-        <v>309.1067261403045</v>
+        <v>10671.94627217386</v>
       </c>
       <c r="C40" t="n">
-        <v>6723.632722507931</v>
+        <v>2752.049490453433</v>
       </c>
       <c r="D40" t="n">
-        <v>2353.110706778622</v>
+        <v>4504.601116280875</v>
       </c>
       <c r="E40" t="n">
-        <v>4240.533164158561</v>
+        <v>1.332686868686869</v>
       </c>
       <c r="F40" t="n">
-        <v>0.7615353535353535</v>
+        <v>10952.93011701001</v>
       </c>
       <c r="G40" t="n">
-        <v>389.7209586482953</v>
+        <v>2699.028986313509</v>
       </c>
       <c r="H40" t="n">
-        <v>8669.963377809343</v>
-      </c>
-      <c r="I40" t="n">
-        <v>2646.185193564489</v>
-      </c>
-      <c r="J40" t="n">
-        <v>5022.92963730616</v>
+        <v>4476.47510343916</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="n">
-        <v>0.9220151515151515</v>
+        <v>1.4105</v>
       </c>
       <c r="B41" t="n">
-        <v>302.6003436088359</v>
+        <v>10400.42414441343</v>
       </c>
       <c r="C41" t="n">
-        <v>6715.453644203507</v>
+        <v>2666.826681643555</v>
       </c>
       <c r="D41" t="n">
-        <v>2324.912613144795</v>
+        <v>4352.041955888115</v>
       </c>
       <c r="E41" t="n">
-        <v>4224.01290665659</v>
+        <v>1.367757575757576</v>
       </c>
       <c r="F41" t="n">
-        <v>0.7815757575757575</v>
+        <v>10728.61742877964</v>
       </c>
       <c r="G41" t="n">
-        <v>380.5482156718352</v>
+        <v>2603.08544050687</v>
       </c>
       <c r="H41" t="n">
-        <v>8662.701950133685</v>
-      </c>
-      <c r="I41" t="n">
-        <v>2624.296521903761</v>
-      </c>
-      <c r="J41" t="n">
-        <v>4960.427764620254</v>
+        <v>4327.922120045818</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="n">
-        <v>0.9456565656565656</v>
+        <v>1.446666666666667</v>
       </c>
       <c r="B42" t="n">
-        <v>305.2998391607882</v>
+        <v>10132.85919872051</v>
       </c>
       <c r="C42" t="n">
-        <v>6705.069318379376</v>
+        <v>2581.699863318831</v>
       </c>
       <c r="D42" t="n">
-        <v>2296.963334262897</v>
+        <v>4199.581381658799</v>
       </c>
       <c r="E42" t="n">
-        <v>4202.057854084171</v>
+        <v>1.402828282828283</v>
       </c>
       <c r="F42" t="n">
-        <v>0.8016161616161616</v>
+        <v>10502.87018426743</v>
       </c>
       <c r="G42" t="n">
-        <v>373.2760683740595</v>
+        <v>2507.156739590913</v>
       </c>
       <c r="H42" t="n">
-        <v>8630.828446260384</v>
-      </c>
-      <c r="I42" t="n">
-        <v>2602.407859869885</v>
-      </c>
-      <c r="J42" t="n">
-        <v>4898.522415794494</v>
+        <v>4179.721889171438</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="n">
-        <v>0.9692979797979797</v>
+        <v>1.482833333333333</v>
       </c>
       <c r="B43" t="n">
-        <v>303.7150590236315</v>
+        <v>9869.879464623158</v>
       </c>
       <c r="C43" t="n">
-        <v>6694.631044697471</v>
+        <v>2496.682510870177</v>
       </c>
       <c r="D43" t="n">
-        <v>2269.315724362698</v>
+        <v>4047.485804180198</v>
       </c>
       <c r="E43" t="n">
-        <v>4169.77742583523</v>
+        <v>1.43789898989899</v>
       </c>
       <c r="F43" t="n">
-        <v>0.8216565656565656</v>
+        <v>10275.93453379807</v>
       </c>
       <c r="G43" t="n">
-        <v>371.7005633013539</v>
+        <v>2411.254491533919</v>
       </c>
       <c r="H43" t="n">
-        <v>8580.511537946273</v>
-      </c>
-      <c r="I43" t="n">
-        <v>2580.519354236514</v>
-      </c>
-      <c r="J43" t="n">
-        <v>4837.272987147026</v>
+        <v>4031.951716833582</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="n">
-        <v>0.9929393939393939</v>
+        <v>1.519</v>
       </c>
       <c r="B44" t="n">
-        <v>299.2488492912372</v>
+        <v>9612.112971649432</v>
       </c>
       <c r="C44" t="n">
-        <v>6684.143129848037</v>
+        <v>2411.788099688507</v>
       </c>
       <c r="D44" t="n">
-        <v>2242.022403545883</v>
+        <v>3896.021634039575</v>
       </c>
       <c r="E44" t="n">
-        <v>4134.494058189968</v>
+        <v>1.472969696969697</v>
       </c>
       <c r="F44" t="n">
-        <v>0.8416969696969696</v>
+        <v>10048.05662769625</v>
       </c>
       <c r="G44" t="n">
-        <v>374.8406442679709</v>
+        <v>2315.390304304166</v>
       </c>
       <c r="H44" t="n">
-        <v>8519.178123393684</v>
-      </c>
-      <c r="I44" t="n">
-        <v>2558.631151777301</v>
-      </c>
-      <c r="J44" t="n">
-        <v>4776.213218840374</v>
+        <v>3884.688909049805</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="n">
-        <v>1.016580808080808</v>
+        <v>1.555166666666667</v>
       </c>
       <c r="B45" t="n">
-        <v>294.4389314638427</v>
+        <v>9360.121022165929</v>
       </c>
       <c r="C45" t="n">
-        <v>6673.609880521308</v>
+        <v>2327.030105164735</v>
       </c>
       <c r="D45" t="n">
-        <v>2214.973190137259</v>
+        <v>3745.4552818242</v>
       </c>
       <c r="E45" t="n">
-        <v>4098.885710100786</v>
+        <v>1.508040404040404</v>
       </c>
       <c r="F45" t="n">
-        <v>0.8617373737373737</v>
+        <v>9819.482616286647</v>
       </c>
       <c r="G45" t="n">
-        <v>368.4573476672293</v>
+        <v>2219.575785869935</v>
       </c>
       <c r="H45" t="n">
-        <v>8454.255100804941</v>
-      </c>
-      <c r="I45" t="n">
-        <v>2536.743364668215</v>
-      </c>
-      <c r="J45" t="n">
-        <v>4715.317577503697</v>
+        <v>3738.010771837667</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="n">
-        <v>1.040222222222222</v>
+        <v>1.591333333333333</v>
       </c>
       <c r="B46" t="n">
-        <v>289.2082682972321</v>
+        <v>9110.370807388934</v>
       </c>
       <c r="C46" t="n">
-        <v>6663.03560340753</v>
+        <v>2242.422002689778</v>
       </c>
       <c r="D46" t="n">
-        <v>2188.06807987283</v>
+        <v>3596.053158121339</v>
       </c>
       <c r="E46" t="n">
-        <v>4062.703238460052</v>
+        <v>1.543111111111111</v>
       </c>
       <c r="F46" t="n">
-        <v>0.8817777777777778</v>
+        <v>9590.458649893953</v>
       </c>
       <c r="G46" t="n">
-        <v>354.3092289695824</v>
+        <v>2123.950424705885</v>
       </c>
       <c r="H46" t="n">
-        <v>8393.169368382381</v>
-      </c>
-      <c r="I46" t="n">
-        <v>2514.855813779936</v>
-      </c>
-      <c r="J46" t="n">
-        <v>4654.580030159749</v>
+        <v>3591.994611214725</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="n">
-        <v>1.063863636363636</v>
+        <v>1.6275</v>
       </c>
       <c r="B47" t="n">
-        <v>283.940774927812</v>
+        <v>8860.723425639484</v>
       </c>
       <c r="C47" t="n">
-        <v>6652.424605196941</v>
+        <v>2157.977267654549</v>
       </c>
       <c r="D47" t="n">
-        <v>2161.34087829773</v>
+        <v>3449.0142394313</v>
       </c>
       <c r="E47" t="n">
-        <v>4025.697500160137</v>
+        <v>1.578181818181818</v>
       </c>
       <c r="F47" t="n">
-        <v>0.9018181818181817</v>
+        <v>9361.230878842855</v>
       </c>
       <c r="G47" t="n">
-        <v>339.5240776627099</v>
+        <v>2031.345644387354</v>
       </c>
       <c r="H47" t="n">
-        <v>8343.177225297768</v>
-      </c>
-      <c r="I47" t="n">
-        <v>2492.968378842835</v>
-      </c>
-      <c r="J47" t="n">
-        <v>4593.996335343457</v>
+        <v>3447.100544555624</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="n">
-        <v>1.087505050505051</v>
+        <v>1.663666666666667</v>
       </c>
       <c r="B48" t="n">
-        <v>278.7223071770874</v>
+        <v>8611.391257229088</v>
       </c>
       <c r="C48" t="n">
-        <v>6641.781192579784</v>
+        <v>2073.709375449962</v>
       </c>
       <c r="D48" t="n">
-        <v>2134.825390957092</v>
+        <v>3305.942456592344</v>
       </c>
       <c r="E48" t="n">
-        <v>3987.619352093408</v>
+        <v>1.613252525252525</v>
       </c>
       <c r="F48" t="n">
-        <v>0.9218585858585858</v>
+        <v>9132.045453458033</v>
       </c>
       <c r="G48" t="n">
-        <v>329.7173515056626</v>
+        <v>1942.675072762396</v>
       </c>
       <c r="H48" t="n">
-        <v>8299.405421722564</v>
-      </c>
-      <c r="I48" t="n">
-        <v>2471.080975723763</v>
-      </c>
-      <c r="J48" t="n">
-        <v>4533.652637090393</v>
+        <v>3307.487155704769</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="n">
-        <v>1.111146464646465</v>
+        <v>1.699833333333333</v>
       </c>
       <c r="B49" t="n">
-        <v>273.5318336521413</v>
+        <v>8362.586682469266</v>
       </c>
       <c r="C49" t="n">
-        <v>6631.109672246299</v>
+        <v>1989.764202247677</v>
       </c>
       <c r="D49" t="n">
-        <v>2108.55542339605</v>
+        <v>3166.709416885195</v>
       </c>
       <c r="E49" t="n">
-        <v>3948.388659393067</v>
+        <v>1.648323232323232</v>
       </c>
       <c r="F49" t="n">
-        <v>0.9418989898989898</v>
+        <v>8903.148524064178</v>
       </c>
       <c r="G49" t="n">
-        <v>321.8476157201148</v>
+        <v>1857.612926188786</v>
       </c>
       <c r="H49" t="n">
-        <v>8256.486826285054</v>
-      </c>
-      <c r="I49" t="n">
-        <v>2449.193520289568</v>
-      </c>
-      <c r="J49" t="n">
-        <v>4473.527662894822</v>
+        <v>3173.827705303739</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="n">
-        <v>1.134787878787879</v>
+        <v>1.736</v>
       </c>
       <c r="B50" t="n">
-        <v>268.353556248397</v>
+        <v>8114.522081671526</v>
       </c>
       <c r="C50" t="n">
-        <v>6620.414350886725</v>
+        <v>1908.369908774906</v>
       </c>
       <c r="D50" t="n">
-        <v>2082.503228922636</v>
+        <v>3031.159387118688</v>
       </c>
       <c r="E50" t="n">
-        <v>3909.04078362462</v>
+        <v>1.683393939393939</v>
       </c>
       <c r="F50" t="n">
-        <v>0.9619393939393939</v>
+        <v>8674.786240985981</v>
       </c>
       <c r="G50" t="n">
-        <v>314.4237668963621</v>
+        <v>1775.8334210243</v>
       </c>
       <c r="H50" t="n">
-        <v>8214.523896703839</v>
-      </c>
-      <c r="I50" t="n">
-        <v>2427.107135142982</v>
-      </c>
-      <c r="J50" t="n">
-        <v>4413.521704785594</v>
+        <v>3045.558808035288</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="n">
-        <v>1.158429292929293</v>
+        <v>1.772166666666667</v>
       </c>
       <c r="B51" t="n">
-        <v>263.213990865257</v>
+        <v>7867.409835147389</v>
       </c>
       <c r="C51" t="n">
-        <v>6609.702445169305</v>
+        <v>1830.137569532137</v>
       </c>
       <c r="D51" t="n">
-        <v>2056.567095406027</v>
+        <v>2899.13663410166</v>
       </c>
       <c r="E51" t="n">
-        <v>3869.682784499024</v>
+        <v>1.718464646464646</v>
       </c>
       <c r="F51" t="n">
-        <v>0.981979797979798</v>
+        <v>8447.204754548116</v>
       </c>
       <c r="G51" t="n">
-        <v>307.5588329725423</v>
+        <v>1697.010773626711</v>
       </c>
       <c r="H51" t="n">
-        <v>8173.619090697514</v>
-      </c>
-      <c r="I51" t="n">
-        <v>2404.579411018615</v>
-      </c>
-      <c r="J51" t="n">
-        <v>4353.535054791565</v>
+        <v>2922.117078582171</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="n">
-        <v>1.182070707070707</v>
+        <v>1.808333333333333</v>
       </c>
       <c r="B52" t="n">
-        <v>258.0876977098647</v>
+        <v>7621.462323208366</v>
       </c>
       <c r="C52" t="n">
-        <v>6598.991223806432</v>
+        <v>1754.829387432965</v>
       </c>
       <c r="D52" t="n">
-        <v>2030.765153058229</v>
+        <v>2770.485424642947</v>
       </c>
       <c r="E52" t="n">
-        <v>3830.175463599038</v>
+        <v>1.753535353535354</v>
       </c>
       <c r="F52" t="n">
-        <v>1.002020202020202</v>
+        <v>8220.650215075286</v>
       </c>
       <c r="G52" t="n">
-        <v>301.2372782805837</v>
+        <v>1620.819200353794</v>
       </c>
       <c r="H52" t="n">
-        <v>8133.874865984676</v>
-      </c>
-      <c r="I52" t="n">
-        <v>2381.853204080512</v>
-      </c>
-      <c r="J52" t="n">
-        <v>4293.688011667298</v>
+        <v>2802.939131627145</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="n">
-        <v>1.205712121212121</v>
+        <v>1.8445</v>
       </c>
       <c r="B53" t="n">
-        <v>252.9644646612571</v>
+        <v>7376.891926165971</v>
       </c>
       <c r="C53" t="n">
-        <v>6588.273446485336</v>
+        <v>1682.207565390985</v>
       </c>
       <c r="D53" t="n">
-        <v>2005.119558016386</v>
+        <v>2645.050025551386</v>
       </c>
       <c r="E53" t="n">
-        <v>3790.379622507424</v>
+        <v>1.788606060606061</v>
       </c>
       <c r="F53" t="n">
-        <v>1.022060606060606</v>
+        <v>7995.36877289216</v>
       </c>
       <c r="G53" t="n">
-        <v>298.5609813925547</v>
+        <v>1546.932917563325</v>
       </c>
       <c r="H53" t="n">
-        <v>8102.498164002408</v>
-      </c>
-      <c r="I53" t="n">
-        <v>2359.18227496949</v>
-      </c>
-      <c r="J53" t="n">
-        <v>4234.994749375349</v>
+        <v>2687.461581852965</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="n">
-        <v>1.229353535353535</v>
+        <v>1.880666666666667</v>
       </c>
       <c r="B54" t="n">
-        <v>247.8454498298177</v>
+        <v>7133.911024331719</v>
       </c>
       <c r="C54" t="n">
-        <v>6577.537858598625</v>
+        <v>1612.034306319789</v>
       </c>
       <c r="D54" t="n">
-        <v>1979.652466417641</v>
+        <v>2522.674703635811</v>
       </c>
       <c r="E54" t="n">
-        <v>3750.15606280694</v>
+        <v>1.823676767676768</v>
       </c>
       <c r="F54" t="n">
-        <v>1.04210101010101</v>
+        <v>7771.606578323436</v>
       </c>
       <c r="G54" t="n">
-        <v>300.886475725653</v>
+        <v>1475.026141613078</v>
       </c>
       <c r="H54" t="n">
-        <v>8091.974256924526</v>
-      </c>
-      <c r="I54" t="n">
-        <v>2337.063380012346</v>
-      </c>
-      <c r="J54" t="n">
-        <v>4177.048717373336</v>
+        <v>2575.121043942387</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="n">
-        <v>1.252994949494949</v>
+        <v>1.916833333333333</v>
       </c>
       <c r="B55" t="n">
-        <v>242.7331860754865</v>
+        <v>6892.731998017125</v>
       </c>
       <c r="C55" t="n">
-        <v>6566.773205538907</v>
+        <v>1544.071813132974</v>
       </c>
       <c r="D55" t="n">
-        <v>1954.366759869023</v>
+        <v>2403.203725705059</v>
       </c>
       <c r="E55" t="n">
-        <v>3709.452015205816</v>
+        <v>1.858747474747475</v>
       </c>
       <c r="F55" t="n">
-        <v>1.062141414141414</v>
+        <v>7549.609781693796</v>
       </c>
       <c r="G55" t="n">
-        <v>295.7131282856749</v>
+        <v>1404.773088860828</v>
       </c>
       <c r="H55" t="n">
-        <v>8090.64547534335</v>
-      </c>
-      <c r="I55" t="n">
-        <v>2323.786851894931</v>
-      </c>
-      <c r="J55" t="n">
-        <v>4119.200451902005</v>
+        <v>2465.354132578167</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="n">
-        <v>1.276636363636364</v>
+        <v>1.953</v>
       </c>
       <c r="B56" t="n">
-        <v>237.6290068884956</v>
+        <v>6653.567227533704</v>
       </c>
       <c r="C56" t="n">
-        <v>6555.968232698787</v>
+        <v>1478.082288744133</v>
       </c>
       <c r="D56" t="n">
-        <v>1929.186210009029</v>
+        <v>2286.481358567968</v>
       </c>
       <c r="E56" t="n">
-        <v>3668.619067460276</v>
+        <v>1.893818181818182</v>
       </c>
       <c r="F56" t="n">
-        <v>1.082181818181818</v>
+        <v>7329.624533327927</v>
       </c>
       <c r="G56" t="n">
-        <v>283.6390255766435</v>
+        <v>1335.84797566435</v>
       </c>
       <c r="H56" t="n">
-        <v>8085.686813642768</v>
-      </c>
-      <c r="I56" t="n">
-        <v>2318.132562527263</v>
-      </c>
-      <c r="J56" t="n">
-        <v>4060.800489202094</v>
+        <v>2357.59746244306</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="n">
-        <v>1.300277777777778</v>
+        <v>1.989166666666667</v>
       </c>
       <c r="B57" t="n">
-        <v>232.6777469132048</v>
+        <v>6416.629093192967</v>
       </c>
       <c r="C57" t="n">
-        <v>6545.111685470875</v>
+        <v>1413.82793606686</v>
       </c>
       <c r="D57" t="n">
-        <v>1904.112774519198</v>
+        <v>2172.351869033371</v>
       </c>
       <c r="E57" t="n">
-        <v>3627.728374924267</v>
+        <v>1.928888888888889</v>
       </c>
       <c r="F57" t="n">
-        <v>1.102222222222222</v>
+        <v>7111.917529375508</v>
       </c>
       <c r="G57" t="n">
-        <v>270.2807757770113</v>
+        <v>1267.958234187432</v>
       </c>
       <c r="H57" t="n">
-        <v>8064.27326620667</v>
-      </c>
-      <c r="I57" t="n">
-        <v>2312.990158936556</v>
-      </c>
-      <c r="J57" t="n">
-        <v>3991.770825512808</v>
+        <v>2251.287648219821</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="n">
-        <v>1.323919191919192</v>
+        <v>2.025333333333333</v>
       </c>
       <c r="B58" t="n">
-        <v>227.782290687174</v>
+        <v>6182.129975306434</v>
       </c>
       <c r="C58" t="n">
-        <v>6534.192309247776</v>
+        <v>1351.070958014749</v>
       </c>
       <c r="D58" t="n">
-        <v>1879.161094426031</v>
+        <v>2061.387599700171</v>
       </c>
       <c r="E58" t="n">
-        <v>3586.798409640186</v>
+        <v>1.963959595959596</v>
       </c>
       <c r="F58" t="n">
-        <v>1.122262626262626</v>
+        <v>6897.369829863201</v>
       </c>
       <c r="G58" t="n">
-        <v>260.0437022538146</v>
+        <v>1201.987491088448</v>
       </c>
       <c r="H58" t="n">
-        <v>8014.252282535206</v>
-      </c>
-      <c r="I58" t="n">
-        <v>2301.249288150024</v>
-      </c>
-      <c r="J58" t="n">
-        <v>3903.894636950037</v>
+        <v>2145.969792862068</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="n">
-        <v>1.347560606060606</v>
+        <v>2.0615</v>
       </c>
       <c r="B59" t="n">
-        <v>221.625263044545</v>
+        <v>5950.282254185612</v>
       </c>
       <c r="C59" t="n">
-        <v>6523.1988494221</v>
+        <v>1289.573557501394</v>
       </c>
       <c r="D59" t="n">
-        <v>1854.345810756032</v>
+        <v>1955.422269814876</v>
       </c>
       <c r="E59" t="n">
-        <v>3545.84764365043</v>
+        <v>1.999030303030303</v>
       </c>
       <c r="F59" t="n">
-        <v>1.14230303030303</v>
+        <v>6686.325733766036</v>
       </c>
       <c r="G59" t="n">
-        <v>252.0566888553832</v>
+        <v>1138.453036271077</v>
       </c>
       <c r="H59" t="n">
-        <v>7938.60187567658</v>
-      </c>
-      <c r="I59" t="n">
-        <v>2276.893752029626</v>
-      </c>
-      <c r="J59" t="n">
-        <v>3810.601072200572</v>
+        <v>2042.856874903511</v>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="n">
-        <v>1.37120202020202</v>
+        <v>2.097666666666667</v>
       </c>
       <c r="B60" t="n">
-        <v>212.2509408756039</v>
+        <v>5721.298310142022</v>
       </c>
       <c r="C60" t="n">
-        <v>6511.858022217378</v>
+        <v>1229.09793744039</v>
       </c>
       <c r="D60" t="n">
-        <v>1829.677691369941</v>
+        <v>1854.376286538843</v>
       </c>
       <c r="E60" t="n">
-        <v>3504.894548997396</v>
+        <v>2.03410101010101</v>
       </c>
       <c r="F60" t="n">
-        <v>1.162343434343434</v>
+        <v>6478.756063531543</v>
       </c>
       <c r="G60" t="n">
-        <v>245.6840846147143</v>
+        <v>1077.350910390705</v>
       </c>
       <c r="H60" t="n">
-        <v>7846.869546368427</v>
-      </c>
-      <c r="I60" t="n">
-        <v>2242.868632468879</v>
-      </c>
-      <c r="J60" t="n">
-        <v>3725.619136616024</v>
+        <v>1942.514118845788</v>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="n">
-        <v>1.394843434343434</v>
+        <v>2.133833333333333</v>
       </c>
       <c r="B61" t="n">
-        <v>204.8030751171754</v>
+        <v>5495.390523487173</v>
       </c>
       <c r="C61" t="n">
-        <v>6496.26851282281</v>
+        <v>1169.747639309484</v>
       </c>
       <c r="D61" t="n">
-        <v>1805.110522892248</v>
+        <v>1758.053008330821</v>
       </c>
       <c r="E61" t="n">
-        <v>3463.911425780308</v>
+        <v>2.069171717171717</v>
       </c>
       <c r="F61" t="n">
-        <v>1.182383838383838</v>
+        <v>6274.631641607239</v>
       </c>
       <c r="G61" t="n">
-        <v>244.8291020677349</v>
+        <v>1018.677154102716</v>
       </c>
       <c r="H61" t="n">
-        <v>7746.98292294224</v>
-      </c>
-      <c r="I61" t="n">
-        <v>2203.660529952906</v>
-      </c>
-      <c r="J61" t="n">
-        <v>3662.918706758177</v>
+        <v>1845.033274946947</v>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="n">
-        <v>1.418484848484848</v>
+        <v>2.17</v>
       </c>
       <c r="B62" t="n">
-        <v>204.9311810497174</v>
+        <v>5272.771274532586</v>
       </c>
       <c r="C62" t="n">
-        <v>6475.474048301112</v>
+        <v>1112.343616393237</v>
       </c>
       <c r="D62" t="n">
-        <v>1780.634108033587</v>
+        <v>1666.25579364956</v>
       </c>
       <c r="E62" t="n">
-        <v>3422.763983808943</v>
+        <v>2.104242424242424</v>
       </c>
       <c r="F62" t="n">
-        <v>1.202424242424242</v>
+        <v>6073.923290440654</v>
       </c>
       <c r="G62" t="n">
-        <v>245.2788697277825</v>
+        <v>962.4278080624958</v>
       </c>
       <c r="H62" t="n">
-        <v>7646.869633729517</v>
-      </c>
-      <c r="I62" t="n">
-        <v>2163.352416794874</v>
-      </c>
-      <c r="J62" t="n">
-        <v>3633.947361956281</v>
+        <v>1750.506093465038</v>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="n">
-        <v>1.442126262626263</v>
+        <v>2.206166666666667</v>
       </c>
       <c r="B63" t="n">
-        <v>205.3287642672192</v>
+        <v>5053.652943589768</v>
       </c>
       <c r="C63" t="n">
-        <v>6449.920441338441</v>
+        <v>1056.937617864622</v>
       </c>
       <c r="D63" t="n">
-        <v>1756.258021589349</v>
+        <v>1578.788000953812</v>
       </c>
       <c r="E63" t="n">
-        <v>3381.471878968078</v>
+        <v>2.139313131313131</v>
       </c>
       <c r="F63" t="n">
-        <v>1.222464646464646</v>
+        <v>5876.601832479309</v>
       </c>
       <c r="G63" t="n">
-        <v>237.585207394349</v>
+        <v>908.5989129254294</v>
       </c>
       <c r="H63" t="n">
-        <v>7554.457307061753</v>
-      </c>
-      <c r="I63" t="n">
-        <v>2126.027265307949</v>
-      </c>
-      <c r="J63" t="n">
-        <v>3622.720277434838</v>
+        <v>1659.024324658109</v>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="n">
-        <v>1.465767676767677</v>
+        <v>2.242333333333333</v>
       </c>
       <c r="B64" t="n">
-        <v>201.5610861344743</v>
+        <v>4838.247910970239</v>
       </c>
       <c r="C64" t="n">
-        <v>6420.05350462096</v>
+        <v>1003.530019168956</v>
       </c>
       <c r="D64" t="n">
-        <v>1731.991838354928</v>
+        <v>1495.452988702328</v>
       </c>
       <c r="E64" t="n">
-        <v>3340.068579532088</v>
+        <v>2.174383838383839</v>
       </c>
       <c r="F64" t="n">
-        <v>1.24250505050505</v>
+        <v>5682.63809017073</v>
       </c>
       <c r="G64" t="n">
-        <v>225.5200008605781</v>
+        <v>857.1865093469019</v>
       </c>
       <c r="H64" t="n">
-        <v>7477.497530636603</v>
-      </c>
-      <c r="I64" t="n">
-        <v>2095.681892981653</v>
-      </c>
-      <c r="J64" t="n">
-        <v>3606.467417053197</v>
+        <v>1570.679718784209</v>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="n">
-        <v>1.489409090909091</v>
+        <v>2.2785</v>
       </c>
       <c r="B65" t="n">
-        <v>197.6008662120093</v>
+        <v>4626.768556985509</v>
       </c>
       <c r="C65" t="n">
-        <v>6386.319050834828</v>
+        <v>952.1211957515543</v>
       </c>
       <c r="D65" t="n">
-        <v>1707.845038363085</v>
+        <v>1416.054115353857</v>
       </c>
       <c r="E65" t="n">
-        <v>3298.58755377535</v>
+        <v>2.209454545454546</v>
       </c>
       <c r="F65" t="n">
-        <v>1.262545454545454</v>
+        <v>5492.002885962439</v>
       </c>
       <c r="G65" t="n">
-        <v>213.9801486185097</v>
+        <v>808.1866379822976</v>
       </c>
       <c r="H65" t="n">
-        <v>7408.483429931175</v>
-      </c>
-      <c r="I65" t="n">
-        <v>2068.888817553861</v>
-      </c>
-      <c r="J65" t="n">
-        <v>3565.219878560456</v>
+        <v>1485.564026101388</v>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="n">
-        <v>1.513050505050505</v>
+        <v>2.314666666666667</v>
       </c>
       <c r="B66" t="n">
-        <v>193.2955913070484</v>
+        <v>4419.461045452681</v>
       </c>
       <c r="C66" t="n">
-        <v>6349.162892666208</v>
+        <v>902.7115230577361</v>
       </c>
       <c r="D66" t="n">
-        <v>1683.7968677094</v>
+        <v>1340.394739367152</v>
       </c>
       <c r="E66" t="n">
-        <v>3257.062269972242</v>
+        <v>2.244525252525253</v>
       </c>
       <c r="F66" t="n">
-        <v>1.282585858585858</v>
+        <v>5304.667042301961</v>
       </c>
       <c r="G66" t="n">
-        <v>206.2737851884465</v>
+        <v>761.5953394870023</v>
       </c>
       <c r="H66" t="n">
-        <v>7339.671991676648</v>
-      </c>
-      <c r="I66" t="n">
-        <v>2042.240576325594</v>
-      </c>
-      <c r="J66" t="n">
-        <v>3515.976191995514</v>
+        <v>1403.768996867694</v>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="n">
-        <v>1.536691919191919</v>
+        <v>2.350833333333333</v>
       </c>
       <c r="B67" t="n">
-        <v>188.8791107305254</v>
+        <v>4218.519436529325</v>
       </c>
       <c r="C67" t="n">
-        <v>6309.030842801261</v>
+        <v>855.3013765328168</v>
       </c>
       <c r="D67" t="n">
-        <v>1659.830288857087</v>
+        <v>1268.278219200963</v>
       </c>
       <c r="E67" t="n">
-        <v>3212.444848865189</v>
+        <v>2.27959595959596</v>
       </c>
       <c r="F67" t="n">
-        <v>1.302626262626263</v>
+        <v>5120.60138163682</v>
       </c>
       <c r="G67" t="n">
-        <v>199.416633575962</v>
+        <v>717.4086545164006</v>
       </c>
       <c r="H67" t="n">
-        <v>7270.915782090681</v>
-      </c>
-      <c r="I67" t="n">
-        <v>2016.073162854767</v>
-      </c>
-      <c r="J67" t="n">
-        <v>3466.179771594055</v>
+        <v>1325.386381341175</v>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="n">
-        <v>1.560333333333333</v>
+        <v>2.387</v>
       </c>
       <c r="B68" t="n">
-        <v>184.4987693233337</v>
+        <v>4025.053388437386</v>
       </c>
       <c r="C68" t="n">
-        <v>6266.368713926146</v>
+        <v>809.891131622113</v>
       </c>
       <c r="D68" t="n">
-        <v>1635.951331850168</v>
+        <v>1199.507913314039</v>
       </c>
       <c r="E68" t="n">
-        <v>3159.282553111103</v>
+        <v>2.314666666666667</v>
       </c>
       <c r="F68" t="n">
-        <v>1.322666666666667</v>
+        <v>4939.776726414541</v>
       </c>
       <c r="G68" t="n">
-        <v>192.9867974733031</v>
+        <v>675.6094419186585</v>
       </c>
       <c r="H68" t="n">
-        <v>7202.067367390931</v>
-      </c>
-      <c r="I68" t="n">
-        <v>1990.722570699296</v>
-      </c>
-      <c r="J68" t="n">
-        <v>3415.303386394972</v>
+        <v>1250.507929779881</v>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="n">
-        <v>1.583974747474747</v>
+        <v>2.423166666666666</v>
       </c>
       <c r="B69" t="n">
-        <v>180.1884147572049</v>
+        <v>3838.911851575851</v>
       </c>
       <c r="C69" t="n">
-        <v>6221.622318727024</v>
+        <v>766.4811637709423</v>
       </c>
       <c r="D69" t="n">
-        <v>1612.16602673267</v>
+        <v>1133.166877809877</v>
       </c>
       <c r="E69" t="n">
-        <v>3101.316478310922</v>
+        <v>2.349737373737374</v>
       </c>
       <c r="F69" t="n">
-        <v>1.342707070707071</v>
+        <v>4762.163899082648</v>
       </c>
       <c r="G69" t="n">
-        <v>187.0334189848791</v>
+        <v>635.456815394556</v>
       </c>
       <c r="H69" t="n">
-        <v>7132.979313795059</v>
-      </c>
-      <c r="I69" t="n">
-        <v>1966.362187970026</v>
-      </c>
-      <c r="J69" t="n">
-        <v>3362.819805437165</v>
+        <v>1179.225392441861</v>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="n">
-        <v>1.607616161616161</v>
+        <v>2.459333333333333</v>
       </c>
       <c r="B70" t="n">
-        <v>175.8943294123278</v>
+        <v>3659.943776343697</v>
       </c>
       <c r="C70" t="n">
-        <v>6174.948303638306</v>
+        <v>725.0718484246207</v>
       </c>
       <c r="D70" t="n">
-        <v>1588.480403548616</v>
+        <v>1068.585727206333</v>
       </c>
       <c r="E70" t="n">
-        <v>3042.679447576782</v>
+        <v>2.384808080808081</v>
       </c>
       <c r="F70" t="n">
-        <v>1.362747474747475</v>
+        <v>4587.733722088663</v>
       </c>
       <c r="G70" t="n">
-        <v>181.5416504544218</v>
+        <v>596.5974357988787</v>
       </c>
       <c r="H70" t="n">
-        <v>7063.483850808254</v>
-      </c>
-      <c r="I70" t="n">
-        <v>1942.16760506918</v>
-      </c>
-      <c r="J70" t="n">
-        <v>3308.782437908452</v>
+        <v>1111.215427603038</v>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="n">
-        <v>1.631257575757576</v>
+        <v>2.4955</v>
       </c>
       <c r="B71" t="n">
-        <v>171.6432413324024</v>
+        <v>3487.998113139909</v>
       </c>
       <c r="C71" t="n">
-        <v>6124.966154379263</v>
+        <v>685.663561028466</v>
       </c>
       <c r="D71" t="n">
-        <v>1564.889572852203</v>
+        <v>1005.939157583713</v>
       </c>
       <c r="E71" t="n">
-        <v>2987.504284020823</v>
+        <v>2.419878787878788</v>
       </c>
       <c r="F71" t="n">
-        <v>1.382787878787879</v>
+        <v>4416.457017880113</v>
       </c>
       <c r="G71" t="n">
-        <v>179.59719538277</v>
+        <v>559.1322621460743</v>
       </c>
       <c r="H71" t="n">
-        <v>6993.550132466789</v>
-      </c>
-      <c r="I71" t="n">
-        <v>1917.97526762869</v>
-      </c>
-      <c r="J71" t="n">
-        <v>3254.578471478595</v>
+        <v>1045.766595377441</v>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="n">
-        <v>1.65489898989899</v>
+        <v>2.531666666666667</v>
       </c>
       <c r="B72" t="n">
-        <v>167.4439188258293</v>
+        <v>3322.923812363466</v>
       </c>
       <c r="C72" t="n">
-        <v>6072.107132127534</v>
+        <v>648.2465478792732</v>
       </c>
       <c r="D72" t="n">
-        <v>1541.376732164256</v>
+        <v>945.4018650223151</v>
       </c>
       <c r="E72" t="n">
-        <v>2939.923810755179</v>
+        <v>2.454949494949495</v>
       </c>
       <c r="F72" t="n">
-        <v>1.402828282828283</v>
+        <v>4248.304608904517</v>
       </c>
       <c r="G72" t="n">
-        <v>179.4204905881632</v>
+        <v>523.1622534505894</v>
       </c>
       <c r="H72" t="n">
-        <v>6923.377747893051</v>
-      </c>
-      <c r="I72" t="n">
-        <v>1893.791266397177</v>
-      </c>
-      <c r="J72" t="n">
-        <v>3200.36976417727</v>
+        <v>982.9374800878459</v>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="n">
-        <v>1.678540404040404</v>
+        <v>2.567833333333333</v>
       </c>
       <c r="B73" t="n">
-        <v>163.2787075525872</v>
+        <v>3164.569824413354</v>
       </c>
       <c r="C73" t="n">
-        <v>6017.186923755936</v>
+        <v>612.2199714056615</v>
       </c>
       <c r="D73" t="n">
-        <v>1517.944801509226</v>
+        <v>887.1485456024425</v>
       </c>
       <c r="E73" t="n">
-        <v>2903.601276908223</v>
+        <v>2.490020202020202</v>
       </c>
       <c r="F73" t="n">
-        <v>1.422868686868687</v>
+        <v>4083.247317609406</v>
       </c>
       <c r="G73" t="n">
-        <v>173.4639738744669</v>
+        <v>488.7883687268725</v>
       </c>
       <c r="H73" t="n">
-        <v>6853.174596677498</v>
-      </c>
-      <c r="I73" t="n">
-        <v>1869.621692123261</v>
-      </c>
-      <c r="J73" t="n">
-        <v>3146.230559902943</v>
+        <v>922.8062104871773</v>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="n">
-        <v>1.702181818181818</v>
+        <v>2.604</v>
       </c>
       <c r="B74" t="n">
-        <v>159.1416956318567</v>
+        <v>3012.785099688549</v>
       </c>
       <c r="C74" t="n">
-        <v>5961.021216137283</v>
+        <v>577.2867386610528</v>
       </c>
       <c r="D74" t="n">
-        <v>1494.597252106548</v>
+        <v>831.3538954043959</v>
       </c>
       <c r="E74" t="n">
-        <v>2876.596541935546</v>
+        <v>2.525090909090909</v>
       </c>
       <c r="F74" t="n">
-        <v>1.442909090909091</v>
+        <v>3921.255966442302</v>
       </c>
       <c r="G74" t="n">
-        <v>163.9632748878342</v>
+        <v>456.1115669893705</v>
       </c>
       <c r="H74" t="n">
-        <v>6783.148578410582</v>
-      </c>
-      <c r="I74" t="n">
-        <v>1845.462131881072</v>
-      </c>
-      <c r="J74" t="n">
-        <v>3092.234726383886</v>
+        <v>865.4509153283584</v>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="n">
-        <v>1.725823232323232</v>
+        <v>2.640166666666667</v>
       </c>
       <c r="B75" t="n">
-        <v>155.061839788853</v>
+        <v>2867.418588588037</v>
       </c>
       <c r="C75" t="n">
-        <v>5904.425696144388</v>
+        <v>543.5237801323401</v>
       </c>
       <c r="D75" t="n">
-        <v>1471.337555175656</v>
+        <v>778.1926105084776</v>
       </c>
       <c r="E75" t="n">
-        <v>2853.834777251828</v>
+        <v>2.560161616161616</v>
       </c>
       <c r="F75" t="n">
-        <v>1.462949494949495</v>
+        <v>3762.301377850727</v>
       </c>
       <c r="G75" t="n">
-        <v>154.3276596628614</v>
+        <v>425.2328072525306</v>
       </c>
       <c r="H75" t="n">
-        <v>6714.834665420883</v>
-      </c>
-      <c r="I75" t="n">
-        <v>1821.299999907437</v>
-      </c>
-      <c r="J75" t="n">
-        <v>3038.353022776182</v>
+        <v>810.9497233643135</v>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="n">
-        <v>1.749464646464646</v>
+        <v>2.676333333333333</v>
       </c>
       <c r="B76" t="n">
-        <v>151.0004188263789</v>
+        <v>2728.319241510796</v>
       </c>
       <c r="C76" t="n">
-        <v>5848.216050650068</v>
+        <v>511.0080263064145</v>
       </c>
       <c r="D76" t="n">
-        <v>1448.166390863527</v>
+        <v>727.8393869949882</v>
       </c>
       <c r="E76" t="n">
-        <v>2830.220632282786</v>
+        <v>2.595232323232323</v>
       </c>
       <c r="F76" t="n">
-        <v>1.482989898989899</v>
+        <v>3606.766377910363</v>
       </c>
       <c r="G76" t="n">
-        <v>147.0691045145634</v>
+        <v>396.2530485308003</v>
       </c>
       <c r="H76" t="n">
-        <v>6666.246712244022</v>
-      </c>
-      <c r="I76" t="n">
-        <v>1797.140970264764</v>
-      </c>
-      <c r="J76" t="n">
-        <v>2984.515704759706</v>
+        <v>759.3807633479661</v>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="n">
-        <v>1.77310606060606</v>
+        <v>2.7125</v>
       </c>
       <c r="B77" t="n">
-        <v>147.0561538450871</v>
+        <v>2595.336008855812</v>
       </c>
       <c r="C77" t="n">
-        <v>5793.207966527138</v>
+        <v>479.8164076701687</v>
       </c>
       <c r="D77" t="n">
-        <v>1425.073629442485</v>
+        <v>680.4689209442301</v>
       </c>
       <c r="E77" t="n">
-        <v>2800.658756454138</v>
+        <v>2.63030303030303</v>
       </c>
       <c r="F77" t="n">
-        <v>1.503030303030303</v>
+        <v>3456.108377853689</v>
       </c>
       <c r="G77" t="n">
-        <v>141.0106749438438</v>
+        <v>369.2732498386269</v>
       </c>
       <c r="H77" t="n">
-        <v>6633.456817416806</v>
-      </c>
-      <c r="I77" t="n">
-        <v>1772.991076993028</v>
-      </c>
-      <c r="J77" t="n">
-        <v>2930.705628023003</v>
+        <v>710.8221640322405</v>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="n">
-        <v>1.796747474747475</v>
+        <v>2.748666666666667</v>
       </c>
       <c r="B78" t="n">
-        <v>143.2624670525134</v>
+        <v>2468.317841022063</v>
       </c>
       <c r="C78" t="n">
-        <v>5740.217130648411</v>
+        <v>450.0258547104937</v>
       </c>
       <c r="D78" t="n">
-        <v>1402.05931290069</v>
+        <v>636.2559084365041</v>
       </c>
       <c r="E78" t="n">
-        <v>2762.617971489989</v>
+        <v>2.665373737373737</v>
       </c>
       <c r="F78" t="n">
-        <v>1.523070707070707</v>
+        <v>3310.403785971222</v>
       </c>
       <c r="G78" t="n">
-        <v>136.3261592510584</v>
+        <v>344.3943701904579</v>
       </c>
       <c r="H78" t="n">
-        <v>6604.053138713153</v>
-      </c>
-      <c r="I78" t="n">
-        <v>1748.859095201905</v>
-      </c>
-      <c r="J78" t="n">
-        <v>2876.905648254616</v>
+        <v>665.3520541700606</v>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="n">
-        <v>1.820388888888889</v>
+        <v>2.784833333333333</v>
       </c>
       <c r="B79" t="n">
-        <v>139.2031767683214</v>
+        <v>2347.113688408533</v>
       </c>
       <c r="C79" t="n">
-        <v>5690.059229886702</v>
+        <v>421.7132979142822</v>
       </c>
       <c r="D79" t="n">
-        <v>1379.125019168934</v>
+        <v>595.3750455521126</v>
       </c>
       <c r="E79" t="n">
-        <v>2723.554327983008</v>
+        <v>2.700444444444444</v>
       </c>
       <c r="F79" t="n">
-        <v>1.543111111111111</v>
+        <v>3169.590894981511</v>
       </c>
       <c r="G79" t="n">
-        <v>135.228489993346</v>
+        <v>321.7095009775095</v>
       </c>
       <c r="H79" t="n">
-        <v>6565.623833906981</v>
-      </c>
-      <c r="I79" t="n">
-        <v>1724.82516922681</v>
-      </c>
-      <c r="J79" t="n">
-        <v>2823.213435403144</v>
+        <v>623.0485625143501</v>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="n">
-        <v>1.844030303030303</v>
+        <v>2.821</v>
       </c>
       <c r="B80" t="n">
-        <v>132.9056848459302</v>
+        <v>2231.572501414201</v>
       </c>
       <c r="C80" t="n">
-        <v>5643.331543521223</v>
+        <v>394.9556677684254</v>
       </c>
       <c r="D80" t="n">
-        <v>1356.27232617801</v>
+        <v>557.1512055642202</v>
       </c>
       <c r="E80" t="n">
-        <v>2684.286139239245</v>
+        <v>2.735515151515151</v>
       </c>
       <c r="F80" t="n">
-        <v>1.563151515151515</v>
+        <v>3033.607997603101</v>
       </c>
       <c r="G80" t="n">
-        <v>133.5794995031978</v>
+        <v>300.3512498880247</v>
       </c>
       <c r="H80" t="n">
-        <v>6505.757060772209</v>
-      </c>
-      <c r="I80" t="n">
-        <v>1700.886256963114</v>
-      </c>
-      <c r="J80" t="n">
-        <v>2770.378373817116</v>
+        <v>583.9898178180331</v>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="n">
-        <v>1.867671717171717</v>
+        <v>2.857166666666667</v>
       </c>
       <c r="B81" t="n">
-        <v>126.7453008777462</v>
+        <v>2121.543230438052</v>
       </c>
       <c r="C81" t="n">
-        <v>5599.36608988129</v>
+        <v>369.829894759816</v>
       </c>
       <c r="D81" t="n">
-        <v>1333.502519620316</v>
+        <v>520.2660144607003</v>
       </c>
       <c r="E81" t="n">
-        <v>2644.646690937721</v>
+        <v>2.770585858585858</v>
       </c>
       <c r="F81" t="n">
-        <v>1.583191919191919</v>
+        <v>2902.393386554538</v>
       </c>
       <c r="G81" t="n">
-        <v>127.3855418127435</v>
+        <v>279.7218480788413</v>
       </c>
       <c r="H81" t="n">
-        <v>6419.098327622699</v>
-      </c>
-      <c r="I81" t="n">
-        <v>1676.99106224352</v>
-      </c>
-      <c r="J81" t="n">
-        <v>2718.1410771657</v>
+        <v>547.59365780548</v>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="n">
-        <v>1.891313131313131</v>
+        <v>2.893333333333334</v>
       </c>
       <c r="B82" t="n">
-        <v>124.7746695897225</v>
+        <v>2016.874825879065</v>
       </c>
       <c r="C82" t="n">
-        <v>5557.387131177737</v>
+        <v>346.4129093753451</v>
       </c>
       <c r="D82" t="n">
-        <v>1310.812769133657</v>
+        <v>484.7785140882219</v>
       </c>
       <c r="E82" t="n">
-        <v>2604.469268757459</v>
+        <v>2.805656565656566</v>
       </c>
       <c r="F82" t="n">
-        <v>1.603232323232323</v>
+        <v>2775.885354554369</v>
       </c>
       <c r="G82" t="n">
-        <v>119.4520300407993</v>
+        <v>259.8812560796393</v>
       </c>
       <c r="H82" t="n">
-        <v>6315.424948789763</v>
-      </c>
-      <c r="I82" t="n">
-        <v>1653.088288900734</v>
-      </c>
-      <c r="J82" t="n">
-        <v>2666.01441878764</v>
+        <v>512.4491063170505</v>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="n">
-        <v>1.914954545454545</v>
+        <v>2.9295</v>
       </c>
       <c r="B83" t="n">
-        <v>125.7587226029515</v>
+        <v>1917.416238136224</v>
       </c>
       <c r="C83" t="n">
-        <v>5516.656254677833</v>
+        <v>324.7816421019052</v>
       </c>
       <c r="D83" t="n">
-        <v>1288.202070488185</v>
+        <v>450.7710383253945</v>
       </c>
       <c r="E83" t="n">
-        <v>2563.587158377482</v>
+        <v>2.840727272727273</v>
       </c>
       <c r="F83" t="n">
-        <v>1.623272727272727</v>
+        <v>2654.022194321143</v>
       </c>
       <c r="G83" t="n">
-        <v>112.4309566628969</v>
+        <v>240.8894344200993</v>
       </c>
       <c r="H83" t="n">
-        <v>6201.464048743891</v>
-      </c>
-      <c r="I83" t="n">
-        <v>1629.105939262636</v>
-      </c>
-      <c r="J83" t="n">
-        <v>2613.511272021677</v>
+        <v>478.590502061554</v>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="n">
-        <v>1.938595959595959</v>
+        <v>2.965666666666666</v>
       </c>
       <c r="B84" t="n">
-        <v>123.4088135543355</v>
+        <v>1823.016417608509</v>
       </c>
       <c r="C84" t="n">
-        <v>5476.435047648852</v>
+        <v>304.7978851880078</v>
       </c>
       <c r="D84" t="n">
-        <v>1265.670577475041</v>
+        <v>418.3259210508263</v>
       </c>
       <c r="E84" t="n">
-        <v>2522.049041377102</v>
+        <v>2.87579797979798</v>
       </c>
       <c r="F84" t="n">
-        <v>1.643313131313131</v>
+        <v>2536.742198573404</v>
       </c>
       <c r="G84" t="n">
-        <v>107.5567778640637</v>
+        <v>222.8063436299013</v>
       </c>
       <c r="H84" t="n">
-        <v>6083.862016620363</v>
-      </c>
-      <c r="I84" t="n">
-        <v>1604.95386994943</v>
-      </c>
-      <c r="J84" t="n">
-        <v>2554.060134599355</v>
+        <v>446.1096852478375</v>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="n">
-        <v>1.962237373737374</v>
+        <v>3.001833333333333</v>
       </c>
       <c r="B85" t="n">
-        <v>120.7030110406979</v>
+        <v>1733.524314694901</v>
       </c>
       <c r="C85" t="n">
-        <v>5435.985097358061</v>
+        <v>285.544758036957</v>
       </c>
       <c r="D85" t="n">
-        <v>1243.218443885365</v>
+        <v>387.5254961431252</v>
       </c>
       <c r="E85" t="n">
-        <v>2480.408960976864</v>
+        <v>2.910868686868687</v>
       </c>
       <c r="F85" t="n">
-        <v>1.663353535353535</v>
+        <v>2423.983660029699</v>
       </c>
       <c r="G85" t="n">
-        <v>103.1529306018477</v>
+        <v>205.6919442387253</v>
       </c>
       <c r="H85" t="n">
-        <v>5969.26524155446</v>
-      </c>
-      <c r="I85" t="n">
-        <v>1580.708116049139</v>
-      </c>
-      <c r="J85" t="n">
-        <v>2479.964331166571</v>
+        <v>415.0984960847491</v>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="n">
-        <v>1.985878787878788</v>
+        <v>3.038</v>
       </c>
       <c r="B86" t="n">
-        <v>117.9860294610077</v>
+        <v>1648.788879794384</v>
       </c>
       <c r="C86" t="n">
-        <v>5394.567991072731</v>
+        <v>266.9493393622676</v>
       </c>
       <c r="D86" t="n">
-        <v>1220.845833541436</v>
+        <v>358.4520974809007</v>
       </c>
       <c r="E86" t="n">
-        <v>2438.74466695655</v>
+        <v>2.945939393939394</v>
       </c>
       <c r="F86" t="n">
-        <v>1.683393939393939</v>
+        <v>2315.684871408574</v>
       </c>
       <c r="G86" t="n">
-        <v>99.24783664238717</v>
+        <v>189.6061967762515</v>
       </c>
       <c r="H86" t="n">
-        <v>5864.32011268146</v>
-      </c>
-      <c r="I86" t="n">
-        <v>1556.461844299489</v>
-      </c>
-      <c r="J86" t="n">
-        <v>2401.122984393553</v>
+        <v>385.6487747811362</v>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="n">
-        <v>2.009520202020202</v>
+        <v>3.074166666666667</v>
       </c>
       <c r="B87" t="n">
-        <v>115.2578551630757</v>
+        <v>1568.659063305937</v>
       </c>
       <c r="C87" t="n">
-        <v>5351.445316060134</v>
+        <v>249.0588125097754</v>
       </c>
       <c r="D87" t="n">
-        <v>1198.554515618428</v>
+        <v>331.1880589427605</v>
       </c>
       <c r="E87" t="n">
-        <v>2397.098179205187</v>
+        <v>2.981010101010101</v>
       </c>
       <c r="F87" t="n">
-        <v>1.703434343434343</v>
+        <v>2211.784125428577</v>
       </c>
       <c r="G87" t="n">
-        <v>95.76135542556558</v>
+        <v>174.60906177216</v>
       </c>
       <c r="H87" t="n">
-        <v>5771.326699659937</v>
-      </c>
-      <c r="I87" t="n">
-        <v>1532.308221438203</v>
-      </c>
-      <c r="J87" t="n">
-        <v>2327.950874274161</v>
+        <v>357.8523615458467</v>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="n">
-        <v>2.033161616161616</v>
+        <v>3.110333333333333</v>
       </c>
       <c r="B88" t="n">
-        <v>112.5301793947455</v>
+        <v>1492.161869079012</v>
       </c>
       <c r="C88" t="n">
-        <v>5305.878659587539</v>
+        <v>231.9203608253171</v>
       </c>
       <c r="D88" t="n">
-        <v>1176.345081845827</v>
+        <v>305.8157144073139</v>
       </c>
       <c r="E88" t="n">
-        <v>2355.5115176118</v>
+        <v>3.016080808080808</v>
       </c>
       <c r="F88" t="n">
-        <v>1.723474747474747</v>
+        <v>2112.219714808253</v>
       </c>
       <c r="G88" t="n">
-        <v>92.96731415015131</v>
+        <v>160.760499756131</v>
       </c>
       <c r="H88" t="n">
-        <v>5681.135719777762</v>
-      </c>
-      <c r="I88" t="n">
-        <v>1513.048933889144</v>
-      </c>
-      <c r="J88" t="n">
-        <v>2270.942415320824</v>
+        <v>331.8010965877283</v>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="n">
-        <v>2.05680303030303</v>
+        <v>3.1465</v>
       </c>
       <c r="B89" t="n">
-        <v>109.8692816301612</v>
+        <v>1417.024225023974</v>
       </c>
       <c r="C89" t="n">
-        <v>5257.328135559771</v>
+        <v>215.5811676547285</v>
       </c>
       <c r="D89" t="n">
-        <v>1154.216628718233</v>
+        <v>282.4173977531688</v>
       </c>
       <c r="E89" t="n">
-        <v>2314.026702065416</v>
+        <v>3.051151515151515</v>
       </c>
       <c r="F89" t="n">
-        <v>1.743515151515151</v>
+        <v>2016.92993226615</v>
       </c>
       <c r="G89" t="n">
-        <v>91.95368159817276</v>
+        <v>148.1204712578445</v>
       </c>
       <c r="H89" t="n">
-        <v>5593.400209996285</v>
-      </c>
-      <c r="I89" t="n">
-        <v>1501.534116141515</v>
-      </c>
-      <c r="J89" t="n">
-        <v>2239.070313863855</v>
+        <v>307.5868201156285</v>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="n">
-        <v>2.080444444444444</v>
+        <v>3.182666666666667</v>
       </c>
       <c r="B90" t="n">
-        <v>107.5828956053099</v>
+        <v>1343.25870548456</v>
       </c>
       <c r="C90" t="n">
-        <v>5206.750824677188</v>
+        <v>200.0884163438462</v>
       </c>
       <c r="D90" t="n">
-        <v>1132.168252730239</v>
+        <v>261.0754428589343</v>
       </c>
       <c r="E90" t="n">
-        <v>2272.635831782247</v>
+        <v>3.086222222222222</v>
       </c>
       <c r="F90" t="n">
-        <v>1.763555555555556</v>
+        <v>1925.853070520814</v>
       </c>
       <c r="G90" t="n">
-        <v>91.25093883275756</v>
+        <v>136.7479705288094</v>
       </c>
       <c r="H90" t="n">
-        <v>5508.511004271697</v>
-      </c>
-      <c r="I90" t="n">
-        <v>1492.078812050939</v>
-      </c>
-      <c r="J90" t="n">
-        <v>2221.493857884943</v>
+        <v>285.3013723383953</v>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="n">
-        <v>2.104085858585858</v>
+        <v>3.218833333333333</v>
       </c>
       <c r="B91" t="n">
-        <v>105.5187630948688</v>
+        <v>1271.013467085435</v>
       </c>
       <c r="C91" t="n">
-        <v>5154.422059566065</v>
+        <v>185.4892902385061</v>
       </c>
       <c r="D91" t="n">
-        <v>1110.199050376444</v>
+        <v>241.6060996807454</v>
       </c>
       <c r="E91" t="n">
-        <v>2231.258846526405</v>
+        <v>3.121292929292929</v>
       </c>
       <c r="F91" t="n">
-        <v>1.783595959595959</v>
+        <v>1838.92742229079</v>
       </c>
       <c r="G91" t="n">
-        <v>88.50100491874512</v>
+        <v>126.2634800779399</v>
       </c>
       <c r="H91" t="n">
-        <v>5426.858936560189</v>
-      </c>
-      <c r="I91" t="n">
-        <v>1478.958331387628</v>
-      </c>
-      <c r="J91" t="n">
-        <v>2201.469051544785</v>
+        <v>265.0365934648764</v>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="n">
-        <v>2.127727272727272</v>
+        <v>3.255</v>
       </c>
       <c r="B92" t="n">
-        <v>103.6595239323673</v>
+        <v>1200.436666451263</v>
       </c>
       <c r="C92" t="n">
-        <v>5100.374699986033</v>
+        <v>171.8309726845448</v>
       </c>
       <c r="D92" t="n">
-        <v>1088.311454001634</v>
+        <v>223.3540071228641</v>
       </c>
       <c r="E92" t="n">
-        <v>2189.898724841783</v>
+        <v>3.156363636363636</v>
       </c>
       <c r="F92" t="n">
-        <v>1.803636363636363</v>
+        <v>1756.091280294627</v>
       </c>
       <c r="G92" t="n">
-        <v>84.46588168262622</v>
+        <v>116.3583448218785</v>
       </c>
       <c r="H92" t="n">
-        <v>5349.696267969671</v>
-      </c>
-      <c r="I92" t="n">
-        <v>1456.661392795159</v>
-      </c>
-      <c r="J92" t="n">
-        <v>2163.551107773026</v>
+        <v>246.5479733570073</v>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="n">
-        <v>2.151368686868687</v>
+        <v>3.291166666666667</v>
       </c>
       <c r="B93" t="n">
-        <v>102.1978053600221</v>
+        <v>1131.676460206708</v>
       </c>
       <c r="C93" t="n">
-        <v>5044.641605696715</v>
+        <v>159.1606470277982</v>
       </c>
       <c r="D93" t="n">
-        <v>1066.510145042375</v>
+        <v>206.3522730598219</v>
       </c>
       <c r="E93" t="n">
-        <v>2148.561275737456</v>
+        <v>3.191434343434344</v>
       </c>
       <c r="F93" t="n">
-        <v>1.823676767676768</v>
+        <v>1677.28293725087</v>
       </c>
       <c r="G93" t="n">
-        <v>81.61333780692581</v>
+        <v>107.085096572599</v>
       </c>
       <c r="H93" t="n">
-        <v>5289.738334037935</v>
-      </c>
-      <c r="I93" t="n">
-        <v>1425.694856868234</v>
-      </c>
-      <c r="J93" t="n">
-        <v>2118.560289933414</v>
+        <v>229.0190572055144</v>
       </c>
     </row>
     <row r="94">
       <c r="A94" t="n">
-        <v>2.175010101010101</v>
+        <v>3.327333333333333</v>
       </c>
       <c r="B94" t="n">
-        <v>100.9768197063154</v>
+        <v>1064.881004976436</v>
       </c>
       <c r="C94" t="n">
-        <v>4987.255636457739</v>
+        <v>147.5254966141028</v>
       </c>
       <c r="D94" t="n">
-        <v>1044.79341113157</v>
+        <v>190.6764870340711</v>
       </c>
       <c r="E94" t="n">
-        <v>2107.252308222501</v>
+        <v>3.226505050505051</v>
       </c>
       <c r="F94" t="n">
-        <v>1.843717171717172</v>
+        <v>1602.068847868829</v>
       </c>
       <c r="G94" t="n">
-        <v>81.31832488358774</v>
+        <v>98.49626714207542</v>
       </c>
       <c r="H94" t="n">
-        <v>5243.086266596751</v>
-      </c>
-      <c r="I94" t="n">
-        <v>1389.88768097559</v>
-      </c>
-      <c r="J94" t="n">
-        <v>2073.266430230488</v>
+        <v>212.4769157373271</v>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="n">
-        <v>2.198651515151515</v>
+        <v>3.3635</v>
       </c>
       <c r="B95" t="n">
-        <v>100.5821196632509</v>
+        <v>1000.198457385109</v>
       </c>
       <c r="C95" t="n">
-        <v>4928.249652028733</v>
+        <v>136.9727047892946</v>
       </c>
       <c r="D95" t="n">
-        <v>1023.159404262739</v>
+        <v>176.4022385880634</v>
       </c>
       <c r="E95" t="n">
-        <v>2065.977631305995</v>
+        <v>3.261575757575758</v>
       </c>
       <c r="F95" t="n">
-        <v>1.863757575757576</v>
+        <v>1528.351032024578</v>
       </c>
       <c r="G95" t="n">
-        <v>81.63613274220711</v>
+        <v>90.64438834228157</v>
       </c>
       <c r="H95" t="n">
-        <v>5199.281169113385</v>
-      </c>
-      <c r="I95" t="n">
-        <v>1352.443838366184</v>
-      </c>
-      <c r="J95" t="n">
-        <v>2027.370303907213</v>
+        <v>196.9976849264819</v>
       </c>
     </row>
     <row r="96">
       <c r="A96" t="n">
-        <v>2.222292929292929</v>
+        <v>3.399666666666667</v>
       </c>
       <c r="B96" t="n">
-        <v>100.6287917877708</v>
+        <v>937.7769740573951</v>
       </c>
       <c r="C96" t="n">
-        <v>4867.656512169323</v>
+        <v>127.2219696677122</v>
       </c>
       <c r="D96" t="n">
-        <v>1001.606276429404</v>
+        <v>163.605117264251</v>
       </c>
       <c r="E96" t="n">
-        <v>2024.810187310862</v>
+        <v>3.296646464646465</v>
       </c>
       <c r="F96" t="n">
-        <v>1.88379797979798</v>
+        <v>1455.9334407411</v>
       </c>
       <c r="G96" t="n">
-        <v>81.77291315084166</v>
+        <v>83.58199198519124</v>
       </c>
       <c r="H96" t="n">
-        <v>5147.864145055103</v>
-      </c>
-      <c r="I96" t="n">
-        <v>1316.567302288972</v>
-      </c>
-      <c r="J96" t="n">
-        <v>1980.572686206555</v>
+        <v>182.6575007470157</v>
       </c>
     </row>
     <row r="97">
       <c r="A97" t="n">
-        <v>2.245934343434343</v>
+        <v>3.435833333333334</v>
       </c>
       <c r="B97" t="n">
-        <v>99.60635825203003</v>
+        <v>877.7647116179558</v>
       </c>
       <c r="C97" t="n">
-        <v>4805.509076639134</v>
+        <v>117.9886587864959</v>
       </c>
       <c r="D97" t="n">
-        <v>980.1348876448973</v>
+        <v>152.3607126050856</v>
       </c>
       <c r="E97" t="n">
-        <v>1983.820289334123</v>
+        <v>3.331717171717172</v>
       </c>
       <c r="F97" t="n">
-        <v>1.903838383838384</v>
+        <v>1384.962279922315</v>
       </c>
       <c r="G97" t="n">
-        <v>81.38701923334615</v>
+        <v>77.36160988277831</v>
       </c>
       <c r="H97" t="n">
-        <v>5078.376297889171</v>
-      </c>
-      <c r="I97" t="n">
-        <v>1285.46204599291</v>
-      </c>
-      <c r="J97" t="n">
-        <v>1932.781731679139</v>
+        <v>169.5324991729652</v>
       </c>
     </row>
     <row r="98">
       <c r="A98" t="n">
-        <v>2.269575757575757</v>
+        <v>3.472</v>
       </c>
       <c r="B98" t="n">
-        <v>96.09222296757831</v>
+        <v>820.3098266914573</v>
       </c>
       <c r="C98" t="n">
-        <v>4741.840205197797</v>
+        <v>109.3134596256855</v>
       </c>
       <c r="D98" t="n">
-        <v>958.7545995817759</v>
+        <v>142.7446141530193</v>
       </c>
       <c r="E98" t="n">
-        <v>1942.959738421826</v>
+        <v>3.366787878787879</v>
       </c>
       <c r="F98" t="n">
-        <v>1.923878787878788</v>
+        <v>1315.583755472143</v>
       </c>
       <c r="G98" t="n">
-        <v>81.37529908340919</v>
+        <v>72.03577384701661</v>
       </c>
       <c r="H98" t="n">
-        <v>4985.883543098143</v>
-      </c>
-      <c r="I98" t="n">
-        <v>1258.792880992493</v>
-      </c>
-      <c r="J98" t="n">
-        <v>1884.675509184181</v>
+        <v>157.6988161783673</v>
       </c>
     </row>
     <row r="99">
       <c r="A99" t="n">
-        <v>2.293217171717171</v>
+        <v>3.508166666666666</v>
       </c>
       <c r="B99" t="n">
-        <v>93.68030740869769</v>
+        <v>765.5604759025634</v>
       </c>
       <c r="C99" t="n">
-        <v>4676.158719938129</v>
+        <v>101.2370596653203</v>
       </c>
       <c r="D99" t="n">
-        <v>937.4640509462197</v>
+        <v>134.832411450504</v>
       </c>
       <c r="E99" t="n">
-        <v>1902.179428640526</v>
+        <v>3.401858585858586</v>
       </c>
       <c r="F99" t="n">
-        <v>1.943919191919192</v>
+        <v>1247.944073294502</v>
       </c>
       <c r="G99" t="n">
-        <v>97.87367089880728</v>
+        <v>67.65701568988001</v>
       </c>
       <c r="H99" t="n">
-        <v>4878.74136305672</v>
-      </c>
-      <c r="I99" t="n">
-        <v>1232.300538594641</v>
-      </c>
-      <c r="J99" t="n">
-        <v>1836.542031693473</v>
+        <v>147.2325877372589</v>
       </c>
     </row>
     <row r="100">
       <c r="A100" t="n">
-        <v>2.316858585858586</v>
+        <v>3.544333333333333</v>
       </c>
       <c r="B100" t="n">
-        <v>123.1387187623233</v>
+        <v>713.6648158759381</v>
       </c>
       <c r="C100" t="n">
-        <v>4606.898550112566</v>
+        <v>93.80014638543975</v>
       </c>
       <c r="D100" t="n">
-        <v>916.2605423408131</v>
+        <v>128.6996940399916</v>
       </c>
       <c r="E100" t="n">
-        <v>1861.430254056776</v>
+        <v>3.436929292929293</v>
       </c>
       <c r="F100" t="n">
-        <v>1.963959595959596</v>
+        <v>1182.189439293313</v>
       </c>
       <c r="G100" t="n">
-        <v>134.6078625517204</v>
+        <v>64.27786722334234</v>
       </c>
       <c r="H100" t="n">
-        <v>4763.394257343995</v>
-      </c>
-      <c r="I100" t="n">
-        <v>1206.235364203616</v>
-      </c>
-      <c r="J100" t="n">
-        <v>1788.615533981866</v>
+        <v>138.2099498236766</v>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="n">
-        <v>2.3405</v>
+        <v>3.5805</v>
       </c>
       <c r="B101" t="n">
-        <v>192.2432913872947</v>
+        <v>664.7710032362473</v>
       </c>
       <c r="C101" t="n">
-        <v>4534.765102558594</v>
+        <v>87.04340726608351</v>
       </c>
       <c r="D101" t="n">
-        <v>895.1413743681419</v>
+        <v>124.4220514639343</v>
       </c>
       <c r="E101" t="n">
-        <v>1820.663108737132</v>
+        <v>3.472</v>
       </c>
       <c r="F101" t="n">
-        <v>1.984</v>
+        <v>1118.466059372493</v>
       </c>
       <c r="G101" t="n">
-        <v>181.5961679117934</v>
+        <v>61.95086025937746</v>
       </c>
       <c r="H101" t="n">
-        <v>4646.20659420908</v>
-      </c>
-      <c r="I101" t="n">
-        <v>1180.92225332049</v>
-      </c>
-      <c r="J101" t="n">
-        <v>1741.130250824207</v>
+        <v>130.7070384116574</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
finished boltz graphs added y0 changed algorithm for spatial gauss
</commit_message>
<xml_diff>
--- a/results/aligned_results.xlsx
+++ b/results/aligned_results.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L101"/>
+  <dimension ref="A1:J101"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -444,3838 +444,3228 @@
       </c>
       <c r="F1" t="inlineStr">
         <is>
-          <t>Cu I 578.2 nm_Left</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
           <t>Radius_mm_Right</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>Cu I 510.5 nm_Right</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>Cu I 515.3 nm_Right</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>Cu I 521.8 nm_Right</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>Cu I 570.0 nm_Right</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
-        <is>
-          <t>Cu I 578.2 nm_Right</t>
-        </is>
-      </c>
     </row>
     <row r="2">
       <c r="A2" t="n">
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>17820.54901027648</v>
+        <v>16817.43179481263</v>
       </c>
       <c r="C2" t="n">
-        <v>5109.760848954002</v>
+        <v>4700.126000543607</v>
       </c>
       <c r="D2" t="n">
-        <v>8776.385652813544</v>
+        <v>7788.269791938231</v>
       </c>
       <c r="E2" t="n">
-        <v>1117.530994829743</v>
+        <v>1297.455786445589</v>
       </c>
       <c r="F2" t="n">
-        <v>14502.94246904115</v>
+        <v>0</v>
       </c>
       <c r="G2" t="n">
-        <v>0</v>
+        <v>14934.63409119967</v>
       </c>
       <c r="H2" t="n">
-        <v>16286.92680379652</v>
+        <v>4816.638829074795</v>
       </c>
       <c r="I2" t="n">
-        <v>5255.470675070236</v>
+        <v>7312.022891100726</v>
       </c>
       <c r="J2" t="n">
-        <v>8392.534975487006</v>
-      </c>
-      <c r="K2" t="n">
-        <v>1095.867492434052</v>
-      </c>
-      <c r="L2" t="n">
-        <v>5325.6698783317</v>
+        <v>914.5608187242181</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>0.004070707070707071</v>
+        <v>0.01002020202020202</v>
       </c>
       <c r="B3" t="n">
-        <v>17811.30280647099</v>
+        <v>16803.74109725637</v>
       </c>
       <c r="C3" t="n">
-        <v>5108.39931642651</v>
+        <v>4702.77348877269</v>
       </c>
       <c r="D3" t="n">
-        <v>8773.938398175993</v>
+        <v>7774.664563393309</v>
       </c>
       <c r="E3" t="n">
-        <v>1117.522764318373</v>
+        <v>1298.420603914437</v>
       </c>
       <c r="F3" t="n">
-        <v>14503.27307297875</v>
+        <v>0.0382020202020202</v>
       </c>
       <c r="G3" t="n">
-        <v>0.03647979797979798</v>
+        <v>14907.05726031822</v>
       </c>
       <c r="H3" t="n">
-        <v>16274.64790257487</v>
+        <v>4803.141731010205</v>
       </c>
       <c r="I3" t="n">
-        <v>5257.813823309396</v>
+        <v>7355.959844699451</v>
       </c>
       <c r="J3" t="n">
-        <v>8377.153209445225</v>
-      </c>
-      <c r="K3" t="n">
-        <v>1095.268448665632</v>
-      </c>
-      <c r="L3" t="n">
-        <v>5327.324624623878</v>
+        <v>914.3435252723276</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>0.008141414141414142</v>
+        <v>0.02004040404040404</v>
       </c>
       <c r="B4" t="n">
-        <v>17802.00816902019</v>
+        <v>16789.50365245563</v>
       </c>
       <c r="C4" t="n">
-        <v>5107.014422659197</v>
+        <v>4704.891287299928</v>
       </c>
       <c r="D4" t="n">
-        <v>8771.445317050804</v>
+        <v>7761.487976797548</v>
       </c>
       <c r="E4" t="n">
-        <v>1117.508603891849</v>
+        <v>1298.366729330592</v>
       </c>
       <c r="F4" t="n">
-        <v>14504.93829168964</v>
+        <v>0.0764040404040404</v>
       </c>
       <c r="G4" t="n">
-        <v>0.07295959595959596</v>
+        <v>14888.10440164334</v>
       </c>
       <c r="H4" t="n">
-        <v>16258.69650170391</v>
+        <v>4796.096089263902</v>
       </c>
       <c r="I4" t="n">
-        <v>5256.447365024693</v>
+        <v>7382.065225992771</v>
       </c>
       <c r="J4" t="n">
-        <v>8356.738047746154</v>
-      </c>
-      <c r="K4" t="n">
-        <v>1094.204103438469</v>
-      </c>
-      <c r="L4" t="n">
-        <v>5326.491035382999</v>
+        <v>913.6912091523119</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>0.01221212121212121</v>
+        <v>0.03006060606060606</v>
       </c>
       <c r="B5" t="n">
-        <v>17792.66488402526</v>
+        <v>16774.72358233709</v>
       </c>
       <c r="C5" t="n">
-        <v>5105.605769922049</v>
+        <v>4706.448671535674</v>
       </c>
       <c r="D5" t="n">
-        <v>8768.905669697087</v>
+        <v>7748.708654550377</v>
       </c>
       <c r="E5" t="n">
-        <v>1117.488491119721</v>
+        <v>1297.761981187127</v>
       </c>
       <c r="F5" t="n">
-        <v>14507.91394262522</v>
+        <v>0.1146060606060606</v>
       </c>
       <c r="G5" t="n">
-        <v>0.1094393939393939</v>
+        <v>14873.5724716829</v>
       </c>
       <c r="H5" t="n">
-        <v>16238.2794484827</v>
+        <v>4792.151649775627</v>
       </c>
       <c r="I5" t="n">
-        <v>5250.867936820703</v>
+        <v>7394.384448151884</v>
       </c>
       <c r="J5" t="n">
-        <v>8331.057834369121</v>
-      </c>
-      <c r="K5" t="n">
-        <v>1092.645963343587</v>
-      </c>
-      <c r="L5" t="n">
-        <v>5323.003947388992</v>
+        <v>912.6013860735918</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>0.01628282828282828</v>
+        <v>0.04008080808080808</v>
       </c>
       <c r="B6" t="n">
-        <v>17783.27273758741</v>
+        <v>16759.40500882749</v>
       </c>
       <c r="C6" t="n">
-        <v>5104.172960485049</v>
+        <v>4707.414916890281</v>
       </c>
       <c r="D6" t="n">
-        <v>8766.318716373942</v>
+        <v>7736.295219051228</v>
       </c>
       <c r="E6" t="n">
-        <v>1117.462403571537</v>
+        <v>1295.540719513275</v>
       </c>
       <c r="F6" t="n">
-        <v>14512.17584323696</v>
+        <v>0.1528080808080808</v>
       </c>
       <c r="G6" t="n">
-        <v>0.1459191919191919</v>
+        <v>14864.34737575397</v>
       </c>
       <c r="H6" t="n">
-        <v>16212.6035902103</v>
+        <v>4813.395376516478</v>
       </c>
       <c r="I6" t="n">
-        <v>5240.572175302001</v>
+        <v>7386.859629298766</v>
       </c>
       <c r="J6" t="n">
-        <v>8299.880913293448</v>
-      </c>
-      <c r="K6" t="n">
-        <v>1090.565534972014</v>
-      </c>
-      <c r="L6" t="n">
-        <v>5316.698197421779</v>
+        <v>911.0822964629467</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
-        <v>0.02035353535353536</v>
+        <v>0.0501010101010101</v>
       </c>
       <c r="B7" t="n">
-        <v>17773.83151580779</v>
+        <v>16743.55205385352</v>
       </c>
       <c r="C7" t="n">
-        <v>5102.715596618185</v>
+        <v>4707.759298774099</v>
       </c>
       <c r="D7" t="n">
-        <v>8763.683717340473</v>
+        <v>7724.216292699532</v>
       </c>
       <c r="E7" t="n">
-        <v>1117.430318816845</v>
+        <v>1291.485159066078</v>
       </c>
       <c r="F7" t="n">
-        <v>14517.69981097626</v>
+        <v>0.191010101010101</v>
       </c>
       <c r="G7" t="n">
-        <v>0.1823989898989899</v>
+        <v>14899.75056263511</v>
       </c>
       <c r="H7" t="n">
-        <v>16180.87577418579</v>
+        <v>4834.138536081819</v>
       </c>
       <c r="I7" t="n">
-        <v>5225.056717073165</v>
+        <v>7359.288366557838</v>
       </c>
       <c r="J7" t="n">
-        <v>8262.97562849846</v>
-      </c>
-      <c r="K7" t="n">
-        <v>1087.934324914772</v>
-      </c>
-      <c r="L7" t="n">
-        <v>5307.408622261288</v>
+        <v>909.1280222605419</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
-        <v>0.02442424242424242</v>
+        <v>0.06012121212121212</v>
       </c>
       <c r="B8" t="n">
-        <v>17764.34100478762</v>
+        <v>16727.1688393419</v>
       </c>
       <c r="C8" t="n">
-        <v>5101.233280591441</v>
+        <v>4707.451092597482</v>
       </c>
       <c r="D8" t="n">
-        <v>8760.999932855784</v>
+        <v>7712.44049789472</v>
       </c>
       <c r="E8" t="n">
-        <v>1117.392214425192</v>
+        <v>1288.517854373453</v>
       </c>
       <c r="F8" t="n">
-        <v>14524.46166329458</v>
+        <v>0.2292121212121212</v>
       </c>
       <c r="G8" t="n">
-        <v>0.2188787878787879</v>
+        <v>14939.87762240889</v>
       </c>
       <c r="H8" t="n">
-        <v>16142.30284770822</v>
+        <v>4806.189030260138</v>
       </c>
       <c r="I8" t="n">
-        <v>5203.818198738772</v>
+        <v>7294.507443567259</v>
       </c>
       <c r="J8" t="n">
-        <v>8220.110323963481</v>
-      </c>
-      <c r="K8" t="n">
-        <v>1084.723839762889</v>
-      </c>
-      <c r="L8" t="n">
-        <v>5294.970058687441</v>
+        <v>906.7550247543426</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
-        <v>0.0284949494949495</v>
+        <v>0.07014141414141414</v>
       </c>
       <c r="B9" t="n">
-        <v>17754.80099062806</v>
+        <v>16710.25948721933</v>
       </c>
       <c r="C9" t="n">
-        <v>5099.725614674802</v>
+        <v>4706.459573770781</v>
       </c>
       <c r="D9" t="n">
-        <v>8758.266623178975</v>
+        <v>7700.936457036223</v>
       </c>
       <c r="E9" t="n">
-        <v>1117.348067966128</v>
+        <v>1292.656571085762</v>
       </c>
       <c r="F9" t="n">
-        <v>14532.43721764333</v>
+        <v>0.2674141414141414</v>
       </c>
       <c r="G9" t="n">
-        <v>0.2553585858585858</v>
+        <v>14922.94209117914</v>
       </c>
       <c r="H9" t="n">
-        <v>16096.09165807667</v>
+        <v>4747.264760603561</v>
       </c>
       <c r="I9" t="n">
-        <v>5176.353256903398</v>
+        <v>7180.847911387366</v>
       </c>
       <c r="J9" t="n">
-        <v>8171.053343667842</v>
-      </c>
-      <c r="K9" t="n">
-        <v>1080.905586107389</v>
-      </c>
-      <c r="L9" t="n">
-        <v>5279.217343480166</v>
+        <v>903.9624998259138</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="n">
-        <v>0.03256565656565657</v>
+        <v>0.08016161616161616</v>
       </c>
       <c r="B10" t="n">
-        <v>17745.21125943031</v>
+        <v>16692.82811941253</v>
       </c>
       <c r="C10" t="n">
-        <v>5098.192201138254</v>
+        <v>4704.754017704348</v>
       </c>
       <c r="D10" t="n">
-        <v>8755.483048569156</v>
+        <v>7689.672792523472</v>
       </c>
       <c r="E10" t="n">
-        <v>1117.2978570092</v>
+        <v>1297.530413196513</v>
       </c>
       <c r="F10" t="n">
-        <v>14541.60229147396</v>
+        <v>0.3056161616161616</v>
       </c>
       <c r="G10" t="n">
-        <v>0.2918383838383838</v>
+        <v>14818.03807590308</v>
       </c>
       <c r="H10" t="n">
-        <v>16041.4490525902</v>
+        <v>4680.844006802598</v>
       </c>
       <c r="I10" t="n">
-        <v>5142.158528171621</v>
+        <v>7087.174576195095</v>
       </c>
       <c r="J10" t="n">
-        <v>8115.573031590864</v>
-      </c>
-      <c r="K10" t="n">
-        <v>1076.451070539298</v>
-      </c>
-      <c r="L10" t="n">
-        <v>5259.985313419389</v>
+        <v>900.7488164075386</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="n">
-        <v>0.03663636363636364</v>
+        <v>0.09018181818181817</v>
       </c>
       <c r="B11" t="n">
-        <v>17735.57159729555</v>
+        <v>16674.87885784821</v>
       </c>
       <c r="C11" t="n">
-        <v>5096.632642251782</v>
+        <v>4702.303699808535</v>
       </c>
       <c r="D11" t="n">
-        <v>8752.648469285423</v>
+        <v>7678.618126755897</v>
       </c>
       <c r="E11" t="n">
-        <v>1117.241559123955</v>
+        <v>1294.358916582011</v>
       </c>
       <c r="F11" t="n">
-        <v>14551.93270223789</v>
+        <v>0.3438181818181818</v>
       </c>
       <c r="G11" t="n">
-        <v>0.3283181818181818</v>
+        <v>14688.76778522958</v>
       </c>
       <c r="H11" t="n">
-        <v>15977.58187854787</v>
+        <v>4618.821135099992</v>
       </c>
       <c r="I11" t="n">
-        <v>5100.730649148015</v>
+        <v>7069.932071523569</v>
       </c>
       <c r="J11" t="n">
-        <v>8053.437731711871</v>
-      </c>
-      <c r="K11" t="n">
-        <v>1071.331799649641</v>
-      </c>
-      <c r="L11" t="n">
-        <v>5237.108805285034</v>
+        <v>897.1405877856085</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="n">
-        <v>0.04070707070707071</v>
+        <v>0.1002020202020202</v>
       </c>
       <c r="B12" t="n">
-        <v>17725.88179032497</v>
+        <v>16656.41582445308</v>
       </c>
       <c r="C12" t="n">
-        <v>5095.046540285372</v>
+        <v>4699.077895493695</v>
       </c>
       <c r="D12" t="n">
-        <v>8749.762145586885</v>
+        <v>7667.74108213293</v>
       </c>
       <c r="E12" t="n">
-        <v>1117.179151879943</v>
+        <v>1289.769819331447</v>
       </c>
       <c r="F12" t="n">
-        <v>14563.40426738657</v>
+        <v>0.382020202020202</v>
       </c>
       <c r="G12" t="n">
-        <v>0.3647979797979798</v>
+        <v>14550.79403034377</v>
       </c>
       <c r="H12" t="n">
-        <v>15903.69698324874</v>
+        <v>4562.432824858386</v>
       </c>
       <c r="I12" t="n">
-        <v>5051.566256437159</v>
+        <v>7078.061369340579</v>
       </c>
       <c r="J12" t="n">
-        <v>7984.415788010192</v>
-      </c>
-      <c r="K12" t="n">
-        <v>1065.519280029444</v>
-      </c>
-      <c r="L12" t="n">
-        <v>5210.422655857027</v>
+        <v>893.1166431117106</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="n">
-        <v>0.04477777777777778</v>
+        <v>0.1102222222222222</v>
       </c>
       <c r="B13" t="n">
-        <v>17716.14162461975</v>
+        <v>16637.44314115385</v>
       </c>
       <c r="C13" t="n">
-        <v>5093.433497509008</v>
+        <v>4695.045880170179</v>
       </c>
       <c r="D13" t="n">
-        <v>8746.823337732643</v>
+        <v>7657.010281054001</v>
       </c>
       <c r="E13" t="n">
-        <v>1117.110612846711</v>
+        <v>1290.205076358574</v>
       </c>
       <c r="F13" t="n">
-        <v>14575.99280437142</v>
+        <v>0.4202222222222222</v>
       </c>
       <c r="G13" t="n">
-        <v>0.4012777777777778</v>
+        <v>14415.04300225935</v>
       </c>
       <c r="H13" t="n">
-        <v>15819.0012139919</v>
+        <v>4507.217026969384</v>
       </c>
       <c r="I13" t="n">
-        <v>4994.642422779512</v>
+        <v>7029.41925772889</v>
       </c>
       <c r="J13" t="n">
-        <v>7908.275544465148</v>
-      </c>
-      <c r="K13" t="n">
-        <v>1058.985018269732</v>
-      </c>
-      <c r="L13" t="n">
-        <v>5179.761701915294</v>
+        <v>888.7220449154381</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="n">
-        <v>0.04884848484848485</v>
+        <v>0.1202424242424242</v>
       </c>
       <c r="B14" t="n">
-        <v>17706.35088628108</v>
+        <v>16617.96492987722</v>
       </c>
       <c r="C14" t="n">
-        <v>5091.793116192675</v>
+        <v>4690.176929248339</v>
       </c>
       <c r="D14" t="n">
-        <v>8743.831305981801</v>
+        <v>7646.394345918544</v>
       </c>
       <c r="E14" t="n">
-        <v>1117.035919593807</v>
+        <v>1299.173381733312</v>
       </c>
       <c r="F14" t="n">
-        <v>14589.7482905477</v>
+        <v>0.4584242424242424</v>
       </c>
       <c r="G14" t="n">
-        <v>0.4377575757575758</v>
+        <v>14288.62170382746</v>
       </c>
       <c r="H14" t="n">
-        <v>15722.70141807639</v>
+        <v>4455.167193609455</v>
       </c>
       <c r="I14" t="n">
-        <v>4934.459385654701</v>
+        <v>6955.404494635865</v>
       </c>
       <c r="J14" t="n">
-        <v>7825.430970691402</v>
-      </c>
-      <c r="K14" t="n">
-        <v>1051.765226675071</v>
-      </c>
-      <c r="L14" t="n">
-        <v>5144.960780239758</v>
+        <v>883.941976575087</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="n">
-        <v>0.05291919191919192</v>
+        <v>0.1302626262626262</v>
       </c>
       <c r="B15" t="n">
-        <v>17696.50936141016</v>
+        <v>16597.98531254991</v>
       </c>
       <c r="C15" t="n">
-        <v>5090.124998606361</v>
+        <v>4684.440318138528</v>
       </c>
       <c r="D15" t="n">
-        <v>8740.785310593465</v>
+        <v>7635.861899125986</v>
       </c>
       <c r="E15" t="n">
-        <v>1116.95504969078</v>
+        <v>1302.780161108366</v>
       </c>
       <c r="F15" t="n">
-        <v>14604.96925931396</v>
+        <v>0.4966262626262626</v>
       </c>
       <c r="G15" t="n">
-        <v>0.4742373737373737</v>
+        <v>14163.96531704633</v>
       </c>
       <c r="H15" t="n">
-        <v>15614.00444280129</v>
+        <v>4436.07377827292</v>
       </c>
       <c r="I15" t="n">
-        <v>4871.972731028045</v>
+        <v>6872.140301891762</v>
       </c>
       <c r="J15" t="n">
-        <v>7739.005693570923</v>
-      </c>
-      <c r="K15" t="n">
-        <v>1044.176291964923</v>
-      </c>
-      <c r="L15" t="n">
-        <v>5105.961695655736</v>
+        <v>878.7686965366103</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="n">
-        <v>0.05698989898989899</v>
+        <v>0.1402828282828283</v>
       </c>
       <c r="B16" t="n">
-        <v>17686.61683610815</v>
+        <v>16577.50841109862</v>
       </c>
       <c r="C16" t="n">
-        <v>5088.428747020049</v>
+        <v>4677.805322251097</v>
       </c>
       <c r="D16" t="n">
-        <v>8737.684611826733</v>
+        <v>7625.38156307576</v>
       </c>
       <c r="E16" t="n">
-        <v>1116.867980707177</v>
+        <v>1303.969582751594</v>
       </c>
       <c r="F16" t="n">
-        <v>14621.650666712</v>
+        <v>0.5348282828282829</v>
       </c>
       <c r="G16" t="n">
-        <v>0.5107171717171717</v>
+        <v>14040.21569515757</v>
       </c>
       <c r="H16" t="n">
-        <v>15492.11713546565</v>
+        <v>4419.384501903766</v>
       </c>
       <c r="I16" t="n">
-        <v>4806.844323145571</v>
+        <v>6781.578009629759</v>
       </c>
       <c r="J16" t="n">
-        <v>7648.996707569349</v>
-      </c>
-      <c r="K16" t="n">
-        <v>1036.233938462379</v>
-      </c>
-      <c r="L16" t="n">
-        <v>5064.872262140706</v>
+        <v>873.2795090175749</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="n">
-        <v>0.06106060606060607</v>
+        <v>0.1503030303030303</v>
       </c>
       <c r="B17" t="n">
-        <v>17676.67309647624</v>
+        <v>16556.53834745008</v>
       </c>
       <c r="C17" t="n">
-        <v>5086.703963703725</v>
+        <v>4670.241216996397</v>
       </c>
       <c r="D17" t="n">
-        <v>8734.528469940711</v>
+        <v>7614.921960167298</v>
       </c>
       <c r="E17" t="n">
-        <v>1116.774690212547</v>
+        <v>1304.096478613242</v>
       </c>
       <c r="F17" t="n">
-        <v>14639.74694939599</v>
+        <v>0.573030303030303</v>
       </c>
       <c r="G17" t="n">
-        <v>0.5471969696969697</v>
+        <v>13917.49580118245</v>
       </c>
       <c r="H17" t="n">
-        <v>15356.24634336856</v>
+        <v>4354.475948908315</v>
       </c>
       <c r="I17" t="n">
-        <v>4738.736026253306</v>
+        <v>6682.967608343727</v>
       </c>
       <c r="J17" t="n">
-        <v>7554.873543217453</v>
-      </c>
-      <c r="K17" t="n">
-        <v>1027.901848976842</v>
-      </c>
-      <c r="L17" t="n">
-        <v>5022.366862314063</v>
+        <v>867.4964243865827</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="n">
-        <v>0.06513131313131314</v>
+        <v>0.1603232323232323</v>
       </c>
       <c r="B18" t="n">
-        <v>17666.67792861564</v>
+        <v>16535.07924353098</v>
       </c>
       <c r="C18" t="n">
-        <v>5084.950250927374</v>
+        <v>4661.669361103153</v>
       </c>
       <c r="D18" t="n">
-        <v>8731.316145194509</v>
+        <v>7604.451712800027</v>
       </c>
       <c r="E18" t="n">
-        <v>1116.675155776438</v>
+        <v>1302.882532692356</v>
       </c>
       <c r="F18" t="n">
-        <v>14659.21254402009</v>
+        <v>0.6112323232323232</v>
       </c>
       <c r="G18" t="n">
-        <v>0.5836767676767677</v>
+        <v>13825.6989926301</v>
       </c>
       <c r="H18" t="n">
-        <v>15205.59891380906</v>
+        <v>4251.082066567666</v>
       </c>
       <c r="I18" t="n">
-        <v>4667.309704597269</v>
+        <v>6575.713590047321</v>
       </c>
       <c r="J18" t="n">
-        <v>7456.105731046008</v>
-      </c>
-      <c r="K18" t="n">
-        <v>1019.143706317722</v>
-      </c>
-      <c r="L18" t="n">
-        <v>4978.18021883593</v>
+        <v>861.3285253781304</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="n">
-        <v>0.06920202020202021</v>
+        <v>0.1703434343434343</v>
       </c>
       <c r="B19" t="n">
-        <v>17656.63111862751</v>
+        <v>16513.13522126805</v>
       </c>
       <c r="C19" t="n">
-        <v>5083.167210960982</v>
+        <v>4651.881075842248</v>
       </c>
       <c r="D19" t="n">
-        <v>8728.046897847218</v>
+        <v>7593.939443373382</v>
       </c>
       <c r="E19" t="n">
-        <v>1116.569354968397</v>
+        <v>1298.568343163733</v>
       </c>
       <c r="F19" t="n">
-        <v>14680.00188723847</v>
+        <v>0.6494343434343435</v>
       </c>
       <c r="G19" t="n">
-        <v>0.6201565656565656</v>
+        <v>13768.04347208872</v>
       </c>
       <c r="H19" t="n">
-        <v>15039.38169408623</v>
+        <v>4137.171860731351</v>
       </c>
       <c r="I19" t="n">
-        <v>4592.22722242349</v>
+        <v>6432.581841215183</v>
       </c>
       <c r="J19" t="n">
-        <v>7352.162801585791</v>
-      </c>
-      <c r="K19" t="n">
-        <v>1009.923193294423</v>
-      </c>
-      <c r="L19" t="n">
-        <v>4932.04705436643</v>
+        <v>854.9973854103924</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="n">
-        <v>0.07327272727272728</v>
+        <v>0.1803636363636363</v>
       </c>
       <c r="B20" t="n">
-        <v>17646.53245261305</v>
+        <v>16490.71040258798</v>
       </c>
       <c r="C20" t="n">
-        <v>5081.354446074533</v>
+        <v>4640.996638815514</v>
       </c>
       <c r="D20" t="n">
-        <v>8724.719988157949</v>
+        <v>7584.976818747464</v>
       </c>
       <c r="E20" t="n">
-        <v>1116.457265357973</v>
+        <v>1294.364847850794</v>
       </c>
       <c r="F20" t="n">
-        <v>14702.06941570529</v>
+        <v>0.6876363636363636</v>
       </c>
       <c r="G20" t="n">
-        <v>0.6566363636363637</v>
+        <v>13701.8905140677</v>
       </c>
       <c r="H20" t="n">
-        <v>14859.11676246835</v>
+        <v>4035.346973701025</v>
       </c>
       <c r="I20" t="n">
-        <v>4513.150443977992</v>
+        <v>6236.820436750746</v>
       </c>
       <c r="J20" t="n">
-        <v>7242.514285367573</v>
-      </c>
-      <c r="K20" t="n">
-        <v>1000.203992716354</v>
-      </c>
-      <c r="L20" t="n">
-        <v>4883.702091565685</v>
+        <v>848.0407574618436</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="n">
-        <v>0.07734343434343435</v>
+        <v>0.1903838383838384</v>
       </c>
       <c r="B21" t="n">
-        <v>17636.38171667344</v>
+        <v>16467.80890941749</v>
       </c>
       <c r="C21" t="n">
-        <v>5079.511558538014</v>
+        <v>4629.180791168783</v>
       </c>
       <c r="D21" t="n">
-        <v>8721.334676385806</v>
+        <v>7578.90442307164</v>
       </c>
       <c r="E21" t="n">
-        <v>1116.338864514715</v>
+        <v>1296.298284927218</v>
       </c>
       <c r="F21" t="n">
-        <v>14725.36956607472</v>
+        <v>0.7258383838383838</v>
       </c>
       <c r="G21" t="n">
-        <v>0.6931161616161616</v>
+        <v>13582.66745583431</v>
       </c>
       <c r="H21" t="n">
-        <v>14674.61649212234</v>
+        <v>3944.608465920226</v>
       </c>
       <c r="I21" t="n">
-        <v>4429.741233506798</v>
+        <v>6070.478874989134</v>
       </c>
       <c r="J21" t="n">
-        <v>7126.629712922128</v>
-      </c>
-      <c r="K21" t="n">
-        <v>989.9497873929196</v>
-      </c>
-      <c r="L21" t="n">
-        <v>4832.880053093818</v>
+        <v>840.5274904865186</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="n">
-        <v>0.08141414141414142</v>
+        <v>0.2004040404040404</v>
       </c>
       <c r="B22" t="n">
-        <v>17626.17869690986</v>
+        <v>16444.43486368329</v>
       </c>
       <c r="C22" t="n">
-        <v>5077.638150621409</v>
+        <v>4616.598274047882</v>
       </c>
       <c r="D22" t="n">
-        <v>8717.890222789891</v>
+        <v>7575.151088550506</v>
       </c>
       <c r="E22" t="n">
-        <v>1116.214130008169</v>
+        <v>1309.171469209161</v>
       </c>
       <c r="F22" t="n">
-        <v>14749.85677500091</v>
+        <v>0.7640404040404041</v>
       </c>
       <c r="G22" t="n">
-        <v>0.7295959595959596</v>
+        <v>13372.14028998327</v>
       </c>
       <c r="H22" t="n">
-        <v>14487.11897009911</v>
+        <v>3857.572629084786</v>
       </c>
       <c r="I22" t="n">
-        <v>4341.661455255934</v>
+        <v>5994.002034481765</v>
       </c>
       <c r="J22" t="n">
-        <v>7003.978614780235</v>
-      </c>
-      <c r="K22" t="n">
-        <v>979.1242601335274</v>
-      </c>
-      <c r="L22" t="n">
-        <v>4779.315661610953</v>
+        <v>835.3539652488811</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="n">
-        <v>0.0854848484848485</v>
+        <v>0.2104242424242424</v>
       </c>
       <c r="B23" t="n">
-        <v>17615.92317942351</v>
+        <v>16420.59238731208</v>
       </c>
       <c r="C23" t="n">
-        <v>5075.733824594704</v>
+        <v>4603.413828598642</v>
       </c>
       <c r="D23" t="n">
-        <v>8714.385887629305</v>
+        <v>7573.145216476677</v>
       </c>
       <c r="E23" t="n">
-        <v>1116.083039407885</v>
+        <v>1308.928281293694</v>
       </c>
       <c r="F23" t="n">
-        <v>14775.48547913804</v>
+        <v>0.8022424242424242</v>
       </c>
       <c r="G23" t="n">
-        <v>0.7660757575757576</v>
+        <v>13110.77164578778</v>
       </c>
       <c r="H23" t="n">
-        <v>14296.66687353203</v>
+        <v>3777.90621048378</v>
       </c>
       <c r="I23" t="n">
-        <v>4248.572973471425</v>
+        <v>5949.21725107258</v>
       </c>
       <c r="J23" t="n">
-        <v>6874.03052147266</v>
-      </c>
-      <c r="K23" t="n">
-        <v>967.6910937475837</v>
-      </c>
-      <c r="L23" t="n">
-        <v>4722.74363977721</v>
+        <v>836.6628217011091</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="n">
-        <v>0.08955555555555557</v>
+        <v>0.2204444444444444</v>
       </c>
       <c r="B24" t="n">
-        <v>17605.61495031556</v>
+        <v>16396.27955851898</v>
       </c>
       <c r="C24" t="n">
-        <v>5073.798182727885</v>
+        <v>4589.792195966892</v>
       </c>
       <c r="D24" t="n">
-        <v>8710.820931163154</v>
+        <v>7572.315208142767</v>
       </c>
       <c r="E24" t="n">
-        <v>1115.945570283409</v>
+        <v>1302.846019644564</v>
       </c>
       <c r="F24" t="n">
-        <v>14802.21011514026</v>
+        <v>0.8404444444444444</v>
       </c>
       <c r="G24" t="n">
-        <v>0.8025555555555556</v>
+        <v>12853.7367964467</v>
       </c>
       <c r="H24" t="n">
-        <v>14103.30287955453</v>
+        <v>3731.260263786602</v>
       </c>
       <c r="I24" t="n">
-        <v>4150.407130956197</v>
+        <v>5855.69223797721</v>
       </c>
       <c r="J24" t="n">
-        <v>6736.254963530183</v>
-      </c>
-      <c r="K24" t="n">
-        <v>955.6139710444954</v>
-      </c>
-      <c r="L24" t="n">
-        <v>4662.898710252715</v>
+        <v>832.7955455565873</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="n">
-        <v>0.09362626262626264</v>
+        <v>0.2304646464646465</v>
       </c>
       <c r="B25" t="n">
-        <v>17595.25379568721</v>
+        <v>16371.42367396103</v>
       </c>
       <c r="C25" t="n">
-        <v>5071.830827290934</v>
+        <v>4575.89811729846</v>
       </c>
       <c r="D25" t="n">
-        <v>8707.194613650543</v>
+        <v>7572.089464841391</v>
       </c>
       <c r="E25" t="n">
-        <v>1115.801700204291</v>
+        <v>1300.482354824174</v>
       </c>
       <c r="F25" t="n">
-        <v>14829.99857389316</v>
+        <v>0.8786464646464647</v>
       </c>
       <c r="G25" t="n">
-        <v>0.8390353535353535</v>
+        <v>12655.75074360799</v>
       </c>
       <c r="H25" t="n">
-        <v>13907.06966529999</v>
+        <v>3685.180517553226</v>
       </c>
       <c r="I25" t="n">
-        <v>4050.523004389733</v>
+        <v>5735.372512493498</v>
       </c>
       <c r="J25" t="n">
-        <v>6590.12855901</v>
-      </c>
-      <c r="K25" t="n">
-        <v>942.8575984348649</v>
-      </c>
-      <c r="L25" t="n">
-        <v>4599.515595697588</v>
+        <v>817.9503320267086</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="n">
-        <v>0.0976969696969697</v>
+        <v>0.2404848484848485</v>
       </c>
       <c r="B26" t="n">
-        <v>17584.83950163965</v>
+        <v>16345.99880141946</v>
       </c>
       <c r="C26" t="n">
-        <v>5069.831360553841</v>
+        <v>4561.896333739178</v>
       </c>
       <c r="D26" t="n">
-        <v>8703.506195350574</v>
+        <v>7571.896387865163</v>
       </c>
       <c r="E26" t="n">
-        <v>1115.651406740079</v>
+        <v>1311.214834751516</v>
       </c>
       <c r="F26" t="n">
-        <v>14859.50815037148</v>
+        <v>0.9168484848484848</v>
       </c>
       <c r="G26" t="n">
-        <v>0.8755151515151516</v>
+        <v>12531.93950809</v>
       </c>
       <c r="H26" t="n">
-        <v>13708.0099079018</v>
+        <v>3594.853899141952</v>
       </c>
       <c r="I26" t="n">
-        <v>3950.120776769236</v>
+        <v>5597.856029989281</v>
       </c>
       <c r="J26" t="n">
-        <v>6437.872028530061</v>
-      </c>
-      <c r="K26" t="n">
-        <v>929.7512340921231</v>
-      </c>
-      <c r="L26" t="n">
-        <v>4532.329018771954</v>
+        <v>799.7500148781119</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="n">
-        <v>0.1017676767676768</v>
+        <v>0.2505050505050505</v>
       </c>
       <c r="B27" t="n">
-        <v>17574.37185427405</v>
+        <v>16320.00041504205</v>
       </c>
       <c r="C27" t="n">
-        <v>5067.799384786587</v>
+        <v>4547.951586434873</v>
       </c>
       <c r="D27" t="n">
-        <v>8699.754936522348</v>
+        <v>7571.164378506698</v>
       </c>
       <c r="E27" t="n">
-        <v>1115.49466746032</v>
+        <v>1320.904738237897</v>
       </c>
       <c r="F27" t="n">
-        <v>14891.04637619535</v>
+        <v>0.955050505050505</v>
       </c>
       <c r="G27" t="n">
-        <v>0.9119949494949495</v>
+        <v>12428.01956390415</v>
       </c>
       <c r="H27" t="n">
-        <v>13506.16628449337</v>
+        <v>3470.16030569754</v>
       </c>
       <c r="I27" t="n">
-        <v>3849.329436744739</v>
+        <v>5428.929475843494</v>
       </c>
       <c r="J27" t="n">
-        <v>6282.059517039761</v>
-      </c>
-      <c r="K27" t="n">
-        <v>916.5613900957538</v>
-      </c>
-      <c r="L27" t="n">
-        <v>4461.073702135935</v>
+        <v>786.0059578998845</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="n">
-        <v>0.1058383838383838</v>
+        <v>0.2605252525252525</v>
       </c>
       <c r="B28" t="n">
-        <v>17563.8506396916</v>
+        <v>16293.42398897659</v>
       </c>
       <c r="C28" t="n">
-        <v>5065.734502259162</v>
+        <v>4534.228616531377</v>
       </c>
       <c r="D28" t="n">
-        <v>8695.940097424973</v>
+        <v>7569.321838058611</v>
       </c>
       <c r="E28" t="n">
-        <v>1115.331459934562</v>
+        <v>1323.645715316494</v>
       </c>
       <c r="F28" t="n">
-        <v>14924.50648973043</v>
+        <v>0.9932525252525253</v>
       </c>
       <c r="G28" t="n">
-        <v>0.9484747474747475</v>
+        <v>12282.69053608455</v>
       </c>
       <c r="H28" t="n">
-        <v>13301.58147220809</v>
+        <v>3337.868460232333</v>
       </c>
       <c r="I28" t="n">
-        <v>3748.277972966272</v>
+        <v>5214.85568203263</v>
       </c>
       <c r="J28" t="n">
-        <v>6123.422944275234</v>
-      </c>
-      <c r="K28" t="n">
-        <v>903.2631181021411</v>
-      </c>
-      <c r="L28" t="n">
-        <v>4385.497082976015</v>
+        <v>774.7811662596667</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="n">
-        <v>0.1099090909090909</v>
+        <v>0.2705454545454545</v>
       </c>
       <c r="B29" t="n">
-        <v>17553.27564399349</v>
+        <v>16266.26499737087</v>
       </c>
       <c r="C29" t="n">
-        <v>5063.636315241546</v>
+        <v>4520.892165174517</v>
       </c>
       <c r="D29" t="n">
-        <v>8692.060938317551</v>
+        <v>7565.797167813516</v>
       </c>
       <c r="E29" t="n">
-        <v>1115.161761732354</v>
+        <v>1324.770084463213</v>
       </c>
       <c r="F29" t="n">
-        <v>14959.78172934238</v>
+        <v>1.031454545454545</v>
       </c>
       <c r="G29" t="n">
-        <v>0.9849545454545454</v>
+        <v>12052.99916562718</v>
       </c>
       <c r="H29" t="n">
-        <v>13094.29814817935</v>
+        <v>3221.135653707758</v>
       </c>
       <c r="I29" t="n">
-        <v>3647.095374083864</v>
+        <v>5024.504390800175</v>
       </c>
       <c r="J29" t="n">
-        <v>5962.694229972612</v>
-      </c>
-      <c r="K29" t="n">
-        <v>889.8314697676689</v>
-      </c>
-      <c r="L29" t="n">
-        <v>4307.60749665219</v>
+        <v>763.778605717358</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="n">
-        <v>0.113979797979798</v>
+        <v>0.2805656565656566</v>
       </c>
       <c r="B30" t="n">
-        <v>17542.6466532809</v>
+        <v>16238.51891437266</v>
       </c>
       <c r="C30" t="n">
-        <v>5061.504426003728</v>
+        <v>4508.106973510124</v>
       </c>
       <c r="D30" t="n">
-        <v>8688.116719459182</v>
+        <v>7560.01876906403</v>
       </c>
       <c r="E30" t="n">
-        <v>1114.985550423244</v>
+        <v>1324.719898180265</v>
       </c>
       <c r="F30" t="n">
-        <v>14996.76533339688</v>
+        <v>1.069656565656566</v>
       </c>
       <c r="G30" t="n">
-        <v>1.021434343434343</v>
+        <v>11783.38762427381</v>
       </c>
       <c r="H30" t="n">
-        <v>12884.35898954055</v>
+        <v>3115.961687578317</v>
       </c>
       <c r="I30" t="n">
-        <v>3545.910628747546</v>
+        <v>4920.376163015544</v>
       </c>
       <c r="J30" t="n">
-        <v>5800.605293868026</v>
-      </c>
-      <c r="K30" t="n">
-        <v>876.241496748721</v>
-      </c>
-      <c r="L30" t="n">
-        <v>4229.083787512144</v>
+        <v>753.1190043435237</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="n">
-        <v>0.1180505050505051</v>
+        <v>0.2905858585858586</v>
       </c>
       <c r="B31" t="n">
-        <v>17531.96345365503</v>
+        <v>16210.18121412976</v>
       </c>
       <c r="C31" t="n">
-        <v>5059.338436815692</v>
+        <v>4496.037782684025</v>
       </c>
       <c r="D31" t="n">
-        <v>8684.106701108971</v>
+        <v>7551.415043102765</v>
       </c>
       <c r="E31" t="n">
-        <v>1114.80280357678</v>
+        <v>1321.139571344375</v>
       </c>
       <c r="F31" t="n">
-        <v>15035.35054025958</v>
+        <v>1.107858585858586</v>
       </c>
       <c r="G31" t="n">
-        <v>1.057914141414142</v>
+        <v>11501.52740964549</v>
       </c>
       <c r="H31" t="n">
-        <v>12671.80667342509</v>
+        <v>3016.433663690384</v>
       </c>
       <c r="I31" t="n">
-        <v>3444.852725607347</v>
+        <v>4856.286578816122</v>
       </c>
       <c r="J31" t="n">
-        <v>5637.88805569761</v>
-      </c>
-      <c r="K31" t="n">
-        <v>862.4682507016814</v>
-      </c>
-      <c r="L31" t="n">
-        <v>4150.046029008818</v>
+        <v>742.4948249980357</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="n">
-        <v>0.1221212121212121</v>
+        <v>0.3006060606060606</v>
       </c>
       <c r="B32" t="n">
-        <v>17521.22583121705</v>
+        <v>16181.24737078995</v>
       </c>
       <c r="C32" t="n">
-        <v>5057.137949947424</v>
+        <v>4484.849333842051</v>
       </c>
       <c r="D32" t="n">
-        <v>8680.030143526023</v>
+        <v>7539.414391222336</v>
       </c>
       <c r="E32" t="n">
-        <v>1114.61349876251</v>
+        <v>1316.043746256184</v>
       </c>
       <c r="F32" t="n">
-        <v>15075.43058829617</v>
+        <v>1.146060606060606</v>
       </c>
       <c r="G32" t="n">
-        <v>1.094393939393939</v>
+        <v>11230.5571444285</v>
       </c>
       <c r="H32" t="n">
-        <v>12456.68387696637</v>
+        <v>2927.463437106834</v>
       </c>
       <c r="I32" t="n">
-        <v>3344.050653313298</v>
+        <v>4739.448538077143</v>
       </c>
       <c r="J32" t="n">
-        <v>5475.274435197497</v>
-      </c>
-      <c r="K32" t="n">
-        <v>848.4867832829341</v>
-      </c>
-      <c r="L32" t="n">
-        <v>4070.614294595159</v>
+        <v>731.6290778002037</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="n">
-        <v>0.1261919191919192</v>
+        <v>0.3106262626262626</v>
       </c>
       <c r="B33" t="n">
-        <v>17510.43357206815</v>
+        <v>16151.71285850101</v>
       </c>
       <c r="C33" t="n">
-        <v>5054.902567668909</v>
+        <v>4474.707664284766</v>
       </c>
       <c r="D33" t="n">
-        <v>8675.886306969442</v>
+        <v>7523.44521471536</v>
       </c>
       <c r="E33" t="n">
-        <v>1114.417613549981</v>
+        <v>1314.146796115082</v>
       </c>
       <c r="F33" t="n">
-        <v>15116.89871587229</v>
+        <v>1.184262626262626</v>
       </c>
       <c r="G33" t="n">
-        <v>1.130873737373737</v>
+        <v>10986.57833317185</v>
       </c>
       <c r="H33" t="n">
-        <v>12239.03327729777</v>
+        <v>2867.052451937181</v>
       </c>
       <c r="I33" t="n">
-        <v>3243.633400515431</v>
+        <v>4600.779628923695</v>
       </c>
       <c r="J33" t="n">
-        <v>5313.496352103819</v>
-      </c>
-      <c r="K33" t="n">
-        <v>834.2721461488626</v>
-      </c>
-      <c r="L33" t="n">
-        <v>3990.908657724111</v>
+        <v>720.5341324756403</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="n">
-        <v>0.1302626262626263</v>
+        <v>0.3206464646464646</v>
       </c>
       <c r="B34" t="n">
-        <v>17499.58646230952</v>
+        <v>16121.57315141074</v>
       </c>
       <c r="C34" t="n">
-        <v>5052.631892250132</v>
+        <v>4466.061711105674</v>
       </c>
       <c r="D34" t="n">
-        <v>8671.674451698329</v>
+        <v>7502.935914874448</v>
       </c>
       <c r="E34" t="n">
-        <v>1114.215125508743</v>
+        <v>1330.150521717156</v>
       </c>
       <c r="F34" t="n">
-        <v>15159.64816135363</v>
+        <v>1.222464646464646</v>
       </c>
       <c r="G34" t="n">
-        <v>1.167353535353535</v>
+        <v>10751.55543891136</v>
       </c>
       <c r="H34" t="n">
-        <v>12018.8975515527</v>
+        <v>2805.722765647534</v>
       </c>
       <c r="I34" t="n">
-        <v>3143.729955863774</v>
+        <v>4459.521170524194</v>
       </c>
       <c r="J34" t="n">
-        <v>5153.285726152709</v>
-      </c>
-      <c r="K34" t="n">
-        <v>819.7993909558514</v>
-      </c>
-      <c r="L34" t="n">
-        <v>3911.049191848618</v>
+        <v>709.238632504579</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="n">
-        <v>0.1343333333333333</v>
+        <v>0.3306666666666667</v>
       </c>
       <c r="B35" t="n">
-        <v>17488.68428804235</v>
+        <v>16090.82372366691</v>
       </c>
       <c r="C35" t="n">
-        <v>5050.325525961079</v>
+        <v>4458.975437998882</v>
       </c>
       <c r="D35" t="n">
-        <v>8667.393837971791</v>
+        <v>7477.979845009359</v>
       </c>
       <c r="E35" t="n">
-        <v>1114.006012208343</v>
+        <v>1337.910965761772</v>
       </c>
       <c r="F35" t="n">
-        <v>15203.57216310585</v>
+        <v>1.260666666666667</v>
       </c>
       <c r="G35" t="n">
-        <v>1.203833333333333</v>
+        <v>10523.70573356396</v>
       </c>
       <c r="H35" t="n">
-        <v>11796.31937686455</v>
+        <v>2708.789703310692</v>
       </c>
       <c r="I35" t="n">
-        <v>3044.442956166844</v>
+        <v>4315.282105422536</v>
       </c>
       <c r="J35" t="n">
-        <v>4995.3744770803</v>
-      </c>
-      <c r="K35" t="n">
-        <v>805.0435693602843</v>
-      </c>
-      <c r="L35" t="n">
-        <v>3831.155970421625</v>
+        <v>697.7827352965579</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="n">
-        <v>0.1384040404040404</v>
+        <v>0.3406868686868686</v>
       </c>
       <c r="B36" t="n">
-        <v>17477.72683536781</v>
+        <v>16059.46004941732</v>
       </c>
       <c r="C36" t="n">
-        <v>5047.983071071734</v>
+        <v>4453.153826200603</v>
       </c>
       <c r="D36" t="n">
-        <v>8663.043726048925</v>
+        <v>7451.989274904658</v>
       </c>
       <c r="E36" t="n">
-        <v>1113.790251218329</v>
+        <v>1332.481201371653</v>
       </c>
       <c r="F36" t="n">
-        <v>15248.56395949461</v>
+        <v>1.298868686868687</v>
       </c>
       <c r="G36" t="n">
-        <v>1.240313131313131</v>
+        <v>10304.59624931891</v>
       </c>
       <c r="H36" t="n">
-        <v>11571.34143036672</v>
+        <v>2586.252800072155</v>
       </c>
       <c r="I36" t="n">
-        <v>2945.413778092697</v>
+        <v>4168.942418198217</v>
       </c>
       <c r="J36" t="n">
-        <v>4840.494524622723</v>
-      </c>
-      <c r="K36" t="n">
-        <v>789.9797330185448</v>
-      </c>
-      <c r="L36" t="n">
-        <v>3751.349066896077</v>
+        <v>686.1914320953025</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="n">
-        <v>0.1424747474747475</v>
+        <v>0.3507070707070707</v>
       </c>
       <c r="B37" t="n">
-        <v>17466.7138903871</v>
+        <v>16027.47760280974</v>
       </c>
       <c r="C37" t="n">
-        <v>5045.604129852083</v>
+        <v>4448.301856947049</v>
       </c>
       <c r="D37" t="n">
-        <v>8658.623376188843</v>
+        <v>7425.565482470579</v>
       </c>
       <c r="E37" t="n">
-        <v>1113.56782010825</v>
+        <v>1327.248099642739</v>
       </c>
       <c r="F37" t="n">
-        <v>15295.10097310399</v>
+        <v>1.337070707070707</v>
       </c>
       <c r="G37" t="n">
-        <v>1.276792929292929</v>
+        <v>10120.74584777647</v>
       </c>
       <c r="H37" t="n">
-        <v>11344.0063891926</v>
+        <v>2460.047391666792</v>
       </c>
       <c r="I37" t="n">
-        <v>2846.516634623521</v>
+        <v>4020.775498287032</v>
       </c>
       <c r="J37" t="n">
-        <v>4689.329676305138</v>
-      </c>
-      <c r="K37" t="n">
-        <v>774.6203914640204</v>
-      </c>
-      <c r="L37" t="n">
-        <v>3671.748554724918</v>
+        <v>674.4372458934937</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="n">
-        <v>0.1465454545454546</v>
+        <v>0.3607272727272727</v>
       </c>
       <c r="B38" t="n">
-        <v>17455.6452392014</v>
+        <v>15994.87185799197</v>
       </c>
       <c r="C38" t="n">
-        <v>5043.188304572112</v>
+        <v>4444.124511474432</v>
       </c>
       <c r="D38" t="n">
-        <v>8654.132048650647</v>
+        <v>7398.746801728502</v>
       </c>
       <c r="E38" t="n">
-        <v>1113.338696447653</v>
+        <v>1334.971460988935</v>
       </c>
       <c r="F38" t="n">
-        <v>15344.55571098136</v>
+        <v>1.375272727272727</v>
       </c>
       <c r="G38" t="n">
-        <v>1.313272727272727</v>
+        <v>9976.523650820238</v>
       </c>
       <c r="H38" t="n">
-        <v>11114.08344299674</v>
+        <v>2349.28740215581</v>
       </c>
       <c r="I38" t="n">
-        <v>2747.786396365197</v>
+        <v>3855.016871887188</v>
       </c>
       <c r="J38" t="n">
-        <v>4540.049986101926</v>
-      </c>
-      <c r="K38" t="n">
-        <v>759.124426297369</v>
-      </c>
-      <c r="L38" t="n">
-        <v>3592.47450736109</v>
+        <v>662.5976845359671</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="n">
-        <v>0.1506161616161616</v>
+        <v>0.3707474747474747</v>
       </c>
       <c r="B39" t="n">
-        <v>17444.5206679119</v>
+        <v>15961.63828911178</v>
       </c>
       <c r="C39" t="n">
-        <v>5040.735197501805</v>
+        <v>4440.326771018962</v>
       </c>
       <c r="D39" t="n">
-        <v>8649.569003693432</v>
+        <v>7371.571566699813</v>
       </c>
       <c r="E39" t="n">
-        <v>1113.102857806086</v>
+        <v>1353.323808201449</v>
       </c>
       <c r="F39" t="n">
-        <v>15396.81143853883</v>
+        <v>1.413474747474748</v>
       </c>
       <c r="G39" t="n">
-        <v>1.349752525252525</v>
+        <v>9822.769332424004</v>
       </c>
       <c r="H39" t="n">
-        <v>10881.09731607644</v>
+        <v>2248.607852710652</v>
       </c>
       <c r="I39" t="n">
-        <v>2649.257933923604</v>
+        <v>3654.579615030288</v>
       </c>
       <c r="J39" t="n">
-        <v>4391.468946598996</v>
-      </c>
-      <c r="K39" t="n">
-        <v>743.5334575117054</v>
-      </c>
-      <c r="L39" t="n">
-        <v>3513.646998257542</v>
+        <v>650.62639119431</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="n">
-        <v>0.1546868686868687</v>
+        <v>0.3807676767676768</v>
       </c>
       <c r="B40" t="n">
-        <v>17433.33996261978</v>
+        <v>15927.77237031698</v>
       </c>
       <c r="C40" t="n">
-        <v>5038.244410911149</v>
+        <v>4436.613616816852</v>
       </c>
       <c r="D40" t="n">
-        <v>8644.93350157631</v>
+        <v>7344.078111405894</v>
       </c>
       <c r="E40" t="n">
-        <v>1112.860281753098</v>
+        <v>1358.586357035532</v>
       </c>
       <c r="F40" t="n">
-        <v>15451.67103587952</v>
+        <v>1.451676767676768</v>
       </c>
       <c r="G40" t="n">
-        <v>1.386232323232323</v>
+        <v>9611.517943622115</v>
       </c>
       <c r="H40" t="n">
-        <v>10645.42574579182</v>
+        <v>2154.892145816172</v>
       </c>
       <c r="I40" t="n">
-        <v>2550.966117904625</v>
+        <v>3475.368319585583</v>
       </c>
       <c r="J40" t="n">
-        <v>4243.674155117001</v>
-      </c>
-      <c r="K40" t="n">
-        <v>727.8714633776768</v>
-      </c>
-      <c r="L40" t="n">
-        <v>3435.386100867217</v>
+        <v>638.565606814198</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="n">
-        <v>0.1587575757575758</v>
+        <v>0.3907878787878787</v>
       </c>
       <c r="B41" t="n">
-        <v>17422.10290942623</v>
+        <v>15893.26957575533</v>
       </c>
       <c r="C41" t="n">
-        <v>5035.715547070128</v>
+        <v>4432.690030104314</v>
       </c>
       <c r="D41" t="n">
-        <v>8640.224802558379</v>
+        <v>7316.304769868128</v>
       </c>
       <c r="E41" t="n">
-        <v>1112.610945858238</v>
+        <v>1361.424822258318</v>
       </c>
       <c r="F41" t="n">
-        <v>15508.93738310654</v>
+        <v>1.489878787878788</v>
       </c>
       <c r="G41" t="n">
-        <v>1.422712121212121</v>
+        <v>9342.48248904291</v>
       </c>
       <c r="H41" t="n">
-        <v>10407.486852584</v>
+        <v>2073.252362657366</v>
       </c>
       <c r="I41" t="n">
-        <v>2452.945818914136</v>
+        <v>3366.936066770271</v>
       </c>
       <c r="J41" t="n">
-        <v>4096.753208976588</v>
-      </c>
-      <c r="K41" t="n">
-        <v>712.1624221659309</v>
-      </c>
-      <c r="L41" t="n">
-        <v>3357.811888643057</v>
+        <v>626.4832265993678</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="n">
-        <v>0.1628282828282828</v>
+        <v>0.4008080808080808</v>
       </c>
       <c r="B42" t="n">
-        <v>17410.80929443243</v>
+        <v>15858.12537957463</v>
       </c>
       <c r="C42" t="n">
-        <v>5033.148208248727</v>
+        <v>4428.260992117559</v>
       </c>
       <c r="D42" t="n">
-        <v>8635.442166898747</v>
+        <v>7288.289876107902</v>
       </c>
       <c r="E42" t="n">
-        <v>1112.354827691051</v>
+        <v>1362.734391466278</v>
       </c>
       <c r="F42" t="n">
-        <v>15568.41336032302</v>
+        <v>1.528080808080808</v>
       </c>
       <c r="G42" t="n">
-        <v>1.459191919191919</v>
+        <v>9047.694691385905</v>
       </c>
       <c r="H42" t="n">
-        <v>10167.69875689413</v>
+        <v>2012.859524057444</v>
       </c>
       <c r="I42" t="n">
-        <v>2355.23190755802</v>
+        <v>3291.198547484204</v>
       </c>
       <c r="J42" t="n">
-        <v>3950.793705498409</v>
-      </c>
-      <c r="K42" t="n">
-        <v>696.430312147115</v>
-      </c>
-      <c r="L42" t="n">
-        <v>3280.707017348507</v>
+        <v>614.3797760815888</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="n">
-        <v>0.1668989898989899</v>
+        <v>0.4108282828282828</v>
       </c>
       <c r="B43" t="n">
-        <v>17399.45890373958</v>
+        <v>15822.33525592266</v>
       </c>
       <c r="C43" t="n">
-        <v>5030.541996716934</v>
+        <v>4423.031484092799</v>
       </c>
       <c r="D43" t="n">
-        <v>8630.584854856515</v>
+        <v>7260.071764146596</v>
       </c>
       <c r="E43" t="n">
-        <v>1112.091904821088</v>
+        <v>1361.365024254509</v>
       </c>
       <c r="F43" t="n">
-        <v>15629.90184763208</v>
+        <v>1.566282828282828</v>
       </c>
       <c r="G43" t="n">
-        <v>1.495671717171717</v>
+        <v>8755.120383072608</v>
       </c>
       <c r="H43" t="n">
-        <v>9926.47957916337</v>
+        <v>1950.769342081132</v>
       </c>
       <c r="I43" t="n">
-        <v>2257.859254442155</v>
+        <v>3177.419230405014</v>
       </c>
       <c r="J43" t="n">
-        <v>3805.883242003114</v>
-      </c>
-      <c r="K43" t="n">
-        <v>680.6991115918764</v>
-      </c>
-      <c r="L43" t="n">
-        <v>3203.65659644378</v>
+        <v>602.2494344605969</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="n">
-        <v>0.170969696969697</v>
+        <v>0.4208484848484848</v>
       </c>
       <c r="B44" t="n">
-        <v>17388.05152344886</v>
+        <v>15785.89622658684</v>
       </c>
       <c r="C44" t="n">
-        <v>5027.896514744731</v>
+        <v>4416.706487266243</v>
       </c>
       <c r="D44" t="n">
-        <v>8625.652126690788</v>
+        <v>7231.688768005595</v>
       </c>
       <c r="E44" t="n">
-        <v>1111.822154817895</v>
+        <v>1356.50071497816</v>
       </c>
       <c r="F44" t="n">
-        <v>15693.20572513683</v>
+        <v>1.604484848484848</v>
       </c>
       <c r="G44" t="n">
-        <v>1.532151515151515</v>
+        <v>8491.662321395401</v>
       </c>
       <c r="H44" t="n">
-        <v>9684.247439832843</v>
+        <v>1863.712778235317</v>
       </c>
       <c r="I44" t="n">
-        <v>2160.862730172421</v>
+        <v>3050.135810241009</v>
       </c>
       <c r="J44" t="n">
-        <v>3662.109415811355</v>
-      </c>
-      <c r="K44" t="n">
-        <v>664.9927987708621</v>
-      </c>
-      <c r="L44" t="n">
-        <v>3126.677937552585</v>
+        <v>590.1057730239353</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="n">
-        <v>0.1750404040404041</v>
+        <v>0.4308686868686868</v>
       </c>
       <c r="B45" t="n">
-        <v>17376.58693966144</v>
+        <v>15748.84178836995</v>
       </c>
       <c r="C45" t="n">
-        <v>5025.211364602104</v>
+        <v>4408.990982874107</v>
       </c>
       <c r="D45" t="n">
-        <v>8620.643242660666</v>
+        <v>7203.179221706284</v>
       </c>
       <c r="E45" t="n">
-        <v>1111.545555251022</v>
+        <v>1353.286006202741</v>
       </c>
       <c r="F45" t="n">
-        <v>15758.12787294039</v>
+        <v>1.642686868686869</v>
       </c>
       <c r="G45" t="n">
-        <v>1.568631313131313</v>
+        <v>8246.777369709407</v>
       </c>
       <c r="H45" t="n">
-        <v>9441.420459343704</v>
+        <v>1760.386391171054</v>
       </c>
       <c r="I45" t="n">
-        <v>2064.277205354699</v>
+        <v>2922.991486027365</v>
       </c>
       <c r="J45" t="n">
-        <v>3519.559824243781</v>
-      </c>
-      <c r="K45" t="n">
-        <v>649.3353519547202</v>
-      </c>
-      <c r="L45" t="n">
-        <v>3049.79152828628</v>
+        <v>577.7053713605732</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="n">
-        <v>0.1791111111111111</v>
+        <v>0.4408888888888889</v>
       </c>
       <c r="B46" t="n">
-        <v>17365.06493847853</v>
+        <v>15711.18299772447</v>
       </c>
       <c r="C46" t="n">
-        <v>5022.486148559039</v>
+        <v>4399.589952152601</v>
       </c>
       <c r="D46" t="n">
-        <v>8615.557463025258</v>
+        <v>7174.581459270044</v>
       </c>
       <c r="E46" t="n">
-        <v>1111.262083690016</v>
+        <v>1364.900454210799</v>
       </c>
       <c r="F46" t="n">
-        <v>15824.47117114588</v>
+        <v>1.680888888888889</v>
       </c>
       <c r="G46" t="n">
-        <v>1.605111111111111</v>
+        <v>8010.670456393733</v>
       </c>
       <c r="H46" t="n">
-        <v>9198.416758137093</v>
+        <v>1656.41927128989</v>
       </c>
       <c r="I46" t="n">
-        <v>1968.250460177065</v>
+        <v>2796.826112908647</v>
       </c>
       <c r="J46" t="n">
-        <v>3378.322064621044</v>
-      </c>
-      <c r="K46" t="n">
-        <v>633.7507494140975</v>
-      </c>
-      <c r="L46" t="n">
-        <v>2973.017856256228</v>
+        <v>565.243992429743</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="n">
-        <v>0.1831818181818182</v>
+        <v>0.4509090909090909</v>
       </c>
       <c r="B47" t="n">
-        <v>17353.4853060013</v>
+        <v>15672.91429507695</v>
       </c>
       <c r="C47" t="n">
-        <v>5019.720468885522</v>
+        <v>4388.207607844804</v>
       </c>
       <c r="D47" t="n">
-        <v>8610.394048043661</v>
+        <v>7145.93381471826</v>
       </c>
       <c r="E47" t="n">
-        <v>1110.971717704424</v>
+        <v>1384.757709323185</v>
       </c>
       <c r="F47" t="n">
-        <v>15892.03849985642</v>
+        <v>1.719090909090909</v>
       </c>
       <c r="G47" t="n">
-        <v>1.641590909090909</v>
+        <v>7786.147242977672</v>
       </c>
       <c r="H47" t="n">
-        <v>8955.654456654158</v>
+        <v>1565.218815444648</v>
       </c>
       <c r="I47" t="n">
-        <v>1875.487450406893</v>
+        <v>2671.220230952637</v>
       </c>
       <c r="J47" t="n">
-        <v>3238.483734263795</v>
-      </c>
-      <c r="K47" t="n">
-        <v>618.2629694196415</v>
-      </c>
-      <c r="L47" t="n">
-        <v>2896.377409073787</v>
+        <v>556.4492583178493</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="n">
-        <v>0.1872525252525253</v>
+        <v>0.4609292929292929</v>
       </c>
       <c r="B48" t="n">
-        <v>17341.84782833094</v>
+        <v>15634.03012085397</v>
       </c>
       <c r="C48" t="n">
-        <v>5016.913927851538</v>
+        <v>4374.624160931831</v>
       </c>
       <c r="D48" t="n">
-        <v>8605.152257974985</v>
+        <v>7117.274622072315</v>
       </c>
       <c r="E48" t="n">
-        <v>1110.674434863797</v>
+        <v>1383.327092162742</v>
       </c>
       <c r="F48" t="n">
-        <v>15960.82627046485</v>
+        <v>1.757292929292929</v>
       </c>
       <c r="G48" t="n">
-        <v>1.678070707070707</v>
+        <v>7581.997581076752</v>
       </c>
       <c r="H48" t="n">
-        <v>8713.551675336039</v>
+        <v>1482.093659495456</v>
       </c>
       <c r="I48" t="n">
-        <v>1786.896845059218</v>
+        <v>2545.551238580165</v>
       </c>
       <c r="J48" t="n">
-        <v>3100.132430492683</v>
-      </c>
-      <c r="K48" t="n">
-        <v>602.8955139695033</v>
-      </c>
-      <c r="L48" t="n">
-        <v>2819.890674350321</v>
+        <v>552.4391614972218</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="n">
-        <v>0.1913232323232323</v>
+        <v>0.4709494949494949</v>
       </c>
       <c r="B49" t="n">
-        <v>17330.15229156863</v>
+        <v>15594.5249154821</v>
       </c>
       <c r="C49" t="n">
-        <v>5014.06612772707</v>
+        <v>4359.015272263192</v>
       </c>
       <c r="D49" t="n">
-        <v>8599.831353078331</v>
+        <v>7088.642215353593</v>
       </c>
       <c r="E49" t="n">
-        <v>1110.370212737681</v>
+        <v>1376.586080317635</v>
       </c>
       <c r="F49" t="n">
-        <v>16033.5036525732</v>
+        <v>1.795494949494949</v>
       </c>
       <c r="G49" t="n">
-        <v>1.714550505050505</v>
+        <v>7415.520847669045</v>
       </c>
       <c r="H49" t="n">
-        <v>8472.526534623881</v>
+        <v>1406.363063554542</v>
       </c>
       <c r="I49" t="n">
-        <v>1702.17141688113</v>
+        <v>2408.776531396565</v>
       </c>
       <c r="J49" t="n">
-        <v>2963.900135404574</v>
-      </c>
-      <c r="K49" t="n">
-        <v>587.6218268895558</v>
-      </c>
-      <c r="L49" t="n">
-        <v>2743.578139697188</v>
+        <v>541.5392031536111</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="n">
-        <v>0.1953939393939394</v>
+        <v>0.4809696969696969</v>
       </c>
       <c r="B50" t="n">
-        <v>17318.39848181557</v>
+        <v>15554.39311938791</v>
       </c>
       <c r="C50" t="n">
-        <v>5011.176670782107</v>
+        <v>4341.655397849573</v>
       </c>
       <c r="D50" t="n">
-        <v>8594.4305936128</v>
+        <v>7060.074928583477</v>
       </c>
       <c r="E50" t="n">
-        <v>1110.059028895624</v>
+        <v>1379.367345921952</v>
       </c>
       <c r="F50" t="n">
-        <v>16110.69581272714</v>
+        <v>1.83369696969697</v>
       </c>
       <c r="G50" t="n">
-        <v>1.751030303030303</v>
+        <v>7259.141275480596</v>
       </c>
       <c r="H50" t="n">
-        <v>8232.997154958828</v>
+        <v>1341.990968697659</v>
       </c>
       <c r="I50" t="n">
-        <v>1621.003938619721</v>
+        <v>2253.918145739176</v>
       </c>
       <c r="J50" t="n">
-        <v>2831.449258306398</v>
-      </c>
-      <c r="K50" t="n">
-        <v>572.41587013802</v>
-      </c>
-      <c r="L50" t="n">
-        <v>2667.460292725749</v>
+        <v>522.2658204877606</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="n">
-        <v>0.1994646464646465</v>
+        <v>0.490989898989899</v>
       </c>
       <c r="B51" t="n">
-        <v>17306.58618517294</v>
+        <v>15513.62917299797</v>
       </c>
       <c r="C51" t="n">
-        <v>5008.245159286632</v>
+        <v>4322.818993701661</v>
       </c>
       <c r="D51" t="n">
-        <v>8588.949239837497</v>
+        <v>7031.611095783352</v>
       </c>
       <c r="E51" t="n">
-        <v>1109.740860907175</v>
+        <v>1403.426374487855</v>
       </c>
       <c r="F51" t="n">
-        <v>16192.03449466143</v>
+        <v>1.87189898989899</v>
       </c>
       <c r="G51" t="n">
-        <v>1.787510101010101</v>
+        <v>7080.356432325135</v>
       </c>
       <c r="H51" t="n">
-        <v>7995.381656782024</v>
+        <v>1290.78736700697</v>
       </c>
       <c r="I51" t="n">
-        <v>1543.087183022087</v>
+        <v>2117.222869691724</v>
       </c>
       <c r="J51" t="n">
-        <v>2702.822233359074</v>
-      </c>
-      <c r="K51" t="n">
-        <v>557.2787914630928</v>
-      </c>
-      <c r="L51" t="n">
-        <v>2591.557621047366</v>
+        <v>502.0498276570724</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="n">
-        <v>0.2035353535353535</v>
+        <v>0.501010101010101</v>
       </c>
       <c r="B52" t="n">
-        <v>17294.71518774192</v>
+        <v>15472.22751673886</v>
       </c>
       <c r="C52" t="n">
-        <v>5005.27119551063</v>
+        <v>4302.780515830146</v>
       </c>
       <c r="D52" t="n">
-        <v>8583.386552011527</v>
+        <v>7003.262235461213</v>
       </c>
       <c r="E52" t="n">
-        <v>1109.415686341881</v>
+        <v>1416.13771977047</v>
       </c>
       <c r="F52" t="n">
-        <v>16277.15144211083</v>
+        <v>1.91010101010101</v>
       </c>
       <c r="G52" t="n">
-        <v>1.823989898989899</v>
+        <v>6850.281548539114</v>
       </c>
       <c r="H52" t="n">
-        <v>7760.098160534615</v>
+        <v>1238.740336561467</v>
       </c>
       <c r="I52" t="n">
-        <v>1468.113922835317</v>
+        <v>2027.906673002324</v>
       </c>
       <c r="J52" t="n">
-        <v>2577.94553745074</v>
-      </c>
-      <c r="K52" t="n">
-        <v>542.2117386129706</v>
-      </c>
-      <c r="L52" t="n">
-        <v>2515.890612273398</v>
+        <v>486.8168059423417</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="n">
-        <v>0.2076060606060606</v>
+        <v>0.5110303030303029</v>
       </c>
       <c r="B53" t="n">
-        <v>17282.7852756237</v>
+        <v>15430.18259103714</v>
       </c>
       <c r="C53" t="n">
-        <v>5002.254381724088</v>
+        <v>4281.814420245714</v>
       </c>
       <c r="D53" t="n">
-        <v>8577.74179039399</v>
+        <v>6974.893872350609</v>
       </c>
       <c r="E53" t="n">
-        <v>1109.083482769291</v>
+        <v>1421.760379557297</v>
       </c>
       <c r="F53" t="n">
-        <v>16365.67839881012</v>
+        <v>1.94830303030303</v>
       </c>
       <c r="G53" t="n">
-        <v>1.860469696969697</v>
+        <v>6582.424753034319</v>
       </c>
       <c r="H53" t="n">
-        <v>7527.564786657744</v>
+        <v>1171.368730948161</v>
       </c>
       <c r="I53" t="n">
-        <v>1395.776930806505</v>
+        <v>1960.428007982312</v>
       </c>
       <c r="J53" t="n">
-        <v>2456.745647469531</v>
-      </c>
-      <c r="K53" t="n">
-        <v>527.2158593358498</v>
-      </c>
-      <c r="L53" t="n">
-        <v>2440.479754015206</v>
+        <v>472.8660423577792</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="n">
-        <v>0.2116767676767677</v>
+        <v>0.521050505050505</v>
       </c>
       <c r="B54" t="n">
-        <v>17270.79623491947</v>
+        <v>15387.48883631938</v>
       </c>
       <c r="C54" t="n">
-        <v>4999.19432019699</v>
+        <v>4260.195162959054</v>
       </c>
       <c r="D54" t="n">
-        <v>8572.014215243993</v>
+        <v>6946.487072429242</v>
       </c>
       <c r="E54" t="n">
-        <v>1108.744227758953</v>
+        <v>1425.412730048904</v>
       </c>
       <c r="F54" t="n">
-        <v>16457.24710849403</v>
+        <v>1.986505050505051</v>
       </c>
       <c r="G54" t="n">
-        <v>1.896949494949495</v>
+        <v>6311.705619137216</v>
       </c>
       <c r="H54" t="n">
-        <v>7298.199655592552</v>
+        <v>1091.583227300003</v>
       </c>
       <c r="I54" t="n">
-        <v>1325.768979682742</v>
+        <v>1874.444485098319</v>
       </c>
       <c r="J54" t="n">
-        <v>2339.149040303585</v>
-      </c>
-      <c r="K54" t="n">
-        <v>512.2923013799274</v>
-      </c>
-      <c r="L54" t="n">
-        <v>2365.363473038212</v>
+        <v>459.7313416709109</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="n">
-        <v>0.2157474747474748</v>
+        <v>0.531070707070707</v>
       </c>
       <c r="B55" t="n">
-        <v>17258.7478517304</v>
+        <v>15344.14069301216</v>
       </c>
       <c r="C55" t="n">
-        <v>4996.090613199322</v>
+        <v>4238.197199980853</v>
       </c>
       <c r="D55" t="n">
-        <v>8566.203086820638</v>
+        <v>6918.048393165155</v>
       </c>
       <c r="E55" t="n">
-        <v>1108.397898880415</v>
+        <v>1427.273441537638</v>
       </c>
       <c r="F55" t="n">
-        <v>16551.48931489735</v>
+        <v>2.024707070707071</v>
       </c>
       <c r="G55" t="n">
-        <v>1.933429292929293</v>
+        <v>6073.10447203325</v>
       </c>
       <c r="H55" t="n">
-        <v>7072.420887780186</v>
+        <v>1015.31059136287</v>
       </c>
       <c r="I55" t="n">
-        <v>1257.782842211123</v>
+        <v>1781.26423944499</v>
       </c>
       <c r="J55" t="n">
-        <v>2225.082192841038</v>
-      </c>
-      <c r="K55" t="n">
-        <v>497.4422124933993</v>
-      </c>
-      <c r="L55" t="n">
-        <v>2291.396013228847</v>
+        <v>447.1306060949139</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="n">
-        <v>0.2198181818181818</v>
+        <v>0.5410909090909091</v>
       </c>
       <c r="B56" t="n">
-        <v>17246.6399121577</v>
+        <v>15300.13260154205</v>
       </c>
       <c r="C56" t="n">
-        <v>4992.942863001069</v>
+        <v>4216.0949873218</v>
       </c>
       <c r="D56" t="n">
-        <v>8560.307665383027</v>
+        <v>6889.584392026379</v>
       </c>
       <c r="E56" t="n">
-        <v>1108.044907572347</v>
+        <v>1424.494773926349</v>
       </c>
       <c r="F56" t="n">
-        <v>16648.03676175483</v>
+        <v>2.062909090909091</v>
       </c>
       <c r="G56" t="n">
-        <v>1.969909090909091</v>
+        <v>5887.487628892707</v>
       </c>
       <c r="H56" t="n">
-        <v>6850.494208993469</v>
+        <v>957.1694460962024</v>
       </c>
       <c r="I56" t="n">
-        <v>1191.511291138738</v>
+        <v>1685.985762260013</v>
       </c>
       <c r="J56" t="n">
-        <v>2114.471581970027</v>
-      </c>
-      <c r="K56" t="n">
-        <v>482.6667404244624</v>
-      </c>
-      <c r="L56" t="n">
-        <v>2218.97309575814</v>
+        <v>434.6010323070251</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="n">
-        <v>0.2238888888888889</v>
+        <v>0.5511111111111111</v>
       </c>
       <c r="B57" t="n">
-        <v>17234.47220230254</v>
+        <v>15255.45900233561</v>
       </c>
       <c r="C57" t="n">
-        <v>4989.750671872216</v>
+        <v>4194.16298099258</v>
       </c>
       <c r="D57" t="n">
-        <v>8554.327211190268</v>
+        <v>6861.101626480954</v>
       </c>
       <c r="E57" t="n">
-        <v>1107.686516415442</v>
+        <v>1421.401648216974</v>
       </c>
       <c r="F57" t="n">
-        <v>16746.52119280122</v>
+        <v>2.101111111111111</v>
       </c>
       <c r="G57" t="n">
-        <v>2.006388888888889</v>
+        <v>5729.289830216704</v>
       </c>
       <c r="H57" t="n">
-        <v>6632.349859905356</v>
+        <v>911.7864542297177</v>
       </c>
       <c r="I57" t="n">
-        <v>1126.668117051214</v>
+        <v>1583.385856049829</v>
       </c>
       <c r="J57" t="n">
-        <v>2007.243684578689</v>
-      </c>
-      <c r="K57" t="n">
-        <v>467.967032921313</v>
-      </c>
-      <c r="L57" t="n">
-        <v>2148.005207080452</v>
+        <v>422.2128704466591</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="n">
-        <v>0.227959595959596</v>
+        <v>0.5611313131313131</v>
       </c>
       <c r="B58" t="n">
-        <v>17222.24450826611</v>
+        <v>15210.11433581942</v>
       </c>
       <c r="C58" t="n">
-        <v>4986.513642082748</v>
+        <v>4172.675637003883</v>
       </c>
       <c r="D58" t="n">
-        <v>8548.260984501459</v>
+        <v>6832.606653996916</v>
       </c>
       <c r="E58" t="n">
-        <v>1107.322776550302</v>
+        <v>1426.545701537372</v>
       </c>
       <c r="F58" t="n">
-        <v>16846.57435177131</v>
+        <v>2.139313131313131</v>
       </c>
       <c r="G58" t="n">
-        <v>2.042868686868687</v>
+        <v>5570.252381355675</v>
       </c>
       <c r="H58" t="n">
-        <v>6417.972862544797</v>
+        <v>867.0152024433283</v>
       </c>
       <c r="I58" t="n">
-        <v>1063.79650911046</v>
+        <v>1467.842543621274</v>
       </c>
       <c r="J58" t="n">
-        <v>1903.324977555162</v>
-      </c>
-      <c r="K58" t="n">
-        <v>453.344237732148</v>
-      </c>
-      <c r="L58" t="n">
-        <v>2078.402833650143</v>
+        <v>409.8626194815014</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="n">
-        <v>0.2320303030303031</v>
+        <v>0.5711515151515151</v>
       </c>
       <c r="B59" t="n">
-        <v>17209.95661614959</v>
+        <v>15164.09304242006</v>
       </c>
       <c r="C59" t="n">
-        <v>4983.231375902652</v>
+        <v>4151.907411366399</v>
       </c>
       <c r="D59" t="n">
-        <v>8542.10824557571</v>
+        <v>6804.106032042299</v>
       </c>
       <c r="E59" t="n">
-        <v>1106.953653220499</v>
+        <v>1458.072133730449</v>
       </c>
       <c r="F59" t="n">
-        <v>16947.82798239984</v>
+        <v>2.177515151515152</v>
       </c>
       <c r="G59" t="n">
-        <v>2.079348484848485</v>
+        <v>5382.866208494302</v>
       </c>
       <c r="H59" t="n">
-        <v>6207.349747485377</v>
+        <v>813.7916103919787</v>
       </c>
       <c r="I59" t="n">
-        <v>1003.281211384819</v>
+        <v>1364.662166527034</v>
       </c>
       <c r="J59" t="n">
-        <v>1802.641937787581</v>
-      </c>
-      <c r="K59" t="n">
-        <v>438.7995026051635</v>
-      </c>
-      <c r="L59" t="n">
-        <v>2010.07646192157</v>
+        <v>397.6000966361032</v>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="n">
-        <v>0.2361010101010101</v>
+        <v>0.5811717171717171</v>
       </c>
       <c r="B60" t="n">
-        <v>17197.60831205418</v>
+        <v>15117.38956256408</v>
       </c>
       <c r="C60" t="n">
-        <v>4979.903475601912</v>
+        <v>4132.132760090811</v>
       </c>
       <c r="D60" t="n">
-        <v>8535.868254672117</v>
+        <v>6775.606318085144</v>
       </c>
       <c r="E60" t="n">
-        <v>1106.579111669599</v>
+        <v>1466.75573468014</v>
       </c>
       <c r="F60" t="n">
-        <v>17052.68463600553</v>
+        <v>2.215717171717172</v>
       </c>
       <c r="G60" t="n">
-        <v>2.115828282828283</v>
+        <v>5167.38238148368</v>
       </c>
       <c r="H60" t="n">
-        <v>6000.467045300692</v>
+        <v>755.9056247766352</v>
       </c>
       <c r="I60" t="n">
-        <v>945.1566343303148</v>
+        <v>1294.616340339738</v>
       </c>
       <c r="J60" t="n">
-        <v>1705.121042164084</v>
-      </c>
-      <c r="K60" t="n">
-        <v>424.4031616267337</v>
-      </c>
-      <c r="L60" t="n">
-        <v>1942.936578349095</v>
+        <v>385.4728091630193</v>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="n">
-        <v>0.2401717171717172</v>
+        <v>0.5911919191919192</v>
       </c>
       <c r="B61" t="n">
-        <v>17185.19938208105</v>
+        <v>15069.99833667806</v>
       </c>
       <c r="C61" t="n">
-        <v>4976.529543450513</v>
+        <v>4113.62613918781</v>
       </c>
       <c r="D61" t="n">
-        <v>8529.540272049788</v>
+        <v>6747.114069593485</v>
       </c>
       <c r="E61" t="n">
-        <v>1106.199117141173</v>
+        <v>1461.442602273491</v>
       </c>
       <c r="F61" t="n">
-        <v>17164.95695113236</v>
+        <v>2.253919191919192</v>
       </c>
       <c r="G61" t="n">
-        <v>2.152308080808081</v>
+        <v>4941.881387492566</v>
       </c>
       <c r="H61" t="n">
-        <v>5797.311286564336</v>
+        <v>698.6528880715231</v>
       </c>
       <c r="I61" t="n">
-        <v>889.4571884029738</v>
+        <v>1241.264466159497</v>
       </c>
       <c r="J61" t="n">
-        <v>1610.99145051362</v>
-      </c>
-      <c r="K61" t="n">
-        <v>410.3922480682413</v>
-      </c>
-      <c r="L61" t="n">
-        <v>1876.893669387078</v>
+        <v>373.465180694072</v>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="n">
-        <v>0.2442424242424243</v>
+        <v>0.6012121212121212</v>
       </c>
       <c r="B62" t="n">
-        <v>17172.7296123314</v>
+        <v>15021.91380518857</v>
       </c>
       <c r="C62" t="n">
-        <v>4973.109181718442</v>
+        <v>4096.662004668083</v>
       </c>
       <c r="D62" t="n">
-        <v>8523.123557967825</v>
+        <v>6718.635844035358</v>
       </c>
       <c r="E62" t="n">
-        <v>1105.81363487879</v>
+        <v>1461.019197924256</v>
       </c>
       <c r="F62" t="n">
-        <v>17284.18443075452</v>
+        <v>2.292121212121212</v>
       </c>
       <c r="G62" t="n">
-        <v>2.188787878787879</v>
+        <v>4719.909193446357</v>
       </c>
       <c r="H62" t="n">
-        <v>5597.869001849896</v>
+        <v>646.58517187158</v>
       </c>
       <c r="I62" t="n">
-        <v>836.2172840588186</v>
+        <v>1178.600461990043</v>
       </c>
       <c r="J62" t="n">
-        <v>1520.844022924488</v>
-      </c>
-      <c r="K62" t="n">
-        <v>396.7652049677255</v>
-      </c>
-      <c r="L62" t="n">
-        <v>1811.858221489877</v>
+        <v>361.575842607851</v>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="n">
-        <v>0.2483131313131313</v>
+        <v>0.6112323232323232</v>
       </c>
       <c r="B63" t="n">
-        <v>17160.1987889064</v>
+        <v>14973.13040852219</v>
       </c>
       <c r="C63" t="n">
-        <v>4969.641992675683</v>
+        <v>4081.477005996694</v>
       </c>
       <c r="D63" t="n">
-        <v>8516.617372685332</v>
+        <v>6690.178198878803</v>
       </c>
       <c r="E63" t="n">
-        <v>1105.422630126018</v>
+        <v>1485.173931308217</v>
       </c>
       <c r="F63" t="n">
-        <v>17409.85912748707</v>
+        <v>2.330323232323232</v>
       </c>
       <c r="G63" t="n">
-        <v>2.225267676767677</v>
+        <v>4514.802361689698</v>
       </c>
       <c r="H63" t="n">
-        <v>5402.126721730971</v>
+        <v>599.994950331968</v>
       </c>
       <c r="I63" t="n">
-        <v>785.4713317538752</v>
+        <v>1109.0112526735</v>
       </c>
       <c r="J63" t="n">
-        <v>1434.659820965619</v>
-      </c>
-      <c r="K63" t="n">
-        <v>383.4979395614874</v>
-      </c>
-      <c r="L63" t="n">
-        <v>1747.740721111852</v>
+        <v>349.836612019833</v>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="n">
-        <v>0.2523838383838384</v>
+        <v>0.6212525252525252</v>
       </c>
       <c r="B64" t="n">
-        <v>17147.60669790725</v>
+        <v>14923.64536891172</v>
       </c>
       <c r="C64" t="n">
-        <v>4966.127578592221</v>
+        <v>4067.9612342234</v>
       </c>
       <c r="D64" t="n">
-        <v>8510.02097646141</v>
+        <v>6661.747691591852</v>
       </c>
       <c r="E64" t="n">
-        <v>1105.026068126427</v>
+        <v>1512.839621025197</v>
       </c>
       <c r="F64" t="n">
-        <v>17541.47309394505</v>
+        <v>2.368525252525253</v>
       </c>
       <c r="G64" t="n">
-        <v>2.261747474747475</v>
+        <v>4324.431232072227</v>
       </c>
       <c r="H64" t="n">
-        <v>5210.070976781145</v>
+        <v>559.520212849396</v>
       </c>
       <c r="I64" t="n">
-        <v>737.2537419441667</v>
+        <v>1040.665995795866</v>
       </c>
       <c r="J64" t="n">
-        <v>1352.398686469938</v>
-      </c>
-      <c r="K64" t="n">
-        <v>370.5663590858279</v>
-      </c>
-      <c r="L64" t="n">
-        <v>1684.451654707363</v>
+        <v>338.2231844783784</v>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="n">
-        <v>0.2564545454545455</v>
+        <v>0.6312727272727272</v>
       </c>
       <c r="B65" t="n">
-        <v>17134.95312543514</v>
+        <v>14873.66757423497</v>
       </c>
       <c r="C65" t="n">
-        <v>4962.565541738041</v>
+        <v>4055.824265103875</v>
       </c>
       <c r="D65" t="n">
-        <v>8503.333629555167</v>
+        <v>6633.350879642547</v>
       </c>
       <c r="E65" t="n">
-        <v>1104.623914123585</v>
+        <v>1523.290632057727</v>
       </c>
       <c r="F65" t="n">
-        <v>17678.51838274348</v>
+        <v>2.406727272727273</v>
       </c>
       <c r="G65" t="n">
-        <v>2.298227272727273</v>
+        <v>4145.017913924275</v>
       </c>
       <c r="H65" t="n">
-        <v>5021.688297574018</v>
+        <v>526.2829669933523</v>
       </c>
       <c r="I65" t="n">
-        <v>691.5989250857187</v>
+        <v>977.144225840202</v>
       </c>
       <c r="J65" t="n">
-        <v>1274.020461270376</v>
-      </c>
-      <c r="K65" t="n">
-        <v>357.9463707770483</v>
-      </c>
-      <c r="L65" t="n">
-        <v>1621.90150873077</v>
+        <v>326.7630252781867</v>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="n">
-        <v>0.2605252525252525</v>
+        <v>0.6412929292929292</v>
       </c>
       <c r="B66" t="n">
-        <v>17122.23785759123</v>
+        <v>14823.31729563667</v>
       </c>
       <c r="C66" t="n">
-        <v>4958.95548438313</v>
+        <v>4044.774534678462</v>
       </c>
       <c r="D66" t="n">
-        <v>8496.554592225704</v>
+        <v>6604.99432049892</v>
       </c>
       <c r="E66" t="n">
-        <v>1104.216133361062</v>
+        <v>1531.3813711821</v>
       </c>
       <c r="F66" t="n">
-        <v>17820.48704649743</v>
+        <v>2.444929292929293</v>
       </c>
       <c r="G66" t="n">
-        <v>2.334707070707071</v>
+        <v>3979.458238212269</v>
       </c>
       <c r="H66" t="n">
-        <v>4836.965214683178</v>
+        <v>497.7247741821901</v>
       </c>
       <c r="I66" t="n">
-        <v>648.5412916345548</v>
+        <v>914.9367496329404</v>
       </c>
       <c r="J66" t="n">
-        <v>1199.48498719986</v>
-      </c>
-      <c r="K66" t="n">
-        <v>345.6138818714495</v>
-      </c>
-      <c r="L66" t="n">
-        <v>1560.000769636433</v>
+        <v>315.496436776778</v>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="n">
-        <v>0.2645959595959596</v>
+        <v>0.6513131313131313</v>
       </c>
       <c r="B67" t="n">
-        <v>17109.46068047673</v>
+        <v>14772.57696318406</v>
       </c>
       <c r="C67" t="n">
-        <v>4955.297008797474</v>
+        <v>4034.520478987506</v>
       </c>
       <c r="D67" t="n">
-        <v>8489.683124732124</v>
+        <v>6576.685822186097</v>
       </c>
       <c r="E67" t="n">
-        <v>1103.802691082427</v>
+        <v>1538.015425548272</v>
       </c>
       <c r="F67" t="n">
-        <v>17966.87113782191</v>
+        <v>2.483131313131313</v>
       </c>
       <c r="G67" t="n">
-        <v>2.371186868686869</v>
+        <v>3831.721125018124</v>
       </c>
       <c r="H67" t="n">
-        <v>4655.888258682217</v>
+        <v>468.9112471582544</v>
       </c>
       <c r="I67" t="n">
-        <v>608.1152520466998</v>
+        <v>852.8057634318183</v>
       </c>
       <c r="J67" t="n">
-        <v>1128.752106091319</v>
-      </c>
-      <c r="K67" t="n">
-        <v>333.5447996053325</v>
-      </c>
-      <c r="L67" t="n">
-        <v>1498.65992387871</v>
+        <v>304.4570188598685</v>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="n">
-        <v>0.2686666666666667</v>
+        <v>0.6613333333333333</v>
       </c>
       <c r="B68" t="n">
-        <v>17096.62138019282</v>
+        <v>14721.42900694442</v>
       </c>
       <c r="C68" t="n">
-        <v>4951.589717251055</v>
+        <v>4024.770534071349</v>
       </c>
       <c r="D68" t="n">
-        <v>8482.718487333532</v>
+        <v>6549.720159286328</v>
       </c>
       <c r="E68" t="n">
-        <v>1103.383552531249</v>
+        <v>1540.624363517733</v>
       </c>
       <c r="F68" t="n">
-        <v>18117.16270933198</v>
+        <v>2.521333333333333</v>
       </c>
       <c r="G68" t="n">
-        <v>2.407666666666667</v>
+        <v>3704.369777440615</v>
       </c>
       <c r="H68" t="n">
-        <v>4478.443960144731</v>
+        <v>435.8453181693327</v>
       </c>
       <c r="I68" t="n">
-        <v>570.3380362607974</v>
+        <v>789.3929425285173</v>
       </c>
       <c r="J68" t="n">
-        <v>1061.781659777681</v>
-      </c>
-      <c r="K68" t="n">
-        <v>321.7150312149987</v>
-      </c>
-      <c r="L68" t="n">
-        <v>1438.44682559321</v>
+        <v>293.5609159343476</v>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="n">
-        <v>0.2727373737373738</v>
+        <v>0.6713535353535353</v>
       </c>
       <c r="B69" t="n">
-        <v>17083.71974284068</v>
+        <v>14669.85585698502</v>
       </c>
       <c r="C69" t="n">
-        <v>4947.83321201386</v>
+        <v>4015.233135970337</v>
       </c>
       <c r="D69" t="n">
-        <v>8475.659940289032</v>
+        <v>6524.973049386299</v>
       </c>
       <c r="E69" t="n">
-        <v>1102.958682951096</v>
+        <v>1540.679633184633</v>
       </c>
       <c r="F69" t="n">
-        <v>18270.85381364267</v>
+        <v>2.559535353535354</v>
       </c>
       <c r="G69" t="n">
-        <v>2.444146464646465</v>
+        <v>3583.08221904414</v>
       </c>
       <c r="H69" t="n">
-        <v>4304.618849644307</v>
+        <v>400.2769136148583</v>
       </c>
       <c r="I69" t="n">
-        <v>534.1995054759634</v>
+        <v>724.2983043076241</v>
       </c>
       <c r="J69" t="n">
-        <v>998.5334900918735</v>
-      </c>
-      <c r="K69" t="n">
-        <v>310.1004839367489</v>
-      </c>
-      <c r="L69" t="n">
-        <v>1379.996528294223</v>
+        <v>282.6871266466695</v>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="n">
-        <v>0.2768080808080808</v>
+        <v>0.6813737373737373</v>
       </c>
       <c r="B70" t="n">
-        <v>17070.7555545215</v>
+        <v>14617.83994337311</v>
       </c>
       <c r="C70" t="n">
-        <v>4944.027095355874</v>
+        <v>4005.616720724813</v>
       </c>
       <c r="D70" t="n">
-        <v>8468.506743857724</v>
+        <v>6502.056751385697</v>
       </c>
       <c r="E70" t="n">
-        <v>1102.528047585539</v>
+        <v>1544.3889504317</v>
       </c>
       <c r="F70" t="n">
-        <v>18427.43650336902</v>
+        <v>2.597737373737374</v>
       </c>
       <c r="G70" t="n">
-        <v>2.480626262626263</v>
+        <v>3451.510711856507</v>
       </c>
       <c r="H70" t="n">
-        <v>4134.399457754545</v>
+        <v>365.2772061201799</v>
       </c>
       <c r="I70" t="n">
-        <v>499.1845278238376</v>
+        <v>662.8628014609826</v>
       </c>
       <c r="J70" t="n">
-        <v>938.9674388668265</v>
-      </c>
-      <c r="K70" t="n">
-        <v>298.6770650068843</v>
-      </c>
-      <c r="L70" t="n">
-        <v>1323.286718240088</v>
+        <v>272.0013071915029</v>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="n">
-        <v>0.2808787878787879</v>
+        <v>0.6913939393939393</v>
       </c>
       <c r="B71" t="n">
-        <v>17057.72860133647</v>
+        <v>14565.36369617596</v>
       </c>
       <c r="C71" t="n">
-        <v>4940.170969547084</v>
+        <v>3995.629724375121</v>
       </c>
       <c r="D71" t="n">
-        <v>8461.258158298715</v>
+        <v>6480.583524184202</v>
       </c>
       <c r="E71" t="n">
-        <v>1102.091611678145</v>
+        <v>1579.896534944971</v>
       </c>
       <c r="F71" t="n">
-        <v>18588.36354873814</v>
+        <v>2.635939393939394</v>
       </c>
       <c r="G71" t="n">
-        <v>2.517106060606061</v>
+        <v>3299.187942412316</v>
       </c>
       <c r="H71" t="n">
-        <v>3967.772315049027</v>
+        <v>333.5817769084395</v>
       </c>
       <c r="I71" t="n">
-        <v>465.4204393078394</v>
+        <v>616.5117560055112</v>
       </c>
       <c r="J71" t="n">
-        <v>883.0433479354665</v>
-      </c>
-      <c r="K71" t="n">
-        <v>287.4238045707042</v>
-      </c>
-      <c r="L71" t="n">
-        <v>1268.295033236739</v>
+        <v>261.468136098957</v>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="n">
-        <v>0.284949494949495</v>
+        <v>0.7014141414141414</v>
       </c>
       <c r="B72" t="n">
-        <v>17044.63866938678</v>
+        <v>14512.40954546084</v>
       </c>
       <c r="C72" t="n">
-        <v>4936.264436857473</v>
+        <v>3984.980582961605</v>
       </c>
       <c r="D72" t="n">
-        <v>8453.913443871104</v>
+        <v>6460.165626681503</v>
       </c>
       <c r="E72" t="n">
-        <v>1101.649340472484</v>
+        <v>1610.985781256536</v>
       </c>
       <c r="F72" t="n">
-        <v>18766.09283275963</v>
+        <v>2.674141414141414</v>
       </c>
       <c r="G72" t="n">
-        <v>2.553585858585858</v>
+        <v>3135.381249145218</v>
       </c>
       <c r="H72" t="n">
-        <v>3804.723952101355</v>
+        <v>305.4802411403003</v>
       </c>
       <c r="I72" t="n">
-        <v>433.034575931389</v>
+        <v>585.7249283161256</v>
       </c>
       <c r="J72" t="n">
-        <v>830.5937814844882</v>
-      </c>
-      <c r="K72" t="n">
-        <v>276.4601680572063</v>
-      </c>
-      <c r="L72" t="n">
-        <v>1214.999111090116</v>
+        <v>254.4141811019514</v>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="n">
-        <v>0.2890202020202021</v>
+        <v>0.7114343434343434</v>
       </c>
       <c r="B73" t="n">
-        <v>17031.48554477359</v>
+        <v>14458.95992129501</v>
       </c>
       <c r="C73" t="n">
-        <v>4932.307099557028</v>
+        <v>3973.377732524609</v>
       </c>
       <c r="D73" t="n">
-        <v>8446.471860834001</v>
+        <v>6440.415317777281</v>
       </c>
       <c r="E73" t="n">
-        <v>1101.201199212125</v>
+        <v>1613.232915858425</v>
       </c>
       <c r="F73" t="n">
-        <v>18960.61015076544</v>
+        <v>2.712343434343434</v>
       </c>
       <c r="G73" t="n">
-        <v>2.590065656565657</v>
+        <v>2970.3631868897</v>
       </c>
       <c r="H73" t="n">
-        <v>3645.241932816964</v>
+        <v>281.757981395898</v>
       </c>
       <c r="I73" t="n">
-        <v>402.1542736979057</v>
+        <v>550.2194658124257</v>
       </c>
       <c r="J73" t="n">
-        <v>779.8402755992595</v>
-      </c>
-      <c r="K73" t="n">
-        <v>265.8433217966181</v>
-      </c>
-      <c r="L73" t="n">
-        <v>1163.376589606157</v>
+        <v>248.8330929640156</v>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="n">
-        <v>0.2930909090909091</v>
+        <v>0.7214545454545453</v>
       </c>
       <c r="B74" t="n">
-        <v>17018.26901359811</v>
+        <v>14404.99725374574</v>
       </c>
       <c r="C74" t="n">
-        <v>4928.298559915733</v>
+        <v>3960.529609104477</v>
       </c>
       <c r="D74" t="n">
-        <v>8438.932669446502</v>
+        <v>6420.94485637122</v>
       </c>
       <c r="E74" t="n">
-        <v>1100.747153140637</v>
+        <v>1613.173046351256</v>
       </c>
       <c r="F74" t="n">
-        <v>19169.12210254572</v>
+        <v>2.750545454545454</v>
       </c>
       <c r="G74" t="n">
-        <v>2.626545454545455</v>
+        <v>2814.298981017003</v>
       </c>
       <c r="H74" t="n">
-        <v>3489.920921284693</v>
+        <v>262.8391196248571</v>
       </c>
       <c r="I74" t="n">
-        <v>372.9068686108097</v>
+        <v>510.9723959970775</v>
       </c>
       <c r="J74" t="n">
-        <v>730.3797296396004</v>
-      </c>
-      <c r="K74" t="n">
-        <v>255.5536786798391</v>
-      </c>
-      <c r="L74" t="n">
-        <v>1113.4051065908</v>
+        <v>238.2156492715816</v>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="n">
-        <v>0.2971616161616162</v>
+        <v>0.7314747474747474</v>
       </c>
       <c r="B75" t="n">
-        <v>17004.98886196153</v>
+        <v>14350.50397288028</v>
       </c>
       <c r="C75" t="n">
-        <v>4924.238420203574</v>
+        <v>3946.144648741553</v>
       </c>
       <c r="D75" t="n">
-        <v>8431.295129967717</v>
+        <v>6401.366501363006</v>
       </c>
       <c r="E75" t="n">
-        <v>1100.287167501589</v>
+        <v>1635.968461579117</v>
       </c>
       <c r="F75" t="n">
-        <v>19388.83528789066</v>
+        <v>2.788747474747475</v>
       </c>
       <c r="G75" t="n">
-        <v>2.663025252525252</v>
+        <v>2672.191127836994</v>
       </c>
       <c r="H75" t="n">
-        <v>3339.26627477472</v>
+        <v>245.6545040471109</v>
       </c>
       <c r="I75" t="n">
-        <v>345.419696673521</v>
+        <v>472.5787655883138</v>
       </c>
       <c r="J75" t="n">
-        <v>682.41554800865</v>
-      </c>
-      <c r="K75" t="n">
-        <v>245.5716515977686</v>
-      </c>
-      <c r="L75" t="n">
-        <v>1065.062299849983</v>
+        <v>223.9786761800931</v>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="n">
-        <v>0.3012323232323232</v>
+        <v>0.7414949494949494</v>
       </c>
       <c r="B76" t="n">
-        <v>16991.64487596502</v>
+        <v>14295.46250876591</v>
       </c>
       <c r="C76" t="n">
-        <v>4920.126282690537</v>
+        <v>3929.931287476181</v>
       </c>
       <c r="D76" t="n">
-        <v>8423.558502656748</v>
+        <v>6381.292511652322</v>
       </c>
       <c r="E76" t="n">
-        <v>1099.82120753855</v>
+        <v>1689.163032759605</v>
       </c>
       <c r="F76" t="n">
-        <v>19616.95630659041</v>
+        <v>2.826949494949495</v>
       </c>
       <c r="G76" t="n">
-        <v>2.699505050505051</v>
+        <v>2538.924397560447</v>
       </c>
       <c r="H76" t="n">
-        <v>3193.270378824334</v>
+        <v>228.2900078845786</v>
       </c>
       <c r="I76" t="n">
-        <v>319.820093889459</v>
+        <v>436.9980728369177</v>
       </c>
       <c r="J76" t="n">
-        <v>636.1511351095457</v>
-      </c>
-      <c r="K76" t="n">
-        <v>235.8776534413057</v>
-      </c>
-      <c r="L76" t="n">
-        <v>1018.325807189644</v>
+        <v>210.3697199534541</v>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="n">
-        <v>0.3053030303030304</v>
+        <v>0.7515151515151515</v>
       </c>
       <c r="B77" t="n">
-        <v>16978.23684170976</v>
+        <v>14239.85529146988</v>
       </c>
       <c r="C77" t="n">
-        <v>4915.961749646605</v>
+        <v>3911.617389382035</v>
       </c>
       <c r="D77" t="n">
-        <v>8415.722047772695</v>
+        <v>6360.335146138854</v>
       </c>
       <c r="E77" t="n">
-        <v>1099.34923849509</v>
+        <v>1711.944624039759</v>
       </c>
       <c r="F77" t="n">
-        <v>19850.69175843518</v>
+        <v>2.865151515151515</v>
       </c>
       <c r="G77" t="n">
-        <v>2.735984848484848</v>
+        <v>2417.039901464518</v>
       </c>
       <c r="H77" t="n">
-        <v>3051.925618970831</v>
+        <v>209.4833862566353</v>
       </c>
       <c r="I77" t="n">
-        <v>296.235396262044</v>
+        <v>403.1696277428924</v>
       </c>
       <c r="J77" t="n">
-        <v>591.7898953454272</v>
-      </c>
-      <c r="K77" t="n">
-        <v>226.4520971013499</v>
-      </c>
-      <c r="L77" t="n">
-        <v>973.1732664157212</v>
+        <v>199.6109017761971</v>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="n">
-        <v>0.3093737373737374</v>
+        <v>0.7615353535353535</v>
       </c>
       <c r="B78" t="n">
-        <v>16964.76454529696</v>
+        <v>14183.66475105946</v>
       </c>
       <c r="C78" t="n">
-        <v>4911.744423341766</v>
+        <v>3891.248588267115</v>
       </c>
       <c r="D78" t="n">
-        <v>8407.785025574665</v>
+        <v>6338.106663722284</v>
       </c>
       <c r="E78" t="n">
-        <v>1098.871225614776</v>
+        <v>1730.135545966722</v>
       </c>
       <c r="F78" t="n">
-        <v>20087.2482432151</v>
+        <v>2.903353535353535</v>
       </c>
       <c r="G78" t="n">
-        <v>2.772464646464647</v>
+        <v>2309.414498098976</v>
       </c>
       <c r="H78" t="n">
-        <v>2915.224380751501</v>
+        <v>189.9290565905605</v>
       </c>
       <c r="I78" t="n">
-        <v>274.7929397946953</v>
+        <v>369.9237700030006</v>
       </c>
       <c r="J78" t="n">
-        <v>549.5352331194318</v>
-      </c>
-      <c r="K78" t="n">
-        <v>217.2753954688</v>
-      </c>
-      <c r="L78" t="n">
-        <v>929.5823153341519</v>
+        <v>189.3321371289318</v>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="n">
-        <v>0.3134444444444445</v>
+        <v>0.7715555555555556</v>
       </c>
       <c r="B79" t="n">
-        <v>16951.22777282779</v>
+        <v>14126.87331760192</v>
       </c>
       <c r="C79" t="n">
-        <v>4907.473906046005</v>
+        <v>3869.097155716702</v>
       </c>
       <c r="D79" t="n">
-        <v>8399.746696321761</v>
+        <v>6314.219323302298</v>
       </c>
       <c r="E79" t="n">
-        <v>1098.387134141179</v>
+        <v>1747.077478970985</v>
       </c>
       <c r="F79" t="n">
-        <v>20323.83236072036</v>
+        <v>2.941555555555555</v>
       </c>
       <c r="G79" t="n">
-        <v>2.808944444444445</v>
+        <v>2215.083674100887</v>
       </c>
       <c r="H79" t="n">
-        <v>2783.15904970364</v>
+        <v>170.7317112557266</v>
       </c>
       <c r="I79" t="n">
-        <v>255.6116965096366</v>
+        <v>335.1653979708791</v>
       </c>
       <c r="J79" t="n">
-        <v>509.5905528346987</v>
-      </c>
-      <c r="K79" t="n">
-        <v>208.3279614345556</v>
-      </c>
-      <c r="L79" t="n">
-        <v>887.5305917508744</v>
+        <v>179.7926057226354</v>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="n">
-        <v>0.3175151515151515</v>
+        <v>0.7815757575757575</v>
       </c>
       <c r="B80" t="n">
-        <v>16937.62631040344</v>
+        <v>14069.46342116452</v>
       </c>
       <c r="C80" t="n">
-        <v>4903.149800029305</v>
+        <v>3845.43911703386</v>
       </c>
       <c r="D80" t="n">
-        <v>8391.606320273084</v>
+        <v>6288.28538377858</v>
       </c>
       <c r="E80" t="n">
-        <v>1097.896929317867</v>
+        <v>1762.294460982843</v>
       </c>
       <c r="F80" t="n">
-        <v>20557.65071074113</v>
+        <v>2.979757575757576</v>
       </c>
       <c r="G80" t="n">
-        <v>2.845424242424242</v>
+        <v>2126.832780534563</v>
       </c>
       <c r="H80" t="n">
-        <v>2655.722011364539</v>
+        <v>153.0062146483001</v>
       </c>
       <c r="I80" t="n">
-        <v>237.7079326196208</v>
+        <v>299.544504318835</v>
       </c>
       <c r="J80" t="n">
-        <v>472.1592588943668</v>
-      </c>
-      <c r="K80" t="n">
-        <v>199.5902078895159</v>
-      </c>
-      <c r="L80" t="n">
-        <v>846.9957334718274</v>
+        <v>170.5156098226244</v>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="n">
-        <v>0.3215858585858586</v>
+        <v>0.7915959595959595</v>
       </c>
       <c r="B81" t="n">
-        <v>16923.9599441251</v>
+        <v>14011.41749181453</v>
       </c>
       <c r="C81" t="n">
-        <v>4898.771707561653</v>
+        <v>3820.550497521654</v>
       </c>
       <c r="D81" t="n">
-        <v>8383.36315768774</v>
+        <v>6259.917104050814</v>
       </c>
       <c r="E81" t="n">
-        <v>1097.400576388409</v>
+        <v>1774.100159156878</v>
       </c>
       <c r="F81" t="n">
-        <v>20785.90989306758</v>
+        <v>3.017959595959596</v>
       </c>
       <c r="G81" t="n">
-        <v>2.881904040404041</v>
+        <v>2037.163311259573</v>
       </c>
       <c r="H81" t="n">
-        <v>2532.905651271492</v>
+        <v>137.7333748374841</v>
       </c>
       <c r="I81" t="n">
-        <v>220.3856995655879</v>
+        <v>271.0438965936635</v>
       </c>
       <c r="J81" t="n">
-        <v>437.4447557015736</v>
-      </c>
-      <c r="K81" t="n">
-        <v>191.04254772458</v>
-      </c>
-      <c r="L81" t="n">
-        <v>807.8777760480136</v>
+        <v>161.409143799711</v>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="n">
-        <v>0.3256565656565657</v>
+        <v>0.8016161616161616</v>
       </c>
       <c r="B82" t="n">
-        <v>16910.22846009394</v>
+        <v>13952.7179596192</v>
       </c>
       <c r="C82" t="n">
-        <v>4894.339230913034</v>
+        <v>3794.707322483148</v>
       </c>
       <c r="D82" t="n">
-        <v>8375.016468824833</v>
+        <v>6228.726743018683</v>
       </c>
       <c r="E82" t="n">
-        <v>1096.898040596375</v>
+        <v>1787.198483521729</v>
       </c>
       <c r="F82" t="n">
-        <v>21005.77994315115</v>
+        <v>3.056161616161616</v>
       </c>
       <c r="G82" t="n">
-        <v>2.918383838383838</v>
+        <v>1938.141893656753</v>
       </c>
       <c r="H82" t="n">
-        <v>2414.702354961794</v>
+        <v>125.3795000999774</v>
       </c>
       <c r="I82" t="n">
-        <v>203.7098777179031</v>
+        <v>251.2623417521364</v>
       </c>
       <c r="J82" t="n">
-        <v>405.6504476594587</v>
-      </c>
-      <c r="K82" t="n">
-        <v>182.6653938306474</v>
-      </c>
-      <c r="L82" t="n">
-        <v>770.0235376876586</v>
+        <v>152.4897495572316</v>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="n">
-        <v>0.3297272727272728</v>
+        <v>0.8116363636363636</v>
       </c>
       <c r="B83" t="n">
-        <v>16896.43164441117</v>
+        <v>13893.34725464581</v>
       </c>
       <c r="C83" t="n">
-        <v>4889.851972353434</v>
+        <v>3768.185617221406</v>
       </c>
       <c r="D83" t="n">
-        <v>8366.565513943462</v>
+        <v>6194.52064336947</v>
       </c>
       <c r="E83" t="n">
-        <v>1096.389287185333</v>
+        <v>1824.871086109558</v>
       </c>
       <c r="F83" t="n">
-        <v>21190.32948085489</v>
+        <v>3.094363636363636</v>
       </c>
       <c r="G83" t="n">
-        <v>2.954863636363636</v>
+        <v>1826.532912938954</v>
       </c>
       <c r="H83" t="n">
-        <v>2301.104507972736</v>
+        <v>115.6418888853846</v>
       </c>
       <c r="I83" t="n">
-        <v>187.7453474469306</v>
+        <v>232.5357260987998</v>
       </c>
       <c r="J83" t="n">
-        <v>376.9797391711596</v>
-      </c>
-      <c r="K83" t="n">
-        <v>174.4714240604437</v>
-      </c>
-      <c r="L83" t="n">
-        <v>733.4407693564702</v>
+        <v>143.6491934676217</v>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="n">
-        <v>0.3337979797979798</v>
+        <v>0.8216565656565656</v>
       </c>
       <c r="B84" t="n">
-        <v>16882.56928317795</v>
+        <v>13833.28787590205</v>
       </c>
       <c r="C84" t="n">
-        <v>4885.309534152837</v>
+        <v>3741.261407039493</v>
       </c>
       <c r="D84" t="n">
-        <v>8358.009553302736</v>
+        <v>6158.077085791596</v>
       </c>
       <c r="E84" t="n">
-        <v>1095.874281398852</v>
+        <v>1904.030487530659</v>
       </c>
       <c r="F84" t="n">
-        <v>21325.24424835535</v>
+        <v>3.132565656565657</v>
       </c>
       <c r="G84" t="n">
-        <v>2.991343434343434</v>
+        <v>1713.103206741812</v>
       </c>
       <c r="H84" t="n">
-        <v>2192.104495841611</v>
+        <v>106.2774103524582</v>
       </c>
       <c r="I84" t="n">
-        <v>172.5569891230358</v>
+        <v>213.7254253503126</v>
       </c>
       <c r="J84" t="n">
-        <v>351.391203920645</v>
-      </c>
-      <c r="K84" t="n">
-        <v>166.5464348355192</v>
-      </c>
-      <c r="L84" t="n">
-        <v>698.1411587908497</v>
+        <v>134.969557523526</v>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="n">
-        <v>0.3378686868686869</v>
+        <v>0.8316767676767676</v>
       </c>
       <c r="B85" t="n">
-        <v>16868.64116249548</v>
+        <v>13772.81245603159</v>
       </c>
       <c r="C85" t="n">
-        <v>4880.711518581231</v>
+        <v>3714.210717240474</v>
       </c>
       <c r="D85" t="n">
-        <v>8349.347847161756</v>
+        <v>6119.722234412954</v>
       </c>
       <c r="E85" t="n">
-        <v>1095.352988480502</v>
+        <v>1932.889415544382</v>
       </c>
       <c r="F85" t="n">
-        <v>21421.12693994663</v>
+        <v>3.170767676767677</v>
       </c>
       <c r="G85" t="n">
-        <v>3.027823232323232</v>
+        <v>1610.052584429029</v>
       </c>
       <c r="H85" t="n">
-        <v>2087.694704105712</v>
+        <v>96.87097535924988</v>
       </c>
       <c r="I85" t="n">
-        <v>158.2096831165831</v>
+        <v>194.8253758923778</v>
       </c>
       <c r="J85" t="n">
-        <v>326.9900133994173</v>
-      </c>
-      <c r="K85" t="n">
-        <v>158.8983259023311</v>
-      </c>
-      <c r="L85" t="n">
-        <v>664.1363937271971</v>
+        <v>126.4005032355901</v>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="n">
-        <v>0.341939393939394</v>
+        <v>0.8416969696969696</v>
       </c>
       <c r="B86" t="n">
-        <v>16854.64706846495</v>
+        <v>13712.17283577094</v>
       </c>
       <c r="C86" t="n">
-        <v>4876.057527908597</v>
+        <v>3687.309573127413</v>
       </c>
       <c r="D86" t="n">
-        <v>8340.579655779624</v>
+        <v>6079.684500554486</v>
       </c>
       <c r="E86" t="n">
-        <v>1094.825373673852</v>
+        <v>1944.734230604351</v>
       </c>
       <c r="F86" t="n">
-        <v>21488.58024992284</v>
+        <v>3.208969696969697</v>
       </c>
       <c r="G86" t="n">
-        <v>3.064303030303031</v>
+        <v>1527.576844643447</v>
       </c>
       <c r="H86" t="n">
-        <v>1987.867518302332</v>
+        <v>87.24599973833477</v>
       </c>
       <c r="I86" t="n">
-        <v>144.7683097979373</v>
+        <v>175.931475552425</v>
       </c>
       <c r="J86" t="n">
-        <v>303.4034504206902</v>
-      </c>
-      <c r="K86" t="n">
-        <v>151.529134137815</v>
-      </c>
-      <c r="L86" t="n">
-        <v>631.4381619019134</v>
+        <v>117.9637539131279</v>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="n">
-        <v>0.346010101010101</v>
+        <v>0.8517171717171717</v>
       </c>
       <c r="B87" t="n">
-        <v>16840.58678718755</v>
+        <v>13651.34641961146</v>
       </c>
       <c r="C87" t="n">
-        <v>4871.347164404924</v>
+        <v>3660.834000003373</v>
       </c>
       <c r="D87" t="n">
-        <v>8331.704239415445</v>
+        <v>6038.192295537136</v>
       </c>
       <c r="E87" t="n">
-        <v>1094.29140222247</v>
+        <v>1979.009302762866</v>
       </c>
       <c r="F87" t="n">
-        <v>21538.20687257808</v>
+        <v>3.247171717171717</v>
       </c>
       <c r="G87" t="n">
-        <v>3.100782828282828</v>
+        <v>1455.318962913013</v>
       </c>
       <c r="H87" t="n">
-        <v>1892.615323968767</v>
+        <v>77.52250121130739</v>
       </c>
       <c r="I87" t="n">
-        <v>132.2977495374635</v>
+        <v>156.744175073762</v>
       </c>
       <c r="J87" t="n">
-        <v>280.7167906634669</v>
-      </c>
-      <c r="K87" t="n">
-        <v>144.4408964189064</v>
-      </c>
-      <c r="L87" t="n">
-        <v>600.0581510513997</v>
+        <v>109.6287373017733</v>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="n">
-        <v>0.3500808080808081</v>
+        <v>0.8617373737373737</v>
       </c>
       <c r="B88" t="n">
-        <v>16826.46010476444</v>
+        <v>13590.31061204448</v>
       </c>
       <c r="C88" t="n">
-        <v>4866.580030340196</v>
+        <v>3635.06002317142</v>
       </c>
       <c r="D88" t="n">
-        <v>8322.720858328323</v>
+        <v>5995.474030681844</v>
       </c>
       <c r="E88" t="n">
-        <v>1093.751039369925</v>
+        <v>2080.930159668395</v>
       </c>
       <c r="F88" t="n">
-        <v>21580.60950220647</v>
+        <v>3.285373737373738</v>
       </c>
       <c r="G88" t="n">
-        <v>3.137262626262626</v>
+        <v>1386.083840700585</v>
       </c>
       <c r="H88" t="n">
-        <v>1801.930506642306</v>
+        <v>67.88367558987956</v>
       </c>
       <c r="I88" t="n">
-        <v>120.8628827055261</v>
+        <v>137.2259195127295</v>
       </c>
       <c r="J88" t="n">
-        <v>259.0153098067496</v>
-      </c>
-      <c r="K88" t="n">
-        <v>137.6356496225404</v>
-      </c>
-      <c r="L88" t="n">
-        <v>570.0080489120558</v>
+        <v>101.3562338255173</v>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="n">
-        <v>0.3541515151515152</v>
+        <v>0.8717575757575757</v>
       </c>
       <c r="B89" t="n">
-        <v>16812.26680729683</v>
+        <v>13529.04281756135</v>
       </c>
       <c r="C89" t="n">
-        <v>4861.755727984397</v>
+        <v>3610.263667934617</v>
       </c>
       <c r="D89" t="n">
-        <v>8313.628772777363</v>
+        <v>5951.758117309556</v>
       </c>
       <c r="E89" t="n">
-        <v>1093.204250359787</v>
+        <v>2165.665238697496</v>
       </c>
       <c r="F89" t="n">
-        <v>21626.39083310209</v>
+        <v>3.323575757575758</v>
       </c>
       <c r="G89" t="n">
-        <v>3.173742424242424</v>
+        <v>1315.632418782857</v>
       </c>
       <c r="H89" t="n">
-        <v>1715.805451860245</v>
+        <v>58.76445057540155</v>
       </c>
       <c r="I89" t="n">
-        <v>110.5285896724903</v>
+        <v>119.9186705267371</v>
       </c>
       <c r="J89" t="n">
-        <v>238.3842835295416</v>
-      </c>
-      <c r="K89" t="n">
-        <v>131.1154306256527</v>
-      </c>
-      <c r="L89" t="n">
-        <v>541.2995432202831</v>
+        <v>93.16459976750272</v>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="n">
-        <v>0.3582222222222223</v>
+        <v>0.8817777777777778</v>
       </c>
       <c r="B90" t="n">
-        <v>16798.00668088589</v>
+        <v>13467.52044065342</v>
       </c>
       <c r="C90" t="n">
-        <v>4856.873859607515</v>
+        <v>3586.720959596031</v>
       </c>
       <c r="D90" t="n">
-        <v>8304.427243021664</v>
+        <v>5907.272966741211</v>
       </c>
       <c r="E90" t="n">
-        <v>1092.651000435625</v>
+        <v>2222.566289660698</v>
       </c>
       <c r="F90" t="n">
-        <v>21686.15355955906</v>
+        <v>3.361777777777778</v>
       </c>
       <c r="G90" t="n">
-        <v>3.210222222222222</v>
+        <v>1241.239702295957</v>
       </c>
       <c r="H90" t="n">
-        <v>1634.232545159875</v>
+        <v>51.30794166844602</v>
       </c>
       <c r="I90" t="n">
-        <v>101.3588059089335</v>
+        <v>106.8787348692916</v>
       </c>
       <c r="J90" t="n">
-        <v>218.9089875108451</v>
-      </c>
-      <c r="K90" t="n">
-        <v>124.8822763051785</v>
-      </c>
-      <c r="L90" t="n">
-        <v>513.9443217124815</v>
+        <v>85.00982322534837</v>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="n">
-        <v>0.3622929292929293</v>
+        <v>0.8917979797979797</v>
       </c>
       <c r="B91" t="n">
-        <v>16783.67951163282</v>
+        <v>13405.72088581202</v>
       </c>
       <c r="C91" t="n">
-        <v>4851.934027479533</v>
+        <v>3564.707923458724</v>
       </c>
       <c r="D91" t="n">
-        <v>8295.115529320332</v>
+        <v>5862.246990297754</v>
       </c>
       <c r="E91" t="n">
-        <v>1092.091254841007</v>
+        <v>2276.879208452097</v>
       </c>
       <c r="F91" t="n">
-        <v>21770.5003758715</v>
+        <v>3.399979797979798</v>
       </c>
       <c r="G91" t="n">
-        <v>3.24670202020202</v>
+        <v>1165.208584231161</v>
       </c>
       <c r="H91" t="n">
-        <v>1557.139277882385</v>
+        <v>45.44617181746772</v>
       </c>
       <c r="I91" t="n">
-        <v>92.95453900765327</v>
+        <v>96.43911040534233</v>
       </c>
       <c r="J91" t="n">
-        <v>200.6746974296634</v>
-      </c>
-      <c r="K91" t="n">
-        <v>118.9382235380534</v>
-      </c>
-      <c r="L91" t="n">
-        <v>487.9540721250524</v>
+        <v>76.84578835356551</v>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="n">
-        <v>0.3663636363636364</v>
+        <v>0.9018181818181817</v>
       </c>
       <c r="B92" t="n">
-        <v>16769.2850856388</v>
+        <v>13343.62155752851</v>
       </c>
       <c r="C92" t="n">
-        <v>4846.935833870437</v>
+        <v>3544.490540411538</v>
       </c>
       <c r="D92" t="n">
-        <v>8285.692891932471</v>
+        <v>5816.908599300124</v>
       </c>
       <c r="E92" t="n">
-        <v>1091.524978819503</v>
+        <v>2334.962778665856</v>
       </c>
       <c r="F92" t="n">
-        <v>21890.03397633349</v>
+        <v>3.438181818181818</v>
       </c>
       <c r="G92" t="n">
-        <v>3.283181818181818</v>
+        <v>1089.235656034273</v>
       </c>
       <c r="H92" t="n">
-        <v>1482.365158722998</v>
+        <v>40.64345757565395</v>
       </c>
       <c r="I92" t="n">
-        <v>84.98751517187077</v>
+        <v>85.99887294819514</v>
       </c>
       <c r="J92" t="n">
-        <v>183.7666889649988</v>
-      </c>
-      <c r="K92" t="n">
-        <v>113.2853092012125</v>
-      </c>
-      <c r="L92" t="n">
-        <v>463.3404821943958</v>
+        <v>68.62782436413838</v>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="n">
-        <v>0.3704343434343434</v>
+        <v>0.9118383838383838</v>
       </c>
       <c r="B93" t="n">
-        <v>16754.82318900502</v>
+        <v>13281.19986029423</v>
       </c>
       <c r="C93" t="n">
-        <v>4841.878881050213</v>
+        <v>3526.016364238615</v>
       </c>
       <c r="D93" t="n">
-        <v>8276.158591117182</v>
+        <v>5771.486205069268</v>
       </c>
       <c r="E93" t="n">
-        <v>1090.952137614682</v>
+        <v>2400.233311044888</v>
       </c>
       <c r="F93" t="n">
-        <v>22055.35705523915</v>
+        <v>3.476383838383839</v>
       </c>
       <c r="G93" t="n">
-        <v>3.319661616161616</v>
+        <v>1014.930027190288</v>
       </c>
       <c r="H93" t="n">
-        <v>1408.978405553113</v>
+        <v>35.96661138278728</v>
       </c>
       <c r="I93" t="n">
-        <v>77.51284567696214</v>
+        <v>75.17383163911967</v>
       </c>
       <c r="J93" t="n">
-        <v>168.2702377958544</v>
-      </c>
-      <c r="K93" t="n">
-        <v>107.9255701715914</v>
-      </c>
-      <c r="L93" t="n">
-        <v>440.1129745721914</v>
+        <v>60.3753762820259</v>
       </c>
     </row>
     <row r="94">
       <c r="A94" t="n">
-        <v>0.3745050505050506</v>
+        <v>0.9218585858585858</v>
       </c>
       <c r="B94" t="n">
-        <v>16740.29360783266</v>
+        <v>13218.43319860052</v>
       </c>
       <c r="C94" t="n">
-        <v>4836.762771288845</v>
+        <v>3508.994272217416</v>
       </c>
       <c r="D94" t="n">
-        <v>8266.511887133571</v>
+        <v>5726.208218926125</v>
       </c>
       <c r="E94" t="n">
-        <v>1090.372696470112</v>
+        <v>2473.452724455107</v>
       </c>
       <c r="F94" t="n">
-        <v>22552.68431404932</v>
+        <v>3.514585858585859</v>
       </c>
       <c r="G94" t="n">
-        <v>3.356141414141414</v>
+        <v>944.7892983800612</v>
       </c>
       <c r="H94" t="n">
-        <v>1337.137509405224</v>
+        <v>31.35652441266736</v>
       </c>
       <c r="I94" t="n">
-        <v>70.5856417983034</v>
+        <v>64.54362507770726</v>
       </c>
       <c r="J94" t="n">
-        <v>154.2706196012331</v>
-      </c>
-      <c r="K94" t="n">
-        <v>102.8647372407218</v>
-      </c>
-      <c r="L94" t="n">
-        <v>417.8051541770399</v>
+        <v>51.92300110064566</v>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="n">
-        <v>0.3785757575757576</v>
+        <v>0.9318787878787879</v>
       </c>
       <c r="B95" t="n">
-        <v>16725.69612822291</v>
+        <v>13155.29897693872</v>
       </c>
       <c r="C95" t="n">
-        <v>4831.587106856321</v>
+        <v>3493.151488400003</v>
       </c>
       <c r="D95" t="n">
-        <v>8256.752040240743</v>
+        <v>5681.30305219164</v>
       </c>
       <c r="E95" t="n">
-        <v>1089.786620629364</v>
+        <v>2563.178431901167</v>
       </c>
       <c r="F95" t="n">
-        <v>24372.97448897948</v>
+        <v>3.552787878787879</v>
       </c>
       <c r="G95" t="n">
-        <v>3.392621212121212</v>
+        <v>882.2971063497258</v>
       </c>
       <c r="H95" t="n">
-        <v>1267.000961311821</v>
+        <v>26.77281422638658</v>
       </c>
       <c r="I95" t="n">
-        <v>64.26101481127037</v>
+        <v>54.51321184755107</v>
       </c>
       <c r="J95" t="n">
-        <v>141.8531100601373</v>
-      </c>
-      <c r="K95" t="n">
-        <v>98.20079965692129</v>
-      </c>
-      <c r="L95" t="n">
-        <v>396.0852533059281</v>
+        <v>43.00510067370772</v>
       </c>
     </row>
     <row r="96">
       <c r="A96" t="n">
-        <v>0.3826464646464647</v>
+        <v>0.9418989898989898</v>
       </c>
       <c r="B96" t="n">
-        <v>16711.03053627694</v>
+        <v>13091.7745998002</v>
       </c>
       <c r="C96" t="n">
-        <v>4826.351490022624</v>
+        <v>3478.215236838442</v>
       </c>
       <c r="D96" t="n">
-        <v>8246.878310697795</v>
+        <v>5636.999116186753</v>
       </c>
       <c r="E96" t="n">
-        <v>1089.193875336005</v>
+        <v>2844.005110752419</v>
       </c>
       <c r="F96" t="n">
-        <v>27428.28825021609</v>
+        <v>3.590989898989899</v>
       </c>
       <c r="G96" t="n">
-        <v>3.42910101010101</v>
+        <v>827.9521227004429</v>
       </c>
       <c r="H96" t="n">
-        <v>1198.727252305396</v>
+        <v>22.2090040590087</v>
       </c>
       <c r="I96" t="n">
-        <v>58.59407599123914</v>
+        <v>45.32063920492548</v>
       </c>
       <c r="J96" t="n">
-        <v>130.5461933592519</v>
-      </c>
-      <c r="K96" t="n">
-        <v>93.96638529666423</v>
-      </c>
-      <c r="L96" t="n">
-        <v>374.9908927613787</v>
+        <v>34.34487469578479</v>
       </c>
     </row>
     <row r="97">
       <c r="A97" t="n">
-        <v>0.3867171717171717</v>
+        <v>0.9519191919191918</v>
       </c>
       <c r="B97" t="n">
-        <v>16696.29661809596</v>
+        <v>13027.83747167627</v>
       </c>
       <c r="C97" t="n">
-        <v>4821.055523057738</v>
+        <v>3463.912741584796</v>
       </c>
       <c r="D97" t="n">
-        <v>8236.889958763835</v>
+        <v>5593.524822232407</v>
       </c>
       <c r="E97" t="n">
-        <v>1088.594425833605</v>
+        <v>3044.596089762154</v>
       </c>
       <c r="F97" t="n">
-        <v>31517.81291701904</v>
+        <v>3.629191919191919</v>
       </c>
       <c r="G97" t="n">
-        <v>3.465580808080808</v>
+        <v>782.0734902165938</v>
       </c>
       <c r="H97" t="n">
-        <v>1132.474873418442</v>
+        <v>17.72380418183005</v>
       </c>
       <c r="I97" t="n">
-        <v>53.63993661358558</v>
+        <v>36.53048603300108</v>
       </c>
       <c r="J97" t="n">
-        <v>119.7475357606462</v>
-      </c>
-      <c r="K97" t="n">
-        <v>90.14778366799001</v>
-      </c>
-      <c r="L97" t="n">
-        <v>354.5596933459137</v>
+        <v>28.199309030838</v>
       </c>
     </row>
     <row r="98">
       <c r="A98" t="n">
-        <v>0.3907878787878788</v>
+        <v>0.9619393939393939</v>
       </c>
       <c r="B98" t="n">
-        <v>16681.49415978115</v>
+        <v>12963.4649970583</v>
       </c>
       <c r="C98" t="n">
-        <v>4815.698808231651</v>
+        <v>3449.971226691129</v>
       </c>
       <c r="D98" t="n">
-        <v>8226.786244697971</v>
+        <v>5551.108581649546</v>
       </c>
       <c r="E98" t="n">
-        <v>1087.988237365733</v>
+        <v>3044.56067149859</v>
       </c>
       <c r="F98" t="n">
-        <v>36440.7358086482</v>
+        <v>3.667393939393939</v>
       </c>
       <c r="G98" t="n">
-        <v>3.502060606060606</v>
+        <v>740.7882946018279</v>
       </c>
       <c r="H98" t="n">
-        <v>1068.402315683449</v>
+        <v>13.5219160001909</v>
       </c>
       <c r="I98" t="n">
-        <v>49.45370795368569</v>
+        <v>27.6287930548419</v>
       </c>
       <c r="J98" t="n">
-        <v>109.5277483888308</v>
-      </c>
-      <c r="K98" t="n">
-        <v>86.73128427893826</v>
-      </c>
-      <c r="L98" t="n">
-        <v>334.8292758620557</v>
+        <v>21.87231537453926</v>
       </c>
     </row>
     <row r="99">
       <c r="A99" t="n">
-        <v>0.3948585858585859</v>
+        <v>0.9719595959595959</v>
       </c>
       <c r="B99" t="n">
-        <v>16666.62294743368</v>
+        <v>12898.63458043762</v>
       </c>
       <c r="C99" t="n">
-        <v>4810.280947814347</v>
+        <v>3436.117916209505</v>
       </c>
       <c r="D99" t="n">
-        <v>8216.566428759297</v>
+        <v>5509.978805759109</v>
       </c>
       <c r="E99" t="n">
-        <v>1087.375275175959</v>
+        <v>3066.351515704926</v>
       </c>
       <c r="F99" t="n">
-        <v>41996.24424436356</v>
+        <v>3.70559595959596</v>
       </c>
       <c r="G99" t="n">
-        <v>3.538540404040404</v>
+        <v>700.2355927539354</v>
       </c>
       <c r="H99" t="n">
-        <v>1006.668070132911</v>
+        <v>10.07377628983441</v>
       </c>
       <c r="I99" t="n">
-        <v>46.0905012869155</v>
+        <v>18.75684816956177</v>
       </c>
       <c r="J99" t="n">
-        <v>99.95907822067313</v>
-      </c>
-      <c r="K99" t="n">
-        <v>83.70317663754854</v>
-      </c>
-      <c r="L99" t="n">
-        <v>315.8372611123275</v>
+        <v>6.875842255374787</v>
       </c>
     </row>
     <row r="100">
       <c r="A100" t="n">
-        <v>0.398929292929293</v>
+        <v>0.981979797979798</v>
       </c>
       <c r="B100" t="n">
-        <v>16651.68276715475</v>
+        <v>12833.32362630558</v>
       </c>
       <c r="C100" t="n">
-        <v>4804.801544075813</v>
+        <v>3422.080034191988</v>
       </c>
       <c r="D100" t="n">
-        <v>8206.229771206923</v>
+        <v>5470.122820306096</v>
       </c>
       <c r="E100" t="n">
-        <v>1086.75550450785</v>
+        <v>3957.864149776401</v>
       </c>
       <c r="F100" t="n">
-        <v>47983.52554342484</v>
+        <v>3.74379797979798</v>
       </c>
       <c r="G100" t="n">
-        <v>3.575020202020202</v>
+        <v>659.5773836503071</v>
       </c>
       <c r="H100" t="n">
-        <v>947.4306277993192</v>
+        <v>7.292464675870475</v>
       </c>
       <c r="I100" t="n">
-        <v>43.60542788865089</v>
+        <v>10.85950542994118</v>
       </c>
       <c r="J100" t="n">
-        <v>91.11377223303994</v>
-      </c>
-      <c r="K100" t="n">
-        <v>81.04975025186029</v>
-      </c>
-      <c r="L100" t="n">
-        <v>297.6212698992508</v>
+        <v>-22.55063289170807</v>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="n">
-        <v>0.403</v>
+        <v>0.992</v>
       </c>
       <c r="B101" t="n">
-        <v>16636.67340504555</v>
+        <v>12767.50953915353</v>
       </c>
       <c r="C101" t="n">
-        <v>4799.260199286032</v>
+        <v>3407.584804690644</v>
       </c>
       <c r="D101" t="n">
-        <v>8195.775532299951</v>
+        <v>5430.479699122773</v>
       </c>
       <c r="E101" t="n">
-        <v>1086.128890604976</v>
+        <v>7681.257290622397</v>
       </c>
       <c r="F101" t="n">
-        <v>54201.767025092</v>
+        <v>3.782</v>
       </c>
       <c r="G101" t="n">
-        <v>3.6115</v>
+        <v>618.0189254781798</v>
       </c>
       <c r="H101" t="n">
-        <v>890.8484797151659</v>
+        <v>4.910216162991642</v>
       </c>
       <c r="I101" t="n">
-        <v>42.0535990342679</v>
+        <v>4.36385352615025</v>
       </c>
       <c r="J101" t="n">
-        <v>83.06407740279859</v>
-      </c>
-      <c r="K101" t="n">
-        <v>78.75729462991312</v>
-      </c>
-      <c r="L101" t="n">
-        <v>280.2189230253486</v>
+        <v>-60.00219998107053</v>
       </c>
     </row>
   </sheetData>

</xml_diff>